<commit_message>
Harden workbook saves and add record deletion
- Probe the file for a real write lock instead of relying on Excel's
  ~$ marker: saves are refused while Excel truly holds the workbook,
  and stale lock files after a crash no longer stall automatic lookup.
- Re-add the Selections dropdowns Excel drops when it re-saves, and
  backfill the Projects count formulas for rows added outside the app.
- Route find_urls.py through WorkbookStore so batch lookups get a
  validated, backed-up, revision-checked save; add a --limit quota guard.
- Keep at most 30 backups and append each save to backups/history.jsonl.
- Quarantine unreadable lookup_state files instead of failing startup.
- Support deleting selections, empty projects, and manufacturers from
  the editor dialog.
- Accept SERPAPI_API_KEY as an alias for SERPAPI_KEY.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -2557,22 +2557,78 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="1" t="n"/>
-      <c r="D9" s="1" t="n"/>
-      <c r="E9" s="1" t="n"/>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
-      <c r="O9" s="1" t="n"/>
-      <c r="P9" s="1" t="n"/>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>UH-103</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Windows &amp; Doors</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Living Room</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Test 1</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Dfw company</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>xyz</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Main Door</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="n"/>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>Search error</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>Automatic lookup is waiting for SERPAPI_KEY in the local .env file. Restart the app after configuring it.</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>

</xml_diff>

<commit_message>
Track the client-approval lifecycle separately from link verification
- Client Status column (Proposed/Presented/Approved/Rejected/Changed)
  records the client decision per selection; identity edits move
  Presented/Approved rows back to Changed and Rejected rows to Proposed.
- Every presentation export is logged in history.jsonl and numbered
  R{n} per project in the filename and document metadata; non-draft
  exports mark included Proposed rows Presented.
- Verified links older than 180 days surface as Re-check flags in the
  tracker, review view, and export summary.
- The project page warns when the presentation date is near and rows
  still need review.
- Add from link prefills a new selection from a pasted product URL.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$P$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$Q$501</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2068,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P501"/>
+  <dimension ref="A1:Q501"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2084,6 +2084,7 @@
     <col width="30" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
     <col width="13.453125" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2165,6 +2166,11 @@
       <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Include in Lookbook</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>Client Status</t>
         </is>
       </c>
     </row>
@@ -2221,6 +2227,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -2277,6 +2288,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2333,6 +2349,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2387,6 +2408,11 @@
       <c r="P5" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Proposed</t>
         </is>
       </c>
     </row>
@@ -2443,6 +2469,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2499,6 +2530,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2555,6 +2591,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2611,7 +2652,7 @@
       </c>
       <c r="M9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr">
@@ -2627,6 +2668,11 @@
       <c r="P9" s="7" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Proposed</t>
         </is>
       </c>
     </row>
@@ -11487,8 +11533,8 @@
       <c r="P501" s="1" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P501"/>
-  <dataValidations count="4">
+  <autoFilter ref="A1:Q501"/>
+  <dataValidations count="5">
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list (edit the Lists sheet to add options)." type="list">
       <formula1>Lists!$A$2:$A$31</formula1>
     </dataValidation>
@@ -11500,6 +11546,9 @@
     </dataValidation>
     <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list (edit the Lists sheet to add options)." type="list">
       <formula1>Projects!$A$2:$A$51</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Proposed,Presented,Approved,Rejected,Changed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Make the workbook complete for direct data entry in Excel
The Lookup Status dropdown was missing 'Search error' and Client Status
had no Lists column, so values the app writes could not be chosen by
hand. The app now owns those list columns and rewrites them on save.

- ensure_list_values keeps Lists complete for Lookup Status, Yes/No and
  Client Status; the section order column stays the user's.
- ensure_validations replaces the dropdowns on managed columns instead
  of appending, so older workbooks cannot keep two lists on one column.
- migrate_workbook.py refreshes an existing workbook: dropdowns, filters
  across every column, header-only freeze, readable widths, and an
  Instructions sheet covering the web app, each column, and the rules.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -13,7 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$L$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$Q$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Manufacturers'!$A$1:$C$101</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -58,6 +60,20 @@
       <name val="Arial"/>
       <family val="2"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -113,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -156,6 +172,21 @@
     </xf>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,131 +487,242 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="120" customWidth="1" style="4" min="1" max="1"/>
+    <col width="118" customWidth="1" style="4" min="1" max="1"/>
     <col width="8.6328125" customWidth="1" style="4" min="2" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>UH Homes - Selections Tracker</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="n"/>
+      <c r="A2" s="16" t="n"/>
     </row>
     <row r="3" ht="15.5" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>How this workbook works</t>
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>This workbook is the source of truth. You can type directly into it, or use the web app (python app.py, then open the address it prints). Both read and write these same sheets.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>1. Add each project once on the Projects sheet (one row per project, unique Project ID).</t>
-        </is>
-      </c>
+      <c r="A4" s="16" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>2. Add every selection on the Selections sheet. Yellow columns are yours to fill; grey columns are filled by find_urls.py.</t>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>How the workflow runs</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>3. Run:  python find_urls.py   - fills Product URL, Product Name, Image URL, Lookup Status, Checked On, Lookup Notes.</t>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>1. Projects sheet - one row per project, with a unique Project ID such as UH-101.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>4. Review every row. When a link is confirmed correct, set Lookup Status to 'Verified'. Verified rows are never overwritten.</t>
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>2. Selections sheet - one row per product. Fill the entry columns listed below.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>5. Run:  python build_lookbook.py --project UH-101   (or --all) - creates the client PDF lookbook in /output.</t>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>3. Product links - the web app finds them automatically while it is running, or run python find_urls.py (add --project UH-101 for one project, --dry-run to preview).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>4. Review each link against the real product page, then set Lookup Status to Verified. Verified rows are never overwritten automatically.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Legend</t>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>5. Client Status records the client's decision: Proposed, Presented, Approved, Rejected, Changed.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Yellow cell = input you type</t>
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>6. Export the finish schedule from the web app, or run python build_lookbook.py --project UH-101 (PDF) or build_powerpoint.py (editable deck).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Grey cell = filled by the scripts (you may edit by hand; set status to Verified to lock it)</t>
-        </is>
-      </c>
+      <c r="A12" s="19" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Columns you fill in (Selections)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15.5" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Rules</t>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Project ID       Must match a Project ID on the Projects sheet. Dropdown.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>- Section values come from the Lists sheet; lookbook sections appear in the order listed there.</t>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Section          Category and print order; values come from the Lists sheet. Dropdown.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>- Add each brand's official website on the Manufacturers sheet - the lookup searches that site first.</t>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Room / Area      Optional location, for example Primary Bath.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>- Image URL may be a web link or a local file path (e.g. images/front-door.jpg) to override the found image.</t>
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Item             What the client sees, for example Kitchen Faucet. Required.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>- Include in Lookbook = No hides a row from the client PDF without deleting it.</t>
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Manufacturer     Brand name. Add its official domain on the Manufacturers sheet.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>- The rows on Projects/Selections are EXAMPLES - replace them with real data.</t>
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Model #          Manufacturer model or SKU. Needed for automatic product lookup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Finish / Color   For example Matte Black or SW 7010.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Qty              Leave blank or 1 to hide the quantity from the client schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Client Notes     Short note printed with the item on the client schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Include in Lookbook   No hides the row from client exports without deleting it. Dropdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Client Status    Proposed / Presented / Approved / Rejected / Changed. Dropdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Columns filled in for you</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Product URL, Product Name, Image URL, Lookup Status, Checked On, Lookup Notes are written by the product lookup. You may correct any of them by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>On the Projects sheet, Total Items, Links Found, Verified and Needs Review are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Rules worth knowing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>- Changing Item, Product Name, Manufacturer, Model # or Finish clears the old link and verification, because they no longer describe the same product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>- A Verified link older than six months is flagged for re-checking in the web app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>- Close this workbook in Excel before saving from the web app; the app will not write to a file Excel has open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>- Every save keeps a timestamped copy in the backups folder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>- Product URLs and images are internal review aids and never appear on client documents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>- Section order on the Lists sheet controls the order of categories in the client schedule.</t>
         </is>
       </c>
     </row>
@@ -604,7 +746,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -2056,6 +2198,7 @@
       <c r="L51" s="7" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -2079,11 +2222,12 @@
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="11"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="13.453125" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
@@ -11535,20 +11679,20 @@
   </sheetData>
   <autoFilter ref="A1:Q501"/>
   <dataValidations count="5">
-    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list (edit the Lists sheet to add options)." type="list">
+    <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Projects!$A$2:$A$51</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Lists!$A$2:$A$31</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list (edit the Lists sheet to add options)." type="list">
-      <formula1>Lists!$B$2:$B$7</formula1>
+    <dataValidation sqref="L2:L501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Lists!$B$2:$B$8</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list (edit the Lists sheet to add options)." type="list">
+    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Lists!$C$2:$C$3</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list (edit the Lists sheet to add options)." type="list">
-      <formula1>Projects!$A$2:$A$51</formula1>
-    </dataValidation>
     <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Proposed,Presented,Approved,Rejected,Changed"</formula1>
+      <formula1>Lists!$D$2:$D$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12253,6 +12397,7 @@
       <c r="C101" s="1" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -12264,13 +12409,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="26" customWidth="1" style="4" min="1" max="1"/>
     <col width="20" customWidth="1" style="4" min="2" max="2"/>
     <col width="10" customWidth="1" style="4" min="3" max="3"/>
-    <col width="8.6328125" customWidth="1" style="4" min="4" max="16384"/>
+    <col width="20" customWidth="1" style="4" min="4" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -12289,6 +12434,11 @@
           <t>Yes / No</t>
         </is>
       </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Client Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -12306,6 +12456,11 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -12323,6 +12478,11 @@
           <t>No</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Presented</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -12336,6 +12496,11 @@
         </is>
       </c>
       <c r="C4" s="6" t="n"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -12349,6 +12514,11 @@
         </is>
       </c>
       <c r="C5" s="6" t="n"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -12362,6 +12532,11 @@
         </is>
       </c>
       <c r="C6" s="6" t="n"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -12371,7 +12546,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Search error</t>
         </is>
       </c>
       <c r="C7" s="6" t="n"/>
@@ -12382,7 +12557,11 @@
           <t>Flooring</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
       <c r="C8" s="6" t="n"/>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Add a priced Price Schedule sheet grouped by project and category
- New optional Unit Price column on Selections, editable in Excel and
  in the web app. Qty and Unit Price are written as real numbers so
  Excel's SUM and ISNUMBER work on them.
- price_schedule.rebuild regenerates a Price Schedule sheet on every
  save: S.No, Code, Description, Qty, Unit Price and Price per line,
  grouped under each project and category, with category subtotals, a
  project total and a grand total. Qty, Unit Price and the line total
  are formulas against Selections, so typed prices flow straight through.
- The sheet is a view and says so; prices stay internal and are kept
  out of the client PDF and PowerPoint, which a test now enforces.
- description() grows an include_quantity flag so the priced table can
  drop the quantity it already shows in its own column.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -11,10 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selections" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturers" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Schedule" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$L$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$Q$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$R$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Manufacturers'!$A$1:$C$101</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -75,8 +76,43 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF2F3337"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF7A7E82"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF2F3337"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF2F3337"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF2F3337"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -101,8 +137,23 @@
         <bgColor rgb="FF333300"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F3337"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9A24A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -125,11 +176,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FFE3E3E1"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF2F3337"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -187,6 +248,51 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="13" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -487,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="118" customWidth="1" style="4" min="1" max="1"/>
@@ -632,95 +738,133 @@
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>Client Notes     Short note printed with the item on the client schedule.</t>
+          <t>Unit Price       Cost per unit. The Price Schedule sheet multiplies it by Qty and totals it.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Include in Lookbook   No hides the row from client exports without deleting it. Dropdown.</t>
+          <t>Client Notes     Short note printed with the item on the client schedule.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
+          <t>Include in Lookbook   No hides the row from client exports without deleting it. Dropdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
           <t>Client Status    Proposed / Presented / Approved / Rejected / Changed. Dropdown.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="16" t="n"/>
-    </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>Columns filled in for you</t>
-        </is>
-      </c>
+      <c r="A26" s="16" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>Product URL, Product Name, Image URL, Lookup Status, Checked On, Lookup Notes are written by the product lookup. You may correct any of them by hand.</t>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Price Schedule sheet</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>On the Projects sheet, Total Items, Links Found, Verified and Needs Review are formulas.</t>
+          <t>Every selection grouped by project and category with S.No, Code, Description, Qty, Unit Price and Price, plus a subtotal per category, a total per project and a grand total.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="n"/>
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>It is rebuilt automatically each time the workbook is saved, so do not type into it. Enter costs in the Unit Price column on Selections and they flow through.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>Rules worth knowing</t>
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Prices stay internal: they never appear on the client PDF or PowerPoint.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>- Changing Item, Product Name, Manufacturer, Model # or Finish clears the old link and verification, because they no longer describe the same product.</t>
-        </is>
-      </c>
+      <c r="A31" s="16" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>- A Verified link older than six months is flagged for re-checking in the web app.</t>
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Columns filled in for you</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>- Close this workbook in Excel before saving from the web app; the app will not write to a file Excel has open.</t>
+          <t>Product URL, Product Name, Image URL, Lookup Status, Checked On, Lookup Notes are written by the product lookup. You may correct any of them by hand.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
         <is>
+          <t>On the Projects sheet, Total Items, Links Found, Verified and Needs Review are formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Rules worth knowing</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>- Changing Item, Product Name, Manufacturer, Model # or Finish clears the old link and verification, because they no longer describe the same product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>- A Verified link older than six months is flagged for re-checking in the web app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>- Close this workbook in Excel before saving from the web app; the app will not write to a file Excel has open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
           <t>- Every save keeps a timestamped copy in the backups folder.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>- Product URLs and images are internal review aids and never appear on client documents.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>- Section order on the Lists sheet controls the order of categories in the client schedule.</t>
         </is>
@@ -2211,7 +2355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q501"/>
+  <dimension ref="A1:R501"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2229,6 +2373,7 @@
     <col width="28" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2315,6 +2460,11 @@
       <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Client Status</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
         </is>
       </c>
     </row>
@@ -2376,6 +2526,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R2" s="20" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -2437,6 +2588,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R3" s="20" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2498,6 +2650,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R4" s="20" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2559,6 +2712,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R5" s="20" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2618,6 +2772,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R6" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2679,6 +2834,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R7" s="20" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2740,6 +2896,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R8" s="20" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2819,6 +2976,7 @@
           <t>Proposed</t>
         </is>
       </c>
+      <c r="R9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
@@ -2837,6 +2995,7 @@
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="n"/>
+      <c r="R10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n"/>
@@ -2855,6 +3014,7 @@
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="n"/>
+      <c r="R11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
@@ -2873,6 +3033,7 @@
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="n"/>
+      <c r="R12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
@@ -2891,6 +3052,7 @@
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="n"/>
+      <c r="R13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n"/>
@@ -2909,6 +3071,7 @@
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="n"/>
+      <c r="R14" s="20" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
@@ -2927,6 +3090,7 @@
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="n"/>
+      <c r="R15" s="20" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n"/>
@@ -2945,6 +3109,7 @@
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="n"/>
+      <c r="R16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -2963,6 +3128,7 @@
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="n"/>
+      <c r="R17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -2981,6 +3147,7 @@
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="1" t="n"/>
       <c r="P18" s="1" t="n"/>
+      <c r="R18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -2999,6 +3166,7 @@
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="n"/>
+      <c r="R19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -3017,6 +3185,7 @@
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="n"/>
+      <c r="R20" s="20" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
@@ -3035,6 +3204,7 @@
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="1" t="n"/>
       <c r="P21" s="1" t="n"/>
+      <c r="R21" s="20" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
@@ -3053,6 +3223,7 @@
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="n"/>
+      <c r="R22" s="20" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
@@ -3071,6 +3242,7 @@
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="n"/>
+      <c r="R23" s="20" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
@@ -3089,6 +3261,7 @@
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="1" t="n"/>
       <c r="P24" s="1" t="n"/>
+      <c r="R24" s="20" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
@@ -3107,6 +3280,7 @@
       <c r="N25" s="2" t="n"/>
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="n"/>
+      <c r="R25" s="20" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
@@ -3125,6 +3299,7 @@
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="n"/>
+      <c r="R26" s="20" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
@@ -3143,6 +3318,7 @@
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="n"/>
+      <c r="R27" s="20" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n"/>
@@ -3161,6 +3337,7 @@
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="n"/>
+      <c r="R28" s="20" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n"/>
@@ -3179,6 +3356,7 @@
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="1" t="n"/>
       <c r="P29" s="1" t="n"/>
+      <c r="R29" s="20" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
@@ -3197,6 +3375,7 @@
       <c r="N30" s="2" t="n"/>
       <c r="O30" s="1" t="n"/>
       <c r="P30" s="1" t="n"/>
+      <c r="R30" s="20" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
@@ -3215,6 +3394,7 @@
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="n"/>
+      <c r="R31" s="20" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n"/>
@@ -3233,6 +3413,7 @@
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="n"/>
+      <c r="R32" s="20" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n"/>
@@ -3251,6 +3432,7 @@
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="n"/>
+      <c r="R33" s="20" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n"/>
@@ -3269,6 +3451,7 @@
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="n"/>
+      <c r="R34" s="20" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n"/>
@@ -3287,6 +3470,7 @@
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="n"/>
+      <c r="R35" s="20" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n"/>
@@ -3305,6 +3489,7 @@
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="n"/>
+      <c r="R36" s="20" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n"/>
@@ -3323,6 +3508,7 @@
       <c r="N37" s="2" t="n"/>
       <c r="O37" s="1" t="n"/>
       <c r="P37" s="1" t="n"/>
+      <c r="R37" s="20" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n"/>
@@ -3341,6 +3527,7 @@
       <c r="N38" s="2" t="n"/>
       <c r="O38" s="1" t="n"/>
       <c r="P38" s="1" t="n"/>
+      <c r="R38" s="20" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n"/>
@@ -3359,6 +3546,7 @@
       <c r="N39" s="2" t="n"/>
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="n"/>
+      <c r="R39" s="20" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n"/>
@@ -3377,6 +3565,7 @@
       <c r="N40" s="2" t="n"/>
       <c r="O40" s="1" t="n"/>
       <c r="P40" s="1" t="n"/>
+      <c r="R40" s="20" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n"/>
@@ -3395,6 +3584,7 @@
       <c r="N41" s="2" t="n"/>
       <c r="O41" s="1" t="n"/>
       <c r="P41" s="1" t="n"/>
+      <c r="R41" s="20" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n"/>
@@ -3413,6 +3603,7 @@
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="1" t="n"/>
       <c r="P42" s="1" t="n"/>
+      <c r="R42" s="20" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n"/>
@@ -3431,6 +3622,7 @@
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="1" t="n"/>
       <c r="P43" s="1" t="n"/>
+      <c r="R43" s="20" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n"/>
@@ -3449,6 +3641,7 @@
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="1" t="n"/>
       <c r="P44" s="1" t="n"/>
+      <c r="R44" s="20" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n"/>
@@ -3467,6 +3660,7 @@
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="n"/>
+      <c r="R45" s="20" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n"/>
@@ -3485,6 +3679,7 @@
       <c r="N46" s="2" t="n"/>
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="n"/>
+      <c r="R46" s="20" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n"/>
@@ -3503,6 +3698,7 @@
       <c r="N47" s="2" t="n"/>
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="n"/>
+      <c r="R47" s="20" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n"/>
@@ -3521,6 +3717,7 @@
       <c r="N48" s="2" t="n"/>
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="n"/>
+      <c r="R48" s="20" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n"/>
@@ -3539,6 +3736,7 @@
       <c r="N49" s="2" t="n"/>
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="n"/>
+      <c r="R49" s="20" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n"/>
@@ -3557,6 +3755,7 @@
       <c r="N50" s="2" t="n"/>
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="n"/>
+      <c r="R50" s="20" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n"/>
@@ -3575,6 +3774,7 @@
       <c r="N51" s="2" t="n"/>
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="n"/>
+      <c r="R51" s="20" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n"/>
@@ -3593,6 +3793,7 @@
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="n"/>
+      <c r="R52" s="20" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n"/>
@@ -3611,6 +3812,7 @@
       <c r="N53" s="2" t="n"/>
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="n"/>
+      <c r="R53" s="20" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n"/>
@@ -3629,6 +3831,7 @@
       <c r="N54" s="2" t="n"/>
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="n"/>
+      <c r="R54" s="20" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n"/>
@@ -3647,6 +3850,7 @@
       <c r="N55" s="2" t="n"/>
       <c r="O55" s="1" t="n"/>
       <c r="P55" s="1" t="n"/>
+      <c r="R55" s="20" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n"/>
@@ -3665,6 +3869,7 @@
       <c r="N56" s="2" t="n"/>
       <c r="O56" s="1" t="n"/>
       <c r="P56" s="1" t="n"/>
+      <c r="R56" s="20" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n"/>
@@ -3683,6 +3888,7 @@
       <c r="N57" s="2" t="n"/>
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="n"/>
+      <c r="R57" s="20" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n"/>
@@ -3701,6 +3907,7 @@
       <c r="N58" s="2" t="n"/>
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="n"/>
+      <c r="R58" s="20" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n"/>
@@ -3719,6 +3926,7 @@
       <c r="N59" s="2" t="n"/>
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="n"/>
+      <c r="R59" s="20" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n"/>
@@ -3737,6 +3945,7 @@
       <c r="N60" s="2" t="n"/>
       <c r="O60" s="1" t="n"/>
       <c r="P60" s="1" t="n"/>
+      <c r="R60" s="20" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n"/>
@@ -3755,6 +3964,7 @@
       <c r="N61" s="2" t="n"/>
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="n"/>
+      <c r="R61" s="20" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n"/>
@@ -3773,6 +3983,7 @@
       <c r="N62" s="2" t="n"/>
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="n"/>
+      <c r="R62" s="20" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n"/>
@@ -3791,6 +4002,7 @@
       <c r="N63" s="2" t="n"/>
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="n"/>
+      <c r="R63" s="20" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n"/>
@@ -3809,6 +4021,7 @@
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="n"/>
+      <c r="R64" s="20" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n"/>
@@ -3827,6 +4040,7 @@
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="n"/>
+      <c r="R65" s="20" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n"/>
@@ -3845,6 +4059,7 @@
       <c r="N66" s="2" t="n"/>
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="n"/>
+      <c r="R66" s="20" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n"/>
@@ -3863,6 +4078,7 @@
       <c r="N67" s="2" t="n"/>
       <c r="O67" s="1" t="n"/>
       <c r="P67" s="1" t="n"/>
+      <c r="R67" s="20" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n"/>
@@ -3881,6 +4097,7 @@
       <c r="N68" s="2" t="n"/>
       <c r="O68" s="1" t="n"/>
       <c r="P68" s="1" t="n"/>
+      <c r="R68" s="20" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n"/>
@@ -3899,6 +4116,7 @@
       <c r="N69" s="2" t="n"/>
       <c r="O69" s="1" t="n"/>
       <c r="P69" s="1" t="n"/>
+      <c r="R69" s="20" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n"/>
@@ -3917,6 +4135,7 @@
       <c r="N70" s="2" t="n"/>
       <c r="O70" s="1" t="n"/>
       <c r="P70" s="1" t="n"/>
+      <c r="R70" s="20" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n"/>
@@ -3935,6 +4154,7 @@
       <c r="N71" s="2" t="n"/>
       <c r="O71" s="1" t="n"/>
       <c r="P71" s="1" t="n"/>
+      <c r="R71" s="20" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n"/>
@@ -3953,6 +4173,7 @@
       <c r="N72" s="2" t="n"/>
       <c r="O72" s="1" t="n"/>
       <c r="P72" s="1" t="n"/>
+      <c r="R72" s="20" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n"/>
@@ -3971,6 +4192,7 @@
       <c r="N73" s="2" t="n"/>
       <c r="O73" s="1" t="n"/>
       <c r="P73" s="1" t="n"/>
+      <c r="R73" s="20" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n"/>
@@ -3989,6 +4211,7 @@
       <c r="N74" s="2" t="n"/>
       <c r="O74" s="1" t="n"/>
       <c r="P74" s="1" t="n"/>
+      <c r="R74" s="20" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n"/>
@@ -4007,6 +4230,7 @@
       <c r="N75" s="2" t="n"/>
       <c r="O75" s="1" t="n"/>
       <c r="P75" s="1" t="n"/>
+      <c r="R75" s="20" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n"/>
@@ -4025,6 +4249,7 @@
       <c r="N76" s="2" t="n"/>
       <c r="O76" s="1" t="n"/>
       <c r="P76" s="1" t="n"/>
+      <c r="R76" s="20" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n"/>
@@ -4043,6 +4268,7 @@
       <c r="N77" s="2" t="n"/>
       <c r="O77" s="1" t="n"/>
       <c r="P77" s="1" t="n"/>
+      <c r="R77" s="20" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n"/>
@@ -4061,6 +4287,7 @@
       <c r="N78" s="2" t="n"/>
       <c r="O78" s="1" t="n"/>
       <c r="P78" s="1" t="n"/>
+      <c r="R78" s="20" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n"/>
@@ -4079,6 +4306,7 @@
       <c r="N79" s="2" t="n"/>
       <c r="O79" s="1" t="n"/>
       <c r="P79" s="1" t="n"/>
+      <c r="R79" s="20" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n"/>
@@ -4097,6 +4325,7 @@
       <c r="N80" s="2" t="n"/>
       <c r="O80" s="1" t="n"/>
       <c r="P80" s="1" t="n"/>
+      <c r="R80" s="20" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n"/>
@@ -4115,6 +4344,7 @@
       <c r="N81" s="2" t="n"/>
       <c r="O81" s="1" t="n"/>
       <c r="P81" s="1" t="n"/>
+      <c r="R81" s="20" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n"/>
@@ -4133,6 +4363,7 @@
       <c r="N82" s="2" t="n"/>
       <c r="O82" s="1" t="n"/>
       <c r="P82" s="1" t="n"/>
+      <c r="R82" s="20" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n"/>
@@ -4151,6 +4382,7 @@
       <c r="N83" s="2" t="n"/>
       <c r="O83" s="1" t="n"/>
       <c r="P83" s="1" t="n"/>
+      <c r="R83" s="20" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n"/>
@@ -4169,6 +4401,7 @@
       <c r="N84" s="2" t="n"/>
       <c r="O84" s="1" t="n"/>
       <c r="P84" s="1" t="n"/>
+      <c r="R84" s="20" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n"/>
@@ -4187,6 +4420,7 @@
       <c r="N85" s="2" t="n"/>
       <c r="O85" s="1" t="n"/>
       <c r="P85" s="1" t="n"/>
+      <c r="R85" s="20" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n"/>
@@ -4205,6 +4439,7 @@
       <c r="N86" s="2" t="n"/>
       <c r="O86" s="1" t="n"/>
       <c r="P86" s="1" t="n"/>
+      <c r="R86" s="20" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n"/>
@@ -4223,6 +4458,7 @@
       <c r="N87" s="2" t="n"/>
       <c r="O87" s="1" t="n"/>
       <c r="P87" s="1" t="n"/>
+      <c r="R87" s="20" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n"/>
@@ -4241,6 +4477,7 @@
       <c r="N88" s="2" t="n"/>
       <c r="O88" s="1" t="n"/>
       <c r="P88" s="1" t="n"/>
+      <c r="R88" s="20" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n"/>
@@ -4259,6 +4496,7 @@
       <c r="N89" s="2" t="n"/>
       <c r="O89" s="1" t="n"/>
       <c r="P89" s="1" t="n"/>
+      <c r="R89" s="20" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n"/>
@@ -4277,6 +4515,7 @@
       <c r="N90" s="2" t="n"/>
       <c r="O90" s="1" t="n"/>
       <c r="P90" s="1" t="n"/>
+      <c r="R90" s="20" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n"/>
@@ -4295,6 +4534,7 @@
       <c r="N91" s="2" t="n"/>
       <c r="O91" s="1" t="n"/>
       <c r="P91" s="1" t="n"/>
+      <c r="R91" s="20" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n"/>
@@ -4313,6 +4553,7 @@
       <c r="N92" s="2" t="n"/>
       <c r="O92" s="1" t="n"/>
       <c r="P92" s="1" t="n"/>
+      <c r="R92" s="20" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n"/>
@@ -4331,6 +4572,7 @@
       <c r="N93" s="2" t="n"/>
       <c r="O93" s="1" t="n"/>
       <c r="P93" s="1" t="n"/>
+      <c r="R93" s="20" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n"/>
@@ -4349,6 +4591,7 @@
       <c r="N94" s="2" t="n"/>
       <c r="O94" s="1" t="n"/>
       <c r="P94" s="1" t="n"/>
+      <c r="R94" s="20" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n"/>
@@ -4367,6 +4610,7 @@
       <c r="N95" s="2" t="n"/>
       <c r="O95" s="1" t="n"/>
       <c r="P95" s="1" t="n"/>
+      <c r="R95" s="20" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n"/>
@@ -4385,6 +4629,7 @@
       <c r="N96" s="2" t="n"/>
       <c r="O96" s="1" t="n"/>
       <c r="P96" s="1" t="n"/>
+      <c r="R96" s="20" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n"/>
@@ -4403,6 +4648,7 @@
       <c r="N97" s="2" t="n"/>
       <c r="O97" s="1" t="n"/>
       <c r="P97" s="1" t="n"/>
+      <c r="R97" s="20" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n"/>
@@ -4421,6 +4667,7 @@
       <c r="N98" s="2" t="n"/>
       <c r="O98" s="1" t="n"/>
       <c r="P98" s="1" t="n"/>
+      <c r="R98" s="20" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n"/>
@@ -4439,6 +4686,7 @@
       <c r="N99" s="2" t="n"/>
       <c r="O99" s="1" t="n"/>
       <c r="P99" s="1" t="n"/>
+      <c r="R99" s="20" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n"/>
@@ -4457,6 +4705,7 @@
       <c r="N100" s="2" t="n"/>
       <c r="O100" s="1" t="n"/>
       <c r="P100" s="1" t="n"/>
+      <c r="R100" s="20" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n"/>
@@ -4475,6 +4724,7 @@
       <c r="N101" s="2" t="n"/>
       <c r="O101" s="1" t="n"/>
       <c r="P101" s="1" t="n"/>
+      <c r="R101" s="20" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n"/>
@@ -4493,6 +4743,7 @@
       <c r="N102" s="2" t="n"/>
       <c r="O102" s="1" t="n"/>
       <c r="P102" s="1" t="n"/>
+      <c r="R102" s="20" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n"/>
@@ -4511,6 +4762,7 @@
       <c r="N103" s="2" t="n"/>
       <c r="O103" s="1" t="n"/>
       <c r="P103" s="1" t="n"/>
+      <c r="R103" s="20" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n"/>
@@ -4529,6 +4781,7 @@
       <c r="N104" s="2" t="n"/>
       <c r="O104" s="1" t="n"/>
       <c r="P104" s="1" t="n"/>
+      <c r="R104" s="20" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n"/>
@@ -4547,6 +4800,7 @@
       <c r="N105" s="2" t="n"/>
       <c r="O105" s="1" t="n"/>
       <c r="P105" s="1" t="n"/>
+      <c r="R105" s="20" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n"/>
@@ -4565,6 +4819,7 @@
       <c r="N106" s="2" t="n"/>
       <c r="O106" s="1" t="n"/>
       <c r="P106" s="1" t="n"/>
+      <c r="R106" s="20" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n"/>
@@ -4583,6 +4838,7 @@
       <c r="N107" s="2" t="n"/>
       <c r="O107" s="1" t="n"/>
       <c r="P107" s="1" t="n"/>
+      <c r="R107" s="20" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n"/>
@@ -4601,6 +4857,7 @@
       <c r="N108" s="2" t="n"/>
       <c r="O108" s="1" t="n"/>
       <c r="P108" s="1" t="n"/>
+      <c r="R108" s="20" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n"/>
@@ -4619,6 +4876,7 @@
       <c r="N109" s="2" t="n"/>
       <c r="O109" s="1" t="n"/>
       <c r="P109" s="1" t="n"/>
+      <c r="R109" s="20" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n"/>
@@ -4637,6 +4895,7 @@
       <c r="N110" s="2" t="n"/>
       <c r="O110" s="1" t="n"/>
       <c r="P110" s="1" t="n"/>
+      <c r="R110" s="20" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n"/>
@@ -4655,6 +4914,7 @@
       <c r="N111" s="2" t="n"/>
       <c r="O111" s="1" t="n"/>
       <c r="P111" s="1" t="n"/>
+      <c r="R111" s="20" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n"/>
@@ -4673,6 +4933,7 @@
       <c r="N112" s="2" t="n"/>
       <c r="O112" s="1" t="n"/>
       <c r="P112" s="1" t="n"/>
+      <c r="R112" s="20" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n"/>
@@ -4691,6 +4952,7 @@
       <c r="N113" s="2" t="n"/>
       <c r="O113" s="1" t="n"/>
       <c r="P113" s="1" t="n"/>
+      <c r="R113" s="20" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n"/>
@@ -4709,6 +4971,7 @@
       <c r="N114" s="2" t="n"/>
       <c r="O114" s="1" t="n"/>
       <c r="P114" s="1" t="n"/>
+      <c r="R114" s="20" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n"/>
@@ -4727,6 +4990,7 @@
       <c r="N115" s="2" t="n"/>
       <c r="O115" s="1" t="n"/>
       <c r="P115" s="1" t="n"/>
+      <c r="R115" s="20" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n"/>
@@ -4745,6 +5009,7 @@
       <c r="N116" s="2" t="n"/>
       <c r="O116" s="1" t="n"/>
       <c r="P116" s="1" t="n"/>
+      <c r="R116" s="20" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n"/>
@@ -4763,6 +5028,7 @@
       <c r="N117" s="2" t="n"/>
       <c r="O117" s="1" t="n"/>
       <c r="P117" s="1" t="n"/>
+      <c r="R117" s="20" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n"/>
@@ -4781,6 +5047,7 @@
       <c r="N118" s="2" t="n"/>
       <c r="O118" s="1" t="n"/>
       <c r="P118" s="1" t="n"/>
+      <c r="R118" s="20" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n"/>
@@ -4799,6 +5066,7 @@
       <c r="N119" s="2" t="n"/>
       <c r="O119" s="1" t="n"/>
       <c r="P119" s="1" t="n"/>
+      <c r="R119" s="20" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n"/>
@@ -4817,6 +5085,7 @@
       <c r="N120" s="2" t="n"/>
       <c r="O120" s="1" t="n"/>
       <c r="P120" s="1" t="n"/>
+      <c r="R120" s="20" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n"/>
@@ -4835,6 +5104,7 @@
       <c r="N121" s="2" t="n"/>
       <c r="O121" s="1" t="n"/>
       <c r="P121" s="1" t="n"/>
+      <c r="R121" s="20" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n"/>
@@ -4853,6 +5123,7 @@
       <c r="N122" s="2" t="n"/>
       <c r="O122" s="1" t="n"/>
       <c r="P122" s="1" t="n"/>
+      <c r="R122" s="20" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n"/>
@@ -4871,6 +5142,7 @@
       <c r="N123" s="2" t="n"/>
       <c r="O123" s="1" t="n"/>
       <c r="P123" s="1" t="n"/>
+      <c r="R123" s="20" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n"/>
@@ -4889,6 +5161,7 @@
       <c r="N124" s="2" t="n"/>
       <c r="O124" s="1" t="n"/>
       <c r="P124" s="1" t="n"/>
+      <c r="R124" s="20" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n"/>
@@ -4907,6 +5180,7 @@
       <c r="N125" s="2" t="n"/>
       <c r="O125" s="1" t="n"/>
       <c r="P125" s="1" t="n"/>
+      <c r="R125" s="20" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n"/>
@@ -4925,6 +5199,7 @@
       <c r="N126" s="2" t="n"/>
       <c r="O126" s="1" t="n"/>
       <c r="P126" s="1" t="n"/>
+      <c r="R126" s="20" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n"/>
@@ -4943,6 +5218,7 @@
       <c r="N127" s="2" t="n"/>
       <c r="O127" s="1" t="n"/>
       <c r="P127" s="1" t="n"/>
+      <c r="R127" s="20" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n"/>
@@ -4961,6 +5237,7 @@
       <c r="N128" s="2" t="n"/>
       <c r="O128" s="1" t="n"/>
       <c r="P128" s="1" t="n"/>
+      <c r="R128" s="20" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n"/>
@@ -4979,6 +5256,7 @@
       <c r="N129" s="2" t="n"/>
       <c r="O129" s="1" t="n"/>
       <c r="P129" s="1" t="n"/>
+      <c r="R129" s="20" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n"/>
@@ -4997,6 +5275,7 @@
       <c r="N130" s="2" t="n"/>
       <c r="O130" s="1" t="n"/>
       <c r="P130" s="1" t="n"/>
+      <c r="R130" s="20" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n"/>
@@ -5015,6 +5294,7 @@
       <c r="N131" s="2" t="n"/>
       <c r="O131" s="1" t="n"/>
       <c r="P131" s="1" t="n"/>
+      <c r="R131" s="20" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n"/>
@@ -5033,6 +5313,7 @@
       <c r="N132" s="2" t="n"/>
       <c r="O132" s="1" t="n"/>
       <c r="P132" s="1" t="n"/>
+      <c r="R132" s="20" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n"/>
@@ -5051,6 +5332,7 @@
       <c r="N133" s="2" t="n"/>
       <c r="O133" s="1" t="n"/>
       <c r="P133" s="1" t="n"/>
+      <c r="R133" s="20" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n"/>
@@ -5069,6 +5351,7 @@
       <c r="N134" s="2" t="n"/>
       <c r="O134" s="1" t="n"/>
       <c r="P134" s="1" t="n"/>
+      <c r="R134" s="20" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n"/>
@@ -5087,6 +5370,7 @@
       <c r="N135" s="2" t="n"/>
       <c r="O135" s="1" t="n"/>
       <c r="P135" s="1" t="n"/>
+      <c r="R135" s="20" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n"/>
@@ -5105,6 +5389,7 @@
       <c r="N136" s="2" t="n"/>
       <c r="O136" s="1" t="n"/>
       <c r="P136" s="1" t="n"/>
+      <c r="R136" s="20" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n"/>
@@ -5123,6 +5408,7 @@
       <c r="N137" s="2" t="n"/>
       <c r="O137" s="1" t="n"/>
       <c r="P137" s="1" t="n"/>
+      <c r="R137" s="20" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n"/>
@@ -5141,6 +5427,7 @@
       <c r="N138" s="2" t="n"/>
       <c r="O138" s="1" t="n"/>
       <c r="P138" s="1" t="n"/>
+      <c r="R138" s="20" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n"/>
@@ -5159,6 +5446,7 @@
       <c r="N139" s="2" t="n"/>
       <c r="O139" s="1" t="n"/>
       <c r="P139" s="1" t="n"/>
+      <c r="R139" s="20" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n"/>
@@ -5177,6 +5465,7 @@
       <c r="N140" s="2" t="n"/>
       <c r="O140" s="1" t="n"/>
       <c r="P140" s="1" t="n"/>
+      <c r="R140" s="20" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n"/>
@@ -5195,6 +5484,7 @@
       <c r="N141" s="2" t="n"/>
       <c r="O141" s="1" t="n"/>
       <c r="P141" s="1" t="n"/>
+      <c r="R141" s="20" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n"/>
@@ -5213,6 +5503,7 @@
       <c r="N142" s="2" t="n"/>
       <c r="O142" s="1" t="n"/>
       <c r="P142" s="1" t="n"/>
+      <c r="R142" s="20" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n"/>
@@ -5231,6 +5522,7 @@
       <c r="N143" s="2" t="n"/>
       <c r="O143" s="1" t="n"/>
       <c r="P143" s="1" t="n"/>
+      <c r="R143" s="20" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n"/>
@@ -5249,6 +5541,7 @@
       <c r="N144" s="2" t="n"/>
       <c r="O144" s="1" t="n"/>
       <c r="P144" s="1" t="n"/>
+      <c r="R144" s="20" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n"/>
@@ -5267,6 +5560,7 @@
       <c r="N145" s="2" t="n"/>
       <c r="O145" s="1" t="n"/>
       <c r="P145" s="1" t="n"/>
+      <c r="R145" s="20" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n"/>
@@ -5285,6 +5579,7 @@
       <c r="N146" s="2" t="n"/>
       <c r="O146" s="1" t="n"/>
       <c r="P146" s="1" t="n"/>
+      <c r="R146" s="20" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n"/>
@@ -5303,6 +5598,7 @@
       <c r="N147" s="2" t="n"/>
       <c r="O147" s="1" t="n"/>
       <c r="P147" s="1" t="n"/>
+      <c r="R147" s="20" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n"/>
@@ -5321,6 +5617,7 @@
       <c r="N148" s="2" t="n"/>
       <c r="O148" s="1" t="n"/>
       <c r="P148" s="1" t="n"/>
+      <c r="R148" s="20" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n"/>
@@ -5339,6 +5636,7 @@
       <c r="N149" s="2" t="n"/>
       <c r="O149" s="1" t="n"/>
       <c r="P149" s="1" t="n"/>
+      <c r="R149" s="20" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n"/>
@@ -5357,6 +5655,7 @@
       <c r="N150" s="2" t="n"/>
       <c r="O150" s="1" t="n"/>
       <c r="P150" s="1" t="n"/>
+      <c r="R150" s="20" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n"/>
@@ -5375,6 +5674,7 @@
       <c r="N151" s="2" t="n"/>
       <c r="O151" s="1" t="n"/>
       <c r="P151" s="1" t="n"/>
+      <c r="R151" s="20" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n"/>
@@ -5393,6 +5693,7 @@
       <c r="N152" s="2" t="n"/>
       <c r="O152" s="1" t="n"/>
       <c r="P152" s="1" t="n"/>
+      <c r="R152" s="20" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n"/>
@@ -5411,6 +5712,7 @@
       <c r="N153" s="2" t="n"/>
       <c r="O153" s="1" t="n"/>
       <c r="P153" s="1" t="n"/>
+      <c r="R153" s="20" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n"/>
@@ -5429,6 +5731,7 @@
       <c r="N154" s="2" t="n"/>
       <c r="O154" s="1" t="n"/>
       <c r="P154" s="1" t="n"/>
+      <c r="R154" s="20" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n"/>
@@ -5447,6 +5750,7 @@
       <c r="N155" s="2" t="n"/>
       <c r="O155" s="1" t="n"/>
       <c r="P155" s="1" t="n"/>
+      <c r="R155" s="20" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n"/>
@@ -5465,6 +5769,7 @@
       <c r="N156" s="2" t="n"/>
       <c r="O156" s="1" t="n"/>
       <c r="P156" s="1" t="n"/>
+      <c r="R156" s="20" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n"/>
@@ -5483,6 +5788,7 @@
       <c r="N157" s="2" t="n"/>
       <c r="O157" s="1" t="n"/>
       <c r="P157" s="1" t="n"/>
+      <c r="R157" s="20" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n"/>
@@ -5501,6 +5807,7 @@
       <c r="N158" s="2" t="n"/>
       <c r="O158" s="1" t="n"/>
       <c r="P158" s="1" t="n"/>
+      <c r="R158" s="20" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n"/>
@@ -5519,6 +5826,7 @@
       <c r="N159" s="2" t="n"/>
       <c r="O159" s="1" t="n"/>
       <c r="P159" s="1" t="n"/>
+      <c r="R159" s="20" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n"/>
@@ -5537,6 +5845,7 @@
       <c r="N160" s="2" t="n"/>
       <c r="O160" s="1" t="n"/>
       <c r="P160" s="1" t="n"/>
+      <c r="R160" s="20" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n"/>
@@ -5555,6 +5864,7 @@
       <c r="N161" s="2" t="n"/>
       <c r="O161" s="1" t="n"/>
       <c r="P161" s="1" t="n"/>
+      <c r="R161" s="20" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n"/>
@@ -5573,6 +5883,7 @@
       <c r="N162" s="2" t="n"/>
       <c r="O162" s="1" t="n"/>
       <c r="P162" s="1" t="n"/>
+      <c r="R162" s="20" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n"/>
@@ -5591,6 +5902,7 @@
       <c r="N163" s="2" t="n"/>
       <c r="O163" s="1" t="n"/>
       <c r="P163" s="1" t="n"/>
+      <c r="R163" s="20" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n"/>
@@ -5609,6 +5921,7 @@
       <c r="N164" s="2" t="n"/>
       <c r="O164" s="1" t="n"/>
       <c r="P164" s="1" t="n"/>
+      <c r="R164" s="20" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n"/>
@@ -5627,6 +5940,7 @@
       <c r="N165" s="2" t="n"/>
       <c r="O165" s="1" t="n"/>
       <c r="P165" s="1" t="n"/>
+      <c r="R165" s="20" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n"/>
@@ -5645,6 +5959,7 @@
       <c r="N166" s="2" t="n"/>
       <c r="O166" s="1" t="n"/>
       <c r="P166" s="1" t="n"/>
+      <c r="R166" s="20" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n"/>
@@ -5663,6 +5978,7 @@
       <c r="N167" s="2" t="n"/>
       <c r="O167" s="1" t="n"/>
       <c r="P167" s="1" t="n"/>
+      <c r="R167" s="20" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n"/>
@@ -5681,6 +5997,7 @@
       <c r="N168" s="2" t="n"/>
       <c r="O168" s="1" t="n"/>
       <c r="P168" s="1" t="n"/>
+      <c r="R168" s="20" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n"/>
@@ -5699,6 +6016,7 @@
       <c r="N169" s="2" t="n"/>
       <c r="O169" s="1" t="n"/>
       <c r="P169" s="1" t="n"/>
+      <c r="R169" s="20" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n"/>
@@ -5717,6 +6035,7 @@
       <c r="N170" s="2" t="n"/>
       <c r="O170" s="1" t="n"/>
       <c r="P170" s="1" t="n"/>
+      <c r="R170" s="20" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n"/>
@@ -5735,6 +6054,7 @@
       <c r="N171" s="2" t="n"/>
       <c r="O171" s="1" t="n"/>
       <c r="P171" s="1" t="n"/>
+      <c r="R171" s="20" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n"/>
@@ -5753,6 +6073,7 @@
       <c r="N172" s="2" t="n"/>
       <c r="O172" s="1" t="n"/>
       <c r="P172" s="1" t="n"/>
+      <c r="R172" s="20" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n"/>
@@ -5771,6 +6092,7 @@
       <c r="N173" s="2" t="n"/>
       <c r="O173" s="1" t="n"/>
       <c r="P173" s="1" t="n"/>
+      <c r="R173" s="20" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n"/>
@@ -5789,6 +6111,7 @@
       <c r="N174" s="2" t="n"/>
       <c r="O174" s="1" t="n"/>
       <c r="P174" s="1" t="n"/>
+      <c r="R174" s="20" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n"/>
@@ -5807,6 +6130,7 @@
       <c r="N175" s="2" t="n"/>
       <c r="O175" s="1" t="n"/>
       <c r="P175" s="1" t="n"/>
+      <c r="R175" s="20" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n"/>
@@ -5825,6 +6149,7 @@
       <c r="N176" s="2" t="n"/>
       <c r="O176" s="1" t="n"/>
       <c r="P176" s="1" t="n"/>
+      <c r="R176" s="20" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n"/>
@@ -5843,6 +6168,7 @@
       <c r="N177" s="2" t="n"/>
       <c r="O177" s="1" t="n"/>
       <c r="P177" s="1" t="n"/>
+      <c r="R177" s="20" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n"/>
@@ -5861,6 +6187,7 @@
       <c r="N178" s="2" t="n"/>
       <c r="O178" s="1" t="n"/>
       <c r="P178" s="1" t="n"/>
+      <c r="R178" s="20" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n"/>
@@ -5879,6 +6206,7 @@
       <c r="N179" s="2" t="n"/>
       <c r="O179" s="1" t="n"/>
       <c r="P179" s="1" t="n"/>
+      <c r="R179" s="20" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n"/>
@@ -5897,6 +6225,7 @@
       <c r="N180" s="2" t="n"/>
       <c r="O180" s="1" t="n"/>
       <c r="P180" s="1" t="n"/>
+      <c r="R180" s="20" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n"/>
@@ -5915,6 +6244,7 @@
       <c r="N181" s="2" t="n"/>
       <c r="O181" s="1" t="n"/>
       <c r="P181" s="1" t="n"/>
+      <c r="R181" s="20" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n"/>
@@ -5933,6 +6263,7 @@
       <c r="N182" s="2" t="n"/>
       <c r="O182" s="1" t="n"/>
       <c r="P182" s="1" t="n"/>
+      <c r="R182" s="20" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n"/>
@@ -5951,6 +6282,7 @@
       <c r="N183" s="2" t="n"/>
       <c r="O183" s="1" t="n"/>
       <c r="P183" s="1" t="n"/>
+      <c r="R183" s="20" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n"/>
@@ -5969,6 +6301,7 @@
       <c r="N184" s="2" t="n"/>
       <c r="O184" s="1" t="n"/>
       <c r="P184" s="1" t="n"/>
+      <c r="R184" s="20" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n"/>
@@ -5987,6 +6320,7 @@
       <c r="N185" s="2" t="n"/>
       <c r="O185" s="1" t="n"/>
       <c r="P185" s="1" t="n"/>
+      <c r="R185" s="20" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n"/>
@@ -6005,6 +6339,7 @@
       <c r="N186" s="2" t="n"/>
       <c r="O186" s="1" t="n"/>
       <c r="P186" s="1" t="n"/>
+      <c r="R186" s="20" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n"/>
@@ -6023,6 +6358,7 @@
       <c r="N187" s="2" t="n"/>
       <c r="O187" s="1" t="n"/>
       <c r="P187" s="1" t="n"/>
+      <c r="R187" s="20" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n"/>
@@ -6041,6 +6377,7 @@
       <c r="N188" s="2" t="n"/>
       <c r="O188" s="1" t="n"/>
       <c r="P188" s="1" t="n"/>
+      <c r="R188" s="20" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n"/>
@@ -6059,6 +6396,7 @@
       <c r="N189" s="2" t="n"/>
       <c r="O189" s="1" t="n"/>
       <c r="P189" s="1" t="n"/>
+      <c r="R189" s="20" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n"/>
@@ -6077,6 +6415,7 @@
       <c r="N190" s="2" t="n"/>
       <c r="O190" s="1" t="n"/>
       <c r="P190" s="1" t="n"/>
+      <c r="R190" s="20" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n"/>
@@ -6095,6 +6434,7 @@
       <c r="N191" s="2" t="n"/>
       <c r="O191" s="1" t="n"/>
       <c r="P191" s="1" t="n"/>
+      <c r="R191" s="20" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n"/>
@@ -6113,6 +6453,7 @@
       <c r="N192" s="2" t="n"/>
       <c r="O192" s="1" t="n"/>
       <c r="P192" s="1" t="n"/>
+      <c r="R192" s="20" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n"/>
@@ -6131,6 +6472,7 @@
       <c r="N193" s="2" t="n"/>
       <c r="O193" s="1" t="n"/>
       <c r="P193" s="1" t="n"/>
+      <c r="R193" s="20" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n"/>
@@ -6149,6 +6491,7 @@
       <c r="N194" s="2" t="n"/>
       <c r="O194" s="1" t="n"/>
       <c r="P194" s="1" t="n"/>
+      <c r="R194" s="20" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n"/>
@@ -6167,6 +6510,7 @@
       <c r="N195" s="2" t="n"/>
       <c r="O195" s="1" t="n"/>
       <c r="P195" s="1" t="n"/>
+      <c r="R195" s="20" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n"/>
@@ -6185,6 +6529,7 @@
       <c r="N196" s="2" t="n"/>
       <c r="O196" s="1" t="n"/>
       <c r="P196" s="1" t="n"/>
+      <c r="R196" s="20" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n"/>
@@ -6203,6 +6548,7 @@
       <c r="N197" s="2" t="n"/>
       <c r="O197" s="1" t="n"/>
       <c r="P197" s="1" t="n"/>
+      <c r="R197" s="20" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n"/>
@@ -6221,6 +6567,7 @@
       <c r="N198" s="2" t="n"/>
       <c r="O198" s="1" t="n"/>
       <c r="P198" s="1" t="n"/>
+      <c r="R198" s="20" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n"/>
@@ -6239,6 +6586,7 @@
       <c r="N199" s="2" t="n"/>
       <c r="O199" s="1" t="n"/>
       <c r="P199" s="1" t="n"/>
+      <c r="R199" s="20" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n"/>
@@ -6257,6 +6605,7 @@
       <c r="N200" s="2" t="n"/>
       <c r="O200" s="1" t="n"/>
       <c r="P200" s="1" t="n"/>
+      <c r="R200" s="20" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n"/>
@@ -6275,6 +6624,7 @@
       <c r="N201" s="2" t="n"/>
       <c r="O201" s="1" t="n"/>
       <c r="P201" s="1" t="n"/>
+      <c r="R201" s="20" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n"/>
@@ -6293,6 +6643,7 @@
       <c r="N202" s="2" t="n"/>
       <c r="O202" s="1" t="n"/>
       <c r="P202" s="1" t="n"/>
+      <c r="R202" s="20" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n"/>
@@ -6311,6 +6662,7 @@
       <c r="N203" s="2" t="n"/>
       <c r="O203" s="1" t="n"/>
       <c r="P203" s="1" t="n"/>
+      <c r="R203" s="20" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n"/>
@@ -6329,6 +6681,7 @@
       <c r="N204" s="2" t="n"/>
       <c r="O204" s="1" t="n"/>
       <c r="P204" s="1" t="n"/>
+      <c r="R204" s="20" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n"/>
@@ -6347,6 +6700,7 @@
       <c r="N205" s="2" t="n"/>
       <c r="O205" s="1" t="n"/>
       <c r="P205" s="1" t="n"/>
+      <c r="R205" s="20" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n"/>
@@ -6365,6 +6719,7 @@
       <c r="N206" s="2" t="n"/>
       <c r="O206" s="1" t="n"/>
       <c r="P206" s="1" t="n"/>
+      <c r="R206" s="20" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n"/>
@@ -6383,6 +6738,7 @@
       <c r="N207" s="2" t="n"/>
       <c r="O207" s="1" t="n"/>
       <c r="P207" s="1" t="n"/>
+      <c r="R207" s="20" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="1" t="n"/>
@@ -6401,6 +6757,7 @@
       <c r="N208" s="2" t="n"/>
       <c r="O208" s="1" t="n"/>
       <c r="P208" s="1" t="n"/>
+      <c r="R208" s="20" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="1" t="n"/>
@@ -6419,6 +6776,7 @@
       <c r="N209" s="2" t="n"/>
       <c r="O209" s="1" t="n"/>
       <c r="P209" s="1" t="n"/>
+      <c r="R209" s="20" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="1" t="n"/>
@@ -6437,6 +6795,7 @@
       <c r="N210" s="2" t="n"/>
       <c r="O210" s="1" t="n"/>
       <c r="P210" s="1" t="n"/>
+      <c r="R210" s="20" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="1" t="n"/>
@@ -6455,6 +6814,7 @@
       <c r="N211" s="2" t="n"/>
       <c r="O211" s="1" t="n"/>
       <c r="P211" s="1" t="n"/>
+      <c r="R211" s="20" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="1" t="n"/>
@@ -6473,6 +6833,7 @@
       <c r="N212" s="2" t="n"/>
       <c r="O212" s="1" t="n"/>
       <c r="P212" s="1" t="n"/>
+      <c r="R212" s="20" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n"/>
@@ -6491,6 +6852,7 @@
       <c r="N213" s="2" t="n"/>
       <c r="O213" s="1" t="n"/>
       <c r="P213" s="1" t="n"/>
+      <c r="R213" s="20" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="1" t="n"/>
@@ -6509,6 +6871,7 @@
       <c r="N214" s="2" t="n"/>
       <c r="O214" s="1" t="n"/>
       <c r="P214" s="1" t="n"/>
+      <c r="R214" s="20" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n"/>
@@ -6527,6 +6890,7 @@
       <c r="N215" s="2" t="n"/>
       <c r="O215" s="1" t="n"/>
       <c r="P215" s="1" t="n"/>
+      <c r="R215" s="20" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n"/>
@@ -6545,6 +6909,7 @@
       <c r="N216" s="2" t="n"/>
       <c r="O216" s="1" t="n"/>
       <c r="P216" s="1" t="n"/>
+      <c r="R216" s="20" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n"/>
@@ -6563,6 +6928,7 @@
       <c r="N217" s="2" t="n"/>
       <c r="O217" s="1" t="n"/>
       <c r="P217" s="1" t="n"/>
+      <c r="R217" s="20" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n"/>
@@ -6581,6 +6947,7 @@
       <c r="N218" s="2" t="n"/>
       <c r="O218" s="1" t="n"/>
       <c r="P218" s="1" t="n"/>
+      <c r="R218" s="20" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="1" t="n"/>
@@ -6599,6 +6966,7 @@
       <c r="N219" s="2" t="n"/>
       <c r="O219" s="1" t="n"/>
       <c r="P219" s="1" t="n"/>
+      <c r="R219" s="20" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n"/>
@@ -6617,6 +6985,7 @@
       <c r="N220" s="2" t="n"/>
       <c r="O220" s="1" t="n"/>
       <c r="P220" s="1" t="n"/>
+      <c r="R220" s="20" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n"/>
@@ -6635,6 +7004,7 @@
       <c r="N221" s="2" t="n"/>
       <c r="O221" s="1" t="n"/>
       <c r="P221" s="1" t="n"/>
+      <c r="R221" s="20" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n"/>
@@ -6653,6 +7023,7 @@
       <c r="N222" s="2" t="n"/>
       <c r="O222" s="1" t="n"/>
       <c r="P222" s="1" t="n"/>
+      <c r="R222" s="20" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n"/>
@@ -6671,6 +7042,7 @@
       <c r="N223" s="2" t="n"/>
       <c r="O223" s="1" t="n"/>
       <c r="P223" s="1" t="n"/>
+      <c r="R223" s="20" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n"/>
@@ -6689,6 +7061,7 @@
       <c r="N224" s="2" t="n"/>
       <c r="O224" s="1" t="n"/>
       <c r="P224" s="1" t="n"/>
+      <c r="R224" s="20" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n"/>
@@ -6707,6 +7080,7 @@
       <c r="N225" s="2" t="n"/>
       <c r="O225" s="1" t="n"/>
       <c r="P225" s="1" t="n"/>
+      <c r="R225" s="20" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n"/>
@@ -6725,6 +7099,7 @@
       <c r="N226" s="2" t="n"/>
       <c r="O226" s="1" t="n"/>
       <c r="P226" s="1" t="n"/>
+      <c r="R226" s="20" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n"/>
@@ -6743,6 +7118,7 @@
       <c r="N227" s="2" t="n"/>
       <c r="O227" s="1" t="n"/>
       <c r="P227" s="1" t="n"/>
+      <c r="R227" s="20" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n"/>
@@ -6761,6 +7137,7 @@
       <c r="N228" s="2" t="n"/>
       <c r="O228" s="1" t="n"/>
       <c r="P228" s="1" t="n"/>
+      <c r="R228" s="20" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n"/>
@@ -6779,6 +7156,7 @@
       <c r="N229" s="2" t="n"/>
       <c r="O229" s="1" t="n"/>
       <c r="P229" s="1" t="n"/>
+      <c r="R229" s="20" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n"/>
@@ -6797,6 +7175,7 @@
       <c r="N230" s="2" t="n"/>
       <c r="O230" s="1" t="n"/>
       <c r="P230" s="1" t="n"/>
+      <c r="R230" s="20" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="1" t="n"/>
@@ -6815,6 +7194,7 @@
       <c r="N231" s="2" t="n"/>
       <c r="O231" s="1" t="n"/>
       <c r="P231" s="1" t="n"/>
+      <c r="R231" s="20" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="1" t="n"/>
@@ -6833,6 +7213,7 @@
       <c r="N232" s="2" t="n"/>
       <c r="O232" s="1" t="n"/>
       <c r="P232" s="1" t="n"/>
+      <c r="R232" s="20" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n"/>
@@ -6851,6 +7232,7 @@
       <c r="N233" s="2" t="n"/>
       <c r="O233" s="1" t="n"/>
       <c r="P233" s="1" t="n"/>
+      <c r="R233" s="20" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n"/>
@@ -6869,6 +7251,7 @@
       <c r="N234" s="2" t="n"/>
       <c r="O234" s="1" t="n"/>
       <c r="P234" s="1" t="n"/>
+      <c r="R234" s="20" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="1" t="n"/>
@@ -6887,6 +7270,7 @@
       <c r="N235" s="2" t="n"/>
       <c r="O235" s="1" t="n"/>
       <c r="P235" s="1" t="n"/>
+      <c r="R235" s="20" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="1" t="n"/>
@@ -6905,6 +7289,7 @@
       <c r="N236" s="2" t="n"/>
       <c r="O236" s="1" t="n"/>
       <c r="P236" s="1" t="n"/>
+      <c r="R236" s="20" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="1" t="n"/>
@@ -6923,6 +7308,7 @@
       <c r="N237" s="2" t="n"/>
       <c r="O237" s="1" t="n"/>
       <c r="P237" s="1" t="n"/>
+      <c r="R237" s="20" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="1" t="n"/>
@@ -6941,6 +7327,7 @@
       <c r="N238" s="2" t="n"/>
       <c r="O238" s="1" t="n"/>
       <c r="P238" s="1" t="n"/>
+      <c r="R238" s="20" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="1" t="n"/>
@@ -6959,6 +7346,7 @@
       <c r="N239" s="2" t="n"/>
       <c r="O239" s="1" t="n"/>
       <c r="P239" s="1" t="n"/>
+      <c r="R239" s="20" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n"/>
@@ -6977,6 +7365,7 @@
       <c r="N240" s="2" t="n"/>
       <c r="O240" s="1" t="n"/>
       <c r="P240" s="1" t="n"/>
+      <c r="R240" s="20" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n"/>
@@ -6995,6 +7384,7 @@
       <c r="N241" s="2" t="n"/>
       <c r="O241" s="1" t="n"/>
       <c r="P241" s="1" t="n"/>
+      <c r="R241" s="20" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="1" t="n"/>
@@ -7013,6 +7403,7 @@
       <c r="N242" s="2" t="n"/>
       <c r="O242" s="1" t="n"/>
       <c r="P242" s="1" t="n"/>
+      <c r="R242" s="20" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n"/>
@@ -7031,6 +7422,7 @@
       <c r="N243" s="2" t="n"/>
       <c r="O243" s="1" t="n"/>
       <c r="P243" s="1" t="n"/>
+      <c r="R243" s="20" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="1" t="n"/>
@@ -7049,6 +7441,7 @@
       <c r="N244" s="2" t="n"/>
       <c r="O244" s="1" t="n"/>
       <c r="P244" s="1" t="n"/>
+      <c r="R244" s="20" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n"/>
@@ -7067,6 +7460,7 @@
       <c r="N245" s="2" t="n"/>
       <c r="O245" s="1" t="n"/>
       <c r="P245" s="1" t="n"/>
+      <c r="R245" s="20" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n"/>
@@ -7085,6 +7479,7 @@
       <c r="N246" s="2" t="n"/>
       <c r="O246" s="1" t="n"/>
       <c r="P246" s="1" t="n"/>
+      <c r="R246" s="20" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="1" t="n"/>
@@ -7103,6 +7498,7 @@
       <c r="N247" s="2" t="n"/>
       <c r="O247" s="1" t="n"/>
       <c r="P247" s="1" t="n"/>
+      <c r="R247" s="20" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="1" t="n"/>
@@ -7121,6 +7517,7 @@
       <c r="N248" s="2" t="n"/>
       <c r="O248" s="1" t="n"/>
       <c r="P248" s="1" t="n"/>
+      <c r="R248" s="20" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n"/>
@@ -7139,6 +7536,7 @@
       <c r="N249" s="2" t="n"/>
       <c r="O249" s="1" t="n"/>
       <c r="P249" s="1" t="n"/>
+      <c r="R249" s="20" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="1" t="n"/>
@@ -7157,6 +7555,7 @@
       <c r="N250" s="2" t="n"/>
       <c r="O250" s="1" t="n"/>
       <c r="P250" s="1" t="n"/>
+      <c r="R250" s="20" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="1" t="n"/>
@@ -7175,6 +7574,7 @@
       <c r="N251" s="2" t="n"/>
       <c r="O251" s="1" t="n"/>
       <c r="P251" s="1" t="n"/>
+      <c r="R251" s="20" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="1" t="n"/>
@@ -7193,6 +7593,7 @@
       <c r="N252" s="2" t="n"/>
       <c r="O252" s="1" t="n"/>
       <c r="P252" s="1" t="n"/>
+      <c r="R252" s="20" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="1" t="n"/>
@@ -7211,6 +7612,7 @@
       <c r="N253" s="2" t="n"/>
       <c r="O253" s="1" t="n"/>
       <c r="P253" s="1" t="n"/>
+      <c r="R253" s="20" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="1" t="n"/>
@@ -7229,6 +7631,7 @@
       <c r="N254" s="2" t="n"/>
       <c r="O254" s="1" t="n"/>
       <c r="P254" s="1" t="n"/>
+      <c r="R254" s="20" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="1" t="n"/>
@@ -7247,6 +7650,7 @@
       <c r="N255" s="2" t="n"/>
       <c r="O255" s="1" t="n"/>
       <c r="P255" s="1" t="n"/>
+      <c r="R255" s="20" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="1" t="n"/>
@@ -7265,6 +7669,7 @@
       <c r="N256" s="2" t="n"/>
       <c r="O256" s="1" t="n"/>
       <c r="P256" s="1" t="n"/>
+      <c r="R256" s="20" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="1" t="n"/>
@@ -7283,6 +7688,7 @@
       <c r="N257" s="2" t="n"/>
       <c r="O257" s="1" t="n"/>
       <c r="P257" s="1" t="n"/>
+      <c r="R257" s="20" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="1" t="n"/>
@@ -7301,6 +7707,7 @@
       <c r="N258" s="2" t="n"/>
       <c r="O258" s="1" t="n"/>
       <c r="P258" s="1" t="n"/>
+      <c r="R258" s="20" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="1" t="n"/>
@@ -7319,6 +7726,7 @@
       <c r="N259" s="2" t="n"/>
       <c r="O259" s="1" t="n"/>
       <c r="P259" s="1" t="n"/>
+      <c r="R259" s="20" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="1" t="n"/>
@@ -7337,6 +7745,7 @@
       <c r="N260" s="2" t="n"/>
       <c r="O260" s="1" t="n"/>
       <c r="P260" s="1" t="n"/>
+      <c r="R260" s="20" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="1" t="n"/>
@@ -7355,6 +7764,7 @@
       <c r="N261" s="2" t="n"/>
       <c r="O261" s="1" t="n"/>
       <c r="P261" s="1" t="n"/>
+      <c r="R261" s="20" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="1" t="n"/>
@@ -7373,6 +7783,7 @@
       <c r="N262" s="2" t="n"/>
       <c r="O262" s="1" t="n"/>
       <c r="P262" s="1" t="n"/>
+      <c r="R262" s="20" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="1" t="n"/>
@@ -7391,6 +7802,7 @@
       <c r="N263" s="2" t="n"/>
       <c r="O263" s="1" t="n"/>
       <c r="P263" s="1" t="n"/>
+      <c r="R263" s="20" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="1" t="n"/>
@@ -7409,6 +7821,7 @@
       <c r="N264" s="2" t="n"/>
       <c r="O264" s="1" t="n"/>
       <c r="P264" s="1" t="n"/>
+      <c r="R264" s="20" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="1" t="n"/>
@@ -7427,6 +7840,7 @@
       <c r="N265" s="2" t="n"/>
       <c r="O265" s="1" t="n"/>
       <c r="P265" s="1" t="n"/>
+      <c r="R265" s="20" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="1" t="n"/>
@@ -7445,6 +7859,7 @@
       <c r="N266" s="2" t="n"/>
       <c r="O266" s="1" t="n"/>
       <c r="P266" s="1" t="n"/>
+      <c r="R266" s="20" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="1" t="n"/>
@@ -7463,6 +7878,7 @@
       <c r="N267" s="2" t="n"/>
       <c r="O267" s="1" t="n"/>
       <c r="P267" s="1" t="n"/>
+      <c r="R267" s="20" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="1" t="n"/>
@@ -7481,6 +7897,7 @@
       <c r="N268" s="2" t="n"/>
       <c r="O268" s="1" t="n"/>
       <c r="P268" s="1" t="n"/>
+      <c r="R268" s="20" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="1" t="n"/>
@@ -7499,6 +7916,7 @@
       <c r="N269" s="2" t="n"/>
       <c r="O269" s="1" t="n"/>
       <c r="P269" s="1" t="n"/>
+      <c r="R269" s="20" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="1" t="n"/>
@@ -7517,6 +7935,7 @@
       <c r="N270" s="2" t="n"/>
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
+      <c r="R270" s="20" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="1" t="n"/>
@@ -7535,6 +7954,7 @@
       <c r="N271" s="2" t="n"/>
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
+      <c r="R271" s="20" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="1" t="n"/>
@@ -7553,6 +7973,7 @@
       <c r="N272" s="2" t="n"/>
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="1" t="n"/>
+      <c r="R272" s="20" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="1" t="n"/>
@@ -7571,6 +7992,7 @@
       <c r="N273" s="2" t="n"/>
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
+      <c r="R273" s="20" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="1" t="n"/>
@@ -7589,6 +8011,7 @@
       <c r="N274" s="2" t="n"/>
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
+      <c r="R274" s="20" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="1" t="n"/>
@@ -7607,6 +8030,7 @@
       <c r="N275" s="2" t="n"/>
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
+      <c r="R275" s="20" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="1" t="n"/>
@@ -7625,6 +8049,7 @@
       <c r="N276" s="2" t="n"/>
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
+      <c r="R276" s="20" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="1" t="n"/>
@@ -7643,6 +8068,7 @@
       <c r="N277" s="2" t="n"/>
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
+      <c r="R277" s="20" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="1" t="n"/>
@@ -7661,6 +8087,7 @@
       <c r="N278" s="2" t="n"/>
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
+      <c r="R278" s="20" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="1" t="n"/>
@@ -7679,6 +8106,7 @@
       <c r="N279" s="2" t="n"/>
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
+      <c r="R279" s="20" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="1" t="n"/>
@@ -7697,6 +8125,7 @@
       <c r="N280" s="2" t="n"/>
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
+      <c r="R280" s="20" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="1" t="n"/>
@@ -7715,6 +8144,7 @@
       <c r="N281" s="2" t="n"/>
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
+      <c r="R281" s="20" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="1" t="n"/>
@@ -7733,6 +8163,7 @@
       <c r="N282" s="2" t="n"/>
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
+      <c r="R282" s="20" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n"/>
@@ -7751,6 +8182,7 @@
       <c r="N283" s="2" t="n"/>
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
+      <c r="R283" s="20" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="1" t="n"/>
@@ -7769,6 +8201,7 @@
       <c r="N284" s="2" t="n"/>
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
+      <c r="R284" s="20" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="1" t="n"/>
@@ -7787,6 +8220,7 @@
       <c r="N285" s="2" t="n"/>
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
+      <c r="R285" s="20" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="1" t="n"/>
@@ -7805,6 +8239,7 @@
       <c r="N286" s="2" t="n"/>
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="n"/>
+      <c r="R286" s="20" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="1" t="n"/>
@@ -7823,6 +8258,7 @@
       <c r="N287" s="2" t="n"/>
       <c r="O287" s="1" t="n"/>
       <c r="P287" s="1" t="n"/>
+      <c r="R287" s="20" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="1" t="n"/>
@@ -7841,6 +8277,7 @@
       <c r="N288" s="2" t="n"/>
       <c r="O288" s="1" t="n"/>
       <c r="P288" s="1" t="n"/>
+      <c r="R288" s="20" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="1" t="n"/>
@@ -7859,6 +8296,7 @@
       <c r="N289" s="2" t="n"/>
       <c r="O289" s="1" t="n"/>
       <c r="P289" s="1" t="n"/>
+      <c r="R289" s="20" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="1" t="n"/>
@@ -7877,6 +8315,7 @@
       <c r="N290" s="2" t="n"/>
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
+      <c r="R290" s="20" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n"/>
@@ -7895,6 +8334,7 @@
       <c r="N291" s="2" t="n"/>
       <c r="O291" s="1" t="n"/>
       <c r="P291" s="1" t="n"/>
+      <c r="R291" s="20" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="1" t="n"/>
@@ -7913,6 +8353,7 @@
       <c r="N292" s="2" t="n"/>
       <c r="O292" s="1" t="n"/>
       <c r="P292" s="1" t="n"/>
+      <c r="R292" s="20" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="1" t="n"/>
@@ -7931,6 +8372,7 @@
       <c r="N293" s="2" t="n"/>
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
+      <c r="R293" s="20" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="1" t="n"/>
@@ -7949,6 +8391,7 @@
       <c r="N294" s="2" t="n"/>
       <c r="O294" s="1" t="n"/>
       <c r="P294" s="1" t="n"/>
+      <c r="R294" s="20" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="1" t="n"/>
@@ -7967,6 +8410,7 @@
       <c r="N295" s="2" t="n"/>
       <c r="O295" s="1" t="n"/>
       <c r="P295" s="1" t="n"/>
+      <c r="R295" s="20" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="1" t="n"/>
@@ -7985,6 +8429,7 @@
       <c r="N296" s="2" t="n"/>
       <c r="O296" s="1" t="n"/>
       <c r="P296" s="1" t="n"/>
+      <c r="R296" s="20" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="1" t="n"/>
@@ -8003,6 +8448,7 @@
       <c r="N297" s="2" t="n"/>
       <c r="O297" s="1" t="n"/>
       <c r="P297" s="1" t="n"/>
+      <c r="R297" s="20" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="1" t="n"/>
@@ -8021,6 +8467,7 @@
       <c r="N298" s="2" t="n"/>
       <c r="O298" s="1" t="n"/>
       <c r="P298" s="1" t="n"/>
+      <c r="R298" s="20" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n"/>
@@ -8039,6 +8486,7 @@
       <c r="N299" s="2" t="n"/>
       <c r="O299" s="1" t="n"/>
       <c r="P299" s="1" t="n"/>
+      <c r="R299" s="20" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="1" t="n"/>
@@ -8057,6 +8505,7 @@
       <c r="N300" s="2" t="n"/>
       <c r="O300" s="1" t="n"/>
       <c r="P300" s="1" t="n"/>
+      <c r="R300" s="20" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="1" t="n"/>
@@ -8075,6 +8524,7 @@
       <c r="N301" s="2" t="n"/>
       <c r="O301" s="1" t="n"/>
       <c r="P301" s="1" t="n"/>
+      <c r="R301" s="20" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="1" t="n"/>
@@ -8093,6 +8543,7 @@
       <c r="N302" s="2" t="n"/>
       <c r="O302" s="1" t="n"/>
       <c r="P302" s="1" t="n"/>
+      <c r="R302" s="20" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="1" t="n"/>
@@ -8111,6 +8562,7 @@
       <c r="N303" s="2" t="n"/>
       <c r="O303" s="1" t="n"/>
       <c r="P303" s="1" t="n"/>
+      <c r="R303" s="20" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="1" t="n"/>
@@ -8129,6 +8581,7 @@
       <c r="N304" s="2" t="n"/>
       <c r="O304" s="1" t="n"/>
       <c r="P304" s="1" t="n"/>
+      <c r="R304" s="20" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="1" t="n"/>
@@ -8147,6 +8600,7 @@
       <c r="N305" s="2" t="n"/>
       <c r="O305" s="1" t="n"/>
       <c r="P305" s="1" t="n"/>
+      <c r="R305" s="20" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="1" t="n"/>
@@ -8165,6 +8619,7 @@
       <c r="N306" s="2" t="n"/>
       <c r="O306" s="1" t="n"/>
       <c r="P306" s="1" t="n"/>
+      <c r="R306" s="20" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="1" t="n"/>
@@ -8183,6 +8638,7 @@
       <c r="N307" s="2" t="n"/>
       <c r="O307" s="1" t="n"/>
       <c r="P307" s="1" t="n"/>
+      <c r="R307" s="20" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="1" t="n"/>
@@ -8201,6 +8657,7 @@
       <c r="N308" s="2" t="n"/>
       <c r="O308" s="1" t="n"/>
       <c r="P308" s="1" t="n"/>
+      <c r="R308" s="20" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="1" t="n"/>
@@ -8219,6 +8676,7 @@
       <c r="N309" s="2" t="n"/>
       <c r="O309" s="1" t="n"/>
       <c r="P309" s="1" t="n"/>
+      <c r="R309" s="20" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="1" t="n"/>
@@ -8237,6 +8695,7 @@
       <c r="N310" s="2" t="n"/>
       <c r="O310" s="1" t="n"/>
       <c r="P310" s="1" t="n"/>
+      <c r="R310" s="20" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="1" t="n"/>
@@ -8255,6 +8714,7 @@
       <c r="N311" s="2" t="n"/>
       <c r="O311" s="1" t="n"/>
       <c r="P311" s="1" t="n"/>
+      <c r="R311" s="20" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="1" t="n"/>
@@ -8273,6 +8733,7 @@
       <c r="N312" s="2" t="n"/>
       <c r="O312" s="1" t="n"/>
       <c r="P312" s="1" t="n"/>
+      <c r="R312" s="20" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="1" t="n"/>
@@ -8291,6 +8752,7 @@
       <c r="N313" s="2" t="n"/>
       <c r="O313" s="1" t="n"/>
       <c r="P313" s="1" t="n"/>
+      <c r="R313" s="20" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="1" t="n"/>
@@ -8309,6 +8771,7 @@
       <c r="N314" s="2" t="n"/>
       <c r="O314" s="1" t="n"/>
       <c r="P314" s="1" t="n"/>
+      <c r="R314" s="20" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="1" t="n"/>
@@ -8327,6 +8790,7 @@
       <c r="N315" s="2" t="n"/>
       <c r="O315" s="1" t="n"/>
       <c r="P315" s="1" t="n"/>
+      <c r="R315" s="20" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="1" t="n"/>
@@ -8345,6 +8809,7 @@
       <c r="N316" s="2" t="n"/>
       <c r="O316" s="1" t="n"/>
       <c r="P316" s="1" t="n"/>
+      <c r="R316" s="20" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="1" t="n"/>
@@ -8363,6 +8828,7 @@
       <c r="N317" s="2" t="n"/>
       <c r="O317" s="1" t="n"/>
       <c r="P317" s="1" t="n"/>
+      <c r="R317" s="20" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="1" t="n"/>
@@ -8381,6 +8847,7 @@
       <c r="N318" s="2" t="n"/>
       <c r="O318" s="1" t="n"/>
       <c r="P318" s="1" t="n"/>
+      <c r="R318" s="20" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="1" t="n"/>
@@ -8399,6 +8866,7 @@
       <c r="N319" s="2" t="n"/>
       <c r="O319" s="1" t="n"/>
       <c r="P319" s="1" t="n"/>
+      <c r="R319" s="20" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="1" t="n"/>
@@ -8417,6 +8885,7 @@
       <c r="N320" s="2" t="n"/>
       <c r="O320" s="1" t="n"/>
       <c r="P320" s="1" t="n"/>
+      <c r="R320" s="20" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="1" t="n"/>
@@ -8435,6 +8904,7 @@
       <c r="N321" s="2" t="n"/>
       <c r="O321" s="1" t="n"/>
       <c r="P321" s="1" t="n"/>
+      <c r="R321" s="20" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="1" t="n"/>
@@ -8453,6 +8923,7 @@
       <c r="N322" s="2" t="n"/>
       <c r="O322" s="1" t="n"/>
       <c r="P322" s="1" t="n"/>
+      <c r="R322" s="20" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="1" t="n"/>
@@ -8471,6 +8942,7 @@
       <c r="N323" s="2" t="n"/>
       <c r="O323" s="1" t="n"/>
       <c r="P323" s="1" t="n"/>
+      <c r="R323" s="20" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="1" t="n"/>
@@ -8489,6 +8961,7 @@
       <c r="N324" s="2" t="n"/>
       <c r="O324" s="1" t="n"/>
       <c r="P324" s="1" t="n"/>
+      <c r="R324" s="20" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="1" t="n"/>
@@ -8507,6 +8980,7 @@
       <c r="N325" s="2" t="n"/>
       <c r="O325" s="1" t="n"/>
       <c r="P325" s="1" t="n"/>
+      <c r="R325" s="20" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="1" t="n"/>
@@ -8525,6 +8999,7 @@
       <c r="N326" s="2" t="n"/>
       <c r="O326" s="1" t="n"/>
       <c r="P326" s="1" t="n"/>
+      <c r="R326" s="20" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="1" t="n"/>
@@ -8543,6 +9018,7 @@
       <c r="N327" s="2" t="n"/>
       <c r="O327" s="1" t="n"/>
       <c r="P327" s="1" t="n"/>
+      <c r="R327" s="20" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="1" t="n"/>
@@ -8561,6 +9037,7 @@
       <c r="N328" s="2" t="n"/>
       <c r="O328" s="1" t="n"/>
       <c r="P328" s="1" t="n"/>
+      <c r="R328" s="20" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="1" t="n"/>
@@ -8579,6 +9056,7 @@
       <c r="N329" s="2" t="n"/>
       <c r="O329" s="1" t="n"/>
       <c r="P329" s="1" t="n"/>
+      <c r="R329" s="20" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="1" t="n"/>
@@ -8597,6 +9075,7 @@
       <c r="N330" s="2" t="n"/>
       <c r="O330" s="1" t="n"/>
       <c r="P330" s="1" t="n"/>
+      <c r="R330" s="20" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="1" t="n"/>
@@ -8615,6 +9094,7 @@
       <c r="N331" s="2" t="n"/>
       <c r="O331" s="1" t="n"/>
       <c r="P331" s="1" t="n"/>
+      <c r="R331" s="20" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="1" t="n"/>
@@ -8633,6 +9113,7 @@
       <c r="N332" s="2" t="n"/>
       <c r="O332" s="1" t="n"/>
       <c r="P332" s="1" t="n"/>
+      <c r="R332" s="20" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="1" t="n"/>
@@ -8651,6 +9132,7 @@
       <c r="N333" s="2" t="n"/>
       <c r="O333" s="1" t="n"/>
       <c r="P333" s="1" t="n"/>
+      <c r="R333" s="20" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="1" t="n"/>
@@ -8669,6 +9151,7 @@
       <c r="N334" s="2" t="n"/>
       <c r="O334" s="1" t="n"/>
       <c r="P334" s="1" t="n"/>
+      <c r="R334" s="20" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="1" t="n"/>
@@ -8687,6 +9170,7 @@
       <c r="N335" s="2" t="n"/>
       <c r="O335" s="1" t="n"/>
       <c r="P335" s="1" t="n"/>
+      <c r="R335" s="20" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="1" t="n"/>
@@ -8705,6 +9189,7 @@
       <c r="N336" s="2" t="n"/>
       <c r="O336" s="1" t="n"/>
       <c r="P336" s="1" t="n"/>
+      <c r="R336" s="20" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="1" t="n"/>
@@ -8723,6 +9208,7 @@
       <c r="N337" s="2" t="n"/>
       <c r="O337" s="1" t="n"/>
       <c r="P337" s="1" t="n"/>
+      <c r="R337" s="20" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="1" t="n"/>
@@ -8741,6 +9227,7 @@
       <c r="N338" s="2" t="n"/>
       <c r="O338" s="1" t="n"/>
       <c r="P338" s="1" t="n"/>
+      <c r="R338" s="20" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="1" t="n"/>
@@ -8759,6 +9246,7 @@
       <c r="N339" s="2" t="n"/>
       <c r="O339" s="1" t="n"/>
       <c r="P339" s="1" t="n"/>
+      <c r="R339" s="20" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="1" t="n"/>
@@ -8777,6 +9265,7 @@
       <c r="N340" s="2" t="n"/>
       <c r="O340" s="1" t="n"/>
       <c r="P340" s="1" t="n"/>
+      <c r="R340" s="20" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="1" t="n"/>
@@ -8795,6 +9284,7 @@
       <c r="N341" s="2" t="n"/>
       <c r="O341" s="1" t="n"/>
       <c r="P341" s="1" t="n"/>
+      <c r="R341" s="20" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="1" t="n"/>
@@ -8813,6 +9303,7 @@
       <c r="N342" s="2" t="n"/>
       <c r="O342" s="1" t="n"/>
       <c r="P342" s="1" t="n"/>
+      <c r="R342" s="20" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="1" t="n"/>
@@ -8831,6 +9322,7 @@
       <c r="N343" s="2" t="n"/>
       <c r="O343" s="1" t="n"/>
       <c r="P343" s="1" t="n"/>
+      <c r="R343" s="20" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="1" t="n"/>
@@ -8849,6 +9341,7 @@
       <c r="N344" s="2" t="n"/>
       <c r="O344" s="1" t="n"/>
       <c r="P344" s="1" t="n"/>
+      <c r="R344" s="20" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="1" t="n"/>
@@ -8867,6 +9360,7 @@
       <c r="N345" s="2" t="n"/>
       <c r="O345" s="1" t="n"/>
       <c r="P345" s="1" t="n"/>
+      <c r="R345" s="20" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="1" t="n"/>
@@ -8885,6 +9379,7 @@
       <c r="N346" s="2" t="n"/>
       <c r="O346" s="1" t="n"/>
       <c r="P346" s="1" t="n"/>
+      <c r="R346" s="20" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="1" t="n"/>
@@ -8903,6 +9398,7 @@
       <c r="N347" s="2" t="n"/>
       <c r="O347" s="1" t="n"/>
       <c r="P347" s="1" t="n"/>
+      <c r="R347" s="20" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="1" t="n"/>
@@ -8921,6 +9417,7 @@
       <c r="N348" s="2" t="n"/>
       <c r="O348" s="1" t="n"/>
       <c r="P348" s="1" t="n"/>
+      <c r="R348" s="20" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="1" t="n"/>
@@ -8939,6 +9436,7 @@
       <c r="N349" s="2" t="n"/>
       <c r="O349" s="1" t="n"/>
       <c r="P349" s="1" t="n"/>
+      <c r="R349" s="20" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="1" t="n"/>
@@ -8957,6 +9455,7 @@
       <c r="N350" s="2" t="n"/>
       <c r="O350" s="1" t="n"/>
       <c r="P350" s="1" t="n"/>
+      <c r="R350" s="20" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="1" t="n"/>
@@ -8975,6 +9474,7 @@
       <c r="N351" s="2" t="n"/>
       <c r="O351" s="1" t="n"/>
       <c r="P351" s="1" t="n"/>
+      <c r="R351" s="20" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="1" t="n"/>
@@ -8993,6 +9493,7 @@
       <c r="N352" s="2" t="n"/>
       <c r="O352" s="1" t="n"/>
       <c r="P352" s="1" t="n"/>
+      <c r="R352" s="20" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="1" t="n"/>
@@ -9011,6 +9512,7 @@
       <c r="N353" s="2" t="n"/>
       <c r="O353" s="1" t="n"/>
       <c r="P353" s="1" t="n"/>
+      <c r="R353" s="20" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="1" t="n"/>
@@ -9029,6 +9531,7 @@
       <c r="N354" s="2" t="n"/>
       <c r="O354" s="1" t="n"/>
       <c r="P354" s="1" t="n"/>
+      <c r="R354" s="20" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="1" t="n"/>
@@ -9047,6 +9550,7 @@
       <c r="N355" s="2" t="n"/>
       <c r="O355" s="1" t="n"/>
       <c r="P355" s="1" t="n"/>
+      <c r="R355" s="20" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="1" t="n"/>
@@ -9065,6 +9569,7 @@
       <c r="N356" s="2" t="n"/>
       <c r="O356" s="1" t="n"/>
       <c r="P356" s="1" t="n"/>
+      <c r="R356" s="20" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="1" t="n"/>
@@ -9083,6 +9588,7 @@
       <c r="N357" s="2" t="n"/>
       <c r="O357" s="1" t="n"/>
       <c r="P357" s="1" t="n"/>
+      <c r="R357" s="20" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="1" t="n"/>
@@ -9101,6 +9607,7 @@
       <c r="N358" s="2" t="n"/>
       <c r="O358" s="1" t="n"/>
       <c r="P358" s="1" t="n"/>
+      <c r="R358" s="20" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="1" t="n"/>
@@ -9119,6 +9626,7 @@
       <c r="N359" s="2" t="n"/>
       <c r="O359" s="1" t="n"/>
       <c r="P359" s="1" t="n"/>
+      <c r="R359" s="20" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="1" t="n"/>
@@ -9137,6 +9645,7 @@
       <c r="N360" s="2" t="n"/>
       <c r="O360" s="1" t="n"/>
       <c r="P360" s="1" t="n"/>
+      <c r="R360" s="20" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="1" t="n"/>
@@ -9155,6 +9664,7 @@
       <c r="N361" s="2" t="n"/>
       <c r="O361" s="1" t="n"/>
       <c r="P361" s="1" t="n"/>
+      <c r="R361" s="20" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="1" t="n"/>
@@ -9173,6 +9683,7 @@
       <c r="N362" s="2" t="n"/>
       <c r="O362" s="1" t="n"/>
       <c r="P362" s="1" t="n"/>
+      <c r="R362" s="20" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="1" t="n"/>
@@ -9191,6 +9702,7 @@
       <c r="N363" s="2" t="n"/>
       <c r="O363" s="1" t="n"/>
       <c r="P363" s="1" t="n"/>
+      <c r="R363" s="20" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="1" t="n"/>
@@ -9209,6 +9721,7 @@
       <c r="N364" s="2" t="n"/>
       <c r="O364" s="1" t="n"/>
       <c r="P364" s="1" t="n"/>
+      <c r="R364" s="20" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="1" t="n"/>
@@ -9227,6 +9740,7 @@
       <c r="N365" s="2" t="n"/>
       <c r="O365" s="1" t="n"/>
       <c r="P365" s="1" t="n"/>
+      <c r="R365" s="20" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="1" t="n"/>
@@ -9245,6 +9759,7 @@
       <c r="N366" s="2" t="n"/>
       <c r="O366" s="1" t="n"/>
       <c r="P366" s="1" t="n"/>
+      <c r="R366" s="20" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="1" t="n"/>
@@ -9263,6 +9778,7 @@
       <c r="N367" s="2" t="n"/>
       <c r="O367" s="1" t="n"/>
       <c r="P367" s="1" t="n"/>
+      <c r="R367" s="20" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="1" t="n"/>
@@ -9281,6 +9797,7 @@
       <c r="N368" s="2" t="n"/>
       <c r="O368" s="1" t="n"/>
       <c r="P368" s="1" t="n"/>
+      <c r="R368" s="20" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="1" t="n"/>
@@ -9299,6 +9816,7 @@
       <c r="N369" s="2" t="n"/>
       <c r="O369" s="1" t="n"/>
       <c r="P369" s="1" t="n"/>
+      <c r="R369" s="20" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="1" t="n"/>
@@ -9317,6 +9835,7 @@
       <c r="N370" s="2" t="n"/>
       <c r="O370" s="1" t="n"/>
       <c r="P370" s="1" t="n"/>
+      <c r="R370" s="20" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="1" t="n"/>
@@ -9335,6 +9854,7 @@
       <c r="N371" s="2" t="n"/>
       <c r="O371" s="1" t="n"/>
       <c r="P371" s="1" t="n"/>
+      <c r="R371" s="20" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="1" t="n"/>
@@ -9353,6 +9873,7 @@
       <c r="N372" s="2" t="n"/>
       <c r="O372" s="1" t="n"/>
       <c r="P372" s="1" t="n"/>
+      <c r="R372" s="20" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="1" t="n"/>
@@ -9371,6 +9892,7 @@
       <c r="N373" s="2" t="n"/>
       <c r="O373" s="1" t="n"/>
       <c r="P373" s="1" t="n"/>
+      <c r="R373" s="20" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="1" t="n"/>
@@ -9389,6 +9911,7 @@
       <c r="N374" s="2" t="n"/>
       <c r="O374" s="1" t="n"/>
       <c r="P374" s="1" t="n"/>
+      <c r="R374" s="20" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="1" t="n"/>
@@ -9407,6 +9930,7 @@
       <c r="N375" s="2" t="n"/>
       <c r="O375" s="1" t="n"/>
       <c r="P375" s="1" t="n"/>
+      <c r="R375" s="20" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="1" t="n"/>
@@ -9425,6 +9949,7 @@
       <c r="N376" s="2" t="n"/>
       <c r="O376" s="1" t="n"/>
       <c r="P376" s="1" t="n"/>
+      <c r="R376" s="20" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="1" t="n"/>
@@ -9443,6 +9968,7 @@
       <c r="N377" s="2" t="n"/>
       <c r="O377" s="1" t="n"/>
       <c r="P377" s="1" t="n"/>
+      <c r="R377" s="20" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="1" t="n"/>
@@ -9461,6 +9987,7 @@
       <c r="N378" s="2" t="n"/>
       <c r="O378" s="1" t="n"/>
       <c r="P378" s="1" t="n"/>
+      <c r="R378" s="20" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="1" t="n"/>
@@ -9479,6 +10006,7 @@
       <c r="N379" s="2" t="n"/>
       <c r="O379" s="1" t="n"/>
       <c r="P379" s="1" t="n"/>
+      <c r="R379" s="20" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="1" t="n"/>
@@ -9497,6 +10025,7 @@
       <c r="N380" s="2" t="n"/>
       <c r="O380" s="1" t="n"/>
       <c r="P380" s="1" t="n"/>
+      <c r="R380" s="20" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="1" t="n"/>
@@ -9515,6 +10044,7 @@
       <c r="N381" s="2" t="n"/>
       <c r="O381" s="1" t="n"/>
       <c r="P381" s="1" t="n"/>
+      <c r="R381" s="20" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="1" t="n"/>
@@ -9533,6 +10063,7 @@
       <c r="N382" s="2" t="n"/>
       <c r="O382" s="1" t="n"/>
       <c r="P382" s="1" t="n"/>
+      <c r="R382" s="20" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="1" t="n"/>
@@ -9551,6 +10082,7 @@
       <c r="N383" s="2" t="n"/>
       <c r="O383" s="1" t="n"/>
       <c r="P383" s="1" t="n"/>
+      <c r="R383" s="20" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="1" t="n"/>
@@ -9569,6 +10101,7 @@
       <c r="N384" s="2" t="n"/>
       <c r="O384" s="1" t="n"/>
       <c r="P384" s="1" t="n"/>
+      <c r="R384" s="20" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="1" t="n"/>
@@ -9587,6 +10120,7 @@
       <c r="N385" s="2" t="n"/>
       <c r="O385" s="1" t="n"/>
       <c r="P385" s="1" t="n"/>
+      <c r="R385" s="20" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="1" t="n"/>
@@ -9605,6 +10139,7 @@
       <c r="N386" s="2" t="n"/>
       <c r="O386" s="1" t="n"/>
       <c r="P386" s="1" t="n"/>
+      <c r="R386" s="20" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="1" t="n"/>
@@ -9623,6 +10158,7 @@
       <c r="N387" s="2" t="n"/>
       <c r="O387" s="1" t="n"/>
       <c r="P387" s="1" t="n"/>
+      <c r="R387" s="20" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="1" t="n"/>
@@ -9641,6 +10177,7 @@
       <c r="N388" s="2" t="n"/>
       <c r="O388" s="1" t="n"/>
       <c r="P388" s="1" t="n"/>
+      <c r="R388" s="20" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="1" t="n"/>
@@ -9659,6 +10196,7 @@
       <c r="N389" s="2" t="n"/>
       <c r="O389" s="1" t="n"/>
       <c r="P389" s="1" t="n"/>
+      <c r="R389" s="20" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="1" t="n"/>
@@ -9677,6 +10215,7 @@
       <c r="N390" s="2" t="n"/>
       <c r="O390" s="1" t="n"/>
       <c r="P390" s="1" t="n"/>
+      <c r="R390" s="20" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="1" t="n"/>
@@ -9695,6 +10234,7 @@
       <c r="N391" s="2" t="n"/>
       <c r="O391" s="1" t="n"/>
       <c r="P391" s="1" t="n"/>
+      <c r="R391" s="20" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="1" t="n"/>
@@ -9713,6 +10253,7 @@
       <c r="N392" s="2" t="n"/>
       <c r="O392" s="1" t="n"/>
       <c r="P392" s="1" t="n"/>
+      <c r="R392" s="20" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="1" t="n"/>
@@ -9731,6 +10272,7 @@
       <c r="N393" s="2" t="n"/>
       <c r="O393" s="1" t="n"/>
       <c r="P393" s="1" t="n"/>
+      <c r="R393" s="20" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="1" t="n"/>
@@ -9749,6 +10291,7 @@
       <c r="N394" s="2" t="n"/>
       <c r="O394" s="1" t="n"/>
       <c r="P394" s="1" t="n"/>
+      <c r="R394" s="20" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="1" t="n"/>
@@ -9767,6 +10310,7 @@
       <c r="N395" s="2" t="n"/>
       <c r="O395" s="1" t="n"/>
       <c r="P395" s="1" t="n"/>
+      <c r="R395" s="20" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n"/>
@@ -9785,6 +10329,7 @@
       <c r="N396" s="2" t="n"/>
       <c r="O396" s="1" t="n"/>
       <c r="P396" s="1" t="n"/>
+      <c r="R396" s="20" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n"/>
@@ -9803,6 +10348,7 @@
       <c r="N397" s="2" t="n"/>
       <c r="O397" s="1" t="n"/>
       <c r="P397" s="1" t="n"/>
+      <c r="R397" s="20" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n"/>
@@ -9821,6 +10367,7 @@
       <c r="N398" s="2" t="n"/>
       <c r="O398" s="1" t="n"/>
       <c r="P398" s="1" t="n"/>
+      <c r="R398" s="20" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n"/>
@@ -9839,6 +10386,7 @@
       <c r="N399" s="2" t="n"/>
       <c r="O399" s="1" t="n"/>
       <c r="P399" s="1" t="n"/>
+      <c r="R399" s="20" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n"/>
@@ -9857,6 +10405,7 @@
       <c r="N400" s="2" t="n"/>
       <c r="O400" s="1" t="n"/>
       <c r="P400" s="1" t="n"/>
+      <c r="R400" s="20" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n"/>
@@ -9875,6 +10424,7 @@
       <c r="N401" s="2" t="n"/>
       <c r="O401" s="1" t="n"/>
       <c r="P401" s="1" t="n"/>
+      <c r="R401" s="20" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="1" t="n"/>
@@ -9893,6 +10443,7 @@
       <c r="N402" s="2" t="n"/>
       <c r="O402" s="1" t="n"/>
       <c r="P402" s="1" t="n"/>
+      <c r="R402" s="20" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="1" t="n"/>
@@ -9911,6 +10462,7 @@
       <c r="N403" s="2" t="n"/>
       <c r="O403" s="1" t="n"/>
       <c r="P403" s="1" t="n"/>
+      <c r="R403" s="20" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="1" t="n"/>
@@ -9929,6 +10481,7 @@
       <c r="N404" s="2" t="n"/>
       <c r="O404" s="1" t="n"/>
       <c r="P404" s="1" t="n"/>
+      <c r="R404" s="20" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="1" t="n"/>
@@ -9947,6 +10500,7 @@
       <c r="N405" s="2" t="n"/>
       <c r="O405" s="1" t="n"/>
       <c r="P405" s="1" t="n"/>
+      <c r="R405" s="20" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="1" t="n"/>
@@ -9965,6 +10519,7 @@
       <c r="N406" s="2" t="n"/>
       <c r="O406" s="1" t="n"/>
       <c r="P406" s="1" t="n"/>
+      <c r="R406" s="20" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="1" t="n"/>
@@ -9983,6 +10538,7 @@
       <c r="N407" s="2" t="n"/>
       <c r="O407" s="1" t="n"/>
       <c r="P407" s="1" t="n"/>
+      <c r="R407" s="20" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="1" t="n"/>
@@ -10001,6 +10557,7 @@
       <c r="N408" s="2" t="n"/>
       <c r="O408" s="1" t="n"/>
       <c r="P408" s="1" t="n"/>
+      <c r="R408" s="20" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="1" t="n"/>
@@ -10019,6 +10576,7 @@
       <c r="N409" s="2" t="n"/>
       <c r="O409" s="1" t="n"/>
       <c r="P409" s="1" t="n"/>
+      <c r="R409" s="20" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="1" t="n"/>
@@ -10037,6 +10595,7 @@
       <c r="N410" s="2" t="n"/>
       <c r="O410" s="1" t="n"/>
       <c r="P410" s="1" t="n"/>
+      <c r="R410" s="20" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="1" t="n"/>
@@ -10055,6 +10614,7 @@
       <c r="N411" s="2" t="n"/>
       <c r="O411" s="1" t="n"/>
       <c r="P411" s="1" t="n"/>
+      <c r="R411" s="20" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="1" t="n"/>
@@ -10073,6 +10633,7 @@
       <c r="N412" s="2" t="n"/>
       <c r="O412" s="1" t="n"/>
       <c r="P412" s="1" t="n"/>
+      <c r="R412" s="20" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="1" t="n"/>
@@ -10091,6 +10652,7 @@
       <c r="N413" s="2" t="n"/>
       <c r="O413" s="1" t="n"/>
       <c r="P413" s="1" t="n"/>
+      <c r="R413" s="20" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="1" t="n"/>
@@ -10109,6 +10671,7 @@
       <c r="N414" s="2" t="n"/>
       <c r="O414" s="1" t="n"/>
       <c r="P414" s="1" t="n"/>
+      <c r="R414" s="20" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="1" t="n"/>
@@ -10127,6 +10690,7 @@
       <c r="N415" s="2" t="n"/>
       <c r="O415" s="1" t="n"/>
       <c r="P415" s="1" t="n"/>
+      <c r="R415" s="20" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="1" t="n"/>
@@ -10145,6 +10709,7 @@
       <c r="N416" s="2" t="n"/>
       <c r="O416" s="1" t="n"/>
       <c r="P416" s="1" t="n"/>
+      <c r="R416" s="20" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="1" t="n"/>
@@ -10163,6 +10728,7 @@
       <c r="N417" s="2" t="n"/>
       <c r="O417" s="1" t="n"/>
       <c r="P417" s="1" t="n"/>
+      <c r="R417" s="20" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="1" t="n"/>
@@ -10181,6 +10747,7 @@
       <c r="N418" s="2" t="n"/>
       <c r="O418" s="1" t="n"/>
       <c r="P418" s="1" t="n"/>
+      <c r="R418" s="20" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="1" t="n"/>
@@ -10199,6 +10766,7 @@
       <c r="N419" s="2" t="n"/>
       <c r="O419" s="1" t="n"/>
       <c r="P419" s="1" t="n"/>
+      <c r="R419" s="20" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="1" t="n"/>
@@ -10217,6 +10785,7 @@
       <c r="N420" s="2" t="n"/>
       <c r="O420" s="1" t="n"/>
       <c r="P420" s="1" t="n"/>
+      <c r="R420" s="20" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="1" t="n"/>
@@ -10235,6 +10804,7 @@
       <c r="N421" s="2" t="n"/>
       <c r="O421" s="1" t="n"/>
       <c r="P421" s="1" t="n"/>
+      <c r="R421" s="20" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="1" t="n"/>
@@ -10253,6 +10823,7 @@
       <c r="N422" s="2" t="n"/>
       <c r="O422" s="1" t="n"/>
       <c r="P422" s="1" t="n"/>
+      <c r="R422" s="20" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="1" t="n"/>
@@ -10271,6 +10842,7 @@
       <c r="N423" s="2" t="n"/>
       <c r="O423" s="1" t="n"/>
       <c r="P423" s="1" t="n"/>
+      <c r="R423" s="20" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="1" t="n"/>
@@ -10289,6 +10861,7 @@
       <c r="N424" s="2" t="n"/>
       <c r="O424" s="1" t="n"/>
       <c r="P424" s="1" t="n"/>
+      <c r="R424" s="20" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="1" t="n"/>
@@ -10307,6 +10880,7 @@
       <c r="N425" s="2" t="n"/>
       <c r="O425" s="1" t="n"/>
       <c r="P425" s="1" t="n"/>
+      <c r="R425" s="20" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="1" t="n"/>
@@ -10325,6 +10899,7 @@
       <c r="N426" s="2" t="n"/>
       <c r="O426" s="1" t="n"/>
       <c r="P426" s="1" t="n"/>
+      <c r="R426" s="20" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="1" t="n"/>
@@ -10343,6 +10918,7 @@
       <c r="N427" s="2" t="n"/>
       <c r="O427" s="1" t="n"/>
       <c r="P427" s="1" t="n"/>
+      <c r="R427" s="20" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="1" t="n"/>
@@ -10361,6 +10937,7 @@
       <c r="N428" s="2" t="n"/>
       <c r="O428" s="1" t="n"/>
       <c r="P428" s="1" t="n"/>
+      <c r="R428" s="20" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="1" t="n"/>
@@ -10379,6 +10956,7 @@
       <c r="N429" s="2" t="n"/>
       <c r="O429" s="1" t="n"/>
       <c r="P429" s="1" t="n"/>
+      <c r="R429" s="20" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="1" t="n"/>
@@ -10397,6 +10975,7 @@
       <c r="N430" s="2" t="n"/>
       <c r="O430" s="1" t="n"/>
       <c r="P430" s="1" t="n"/>
+      <c r="R430" s="20" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="1" t="n"/>
@@ -10415,6 +10994,7 @@
       <c r="N431" s="2" t="n"/>
       <c r="O431" s="1" t="n"/>
       <c r="P431" s="1" t="n"/>
+      <c r="R431" s="20" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="1" t="n"/>
@@ -10433,6 +11013,7 @@
       <c r="N432" s="2" t="n"/>
       <c r="O432" s="1" t="n"/>
       <c r="P432" s="1" t="n"/>
+      <c r="R432" s="20" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="1" t="n"/>
@@ -10451,6 +11032,7 @@
       <c r="N433" s="2" t="n"/>
       <c r="O433" s="1" t="n"/>
       <c r="P433" s="1" t="n"/>
+      <c r="R433" s="20" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="1" t="n"/>
@@ -10469,6 +11051,7 @@
       <c r="N434" s="2" t="n"/>
       <c r="O434" s="1" t="n"/>
       <c r="P434" s="1" t="n"/>
+      <c r="R434" s="20" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="1" t="n"/>
@@ -10487,6 +11070,7 @@
       <c r="N435" s="2" t="n"/>
       <c r="O435" s="1" t="n"/>
       <c r="P435" s="1" t="n"/>
+      <c r="R435" s="20" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="1" t="n"/>
@@ -10505,6 +11089,7 @@
       <c r="N436" s="2" t="n"/>
       <c r="O436" s="1" t="n"/>
       <c r="P436" s="1" t="n"/>
+      <c r="R436" s="20" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="1" t="n"/>
@@ -10523,6 +11108,7 @@
       <c r="N437" s="2" t="n"/>
       <c r="O437" s="1" t="n"/>
       <c r="P437" s="1" t="n"/>
+      <c r="R437" s="20" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="1" t="n"/>
@@ -10541,6 +11127,7 @@
       <c r="N438" s="2" t="n"/>
       <c r="O438" s="1" t="n"/>
       <c r="P438" s="1" t="n"/>
+      <c r="R438" s="20" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="1" t="n"/>
@@ -10559,6 +11146,7 @@
       <c r="N439" s="2" t="n"/>
       <c r="O439" s="1" t="n"/>
       <c r="P439" s="1" t="n"/>
+      <c r="R439" s="20" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="1" t="n"/>
@@ -10577,6 +11165,7 @@
       <c r="N440" s="2" t="n"/>
       <c r="O440" s="1" t="n"/>
       <c r="P440" s="1" t="n"/>
+      <c r="R440" s="20" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="1" t="n"/>
@@ -10595,6 +11184,7 @@
       <c r="N441" s="2" t="n"/>
       <c r="O441" s="1" t="n"/>
       <c r="P441" s="1" t="n"/>
+      <c r="R441" s="20" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="1" t="n"/>
@@ -10613,6 +11203,7 @@
       <c r="N442" s="2" t="n"/>
       <c r="O442" s="1" t="n"/>
       <c r="P442" s="1" t="n"/>
+      <c r="R442" s="20" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="1" t="n"/>
@@ -10631,6 +11222,7 @@
       <c r="N443" s="2" t="n"/>
       <c r="O443" s="1" t="n"/>
       <c r="P443" s="1" t="n"/>
+      <c r="R443" s="20" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="1" t="n"/>
@@ -10649,6 +11241,7 @@
       <c r="N444" s="2" t="n"/>
       <c r="O444" s="1" t="n"/>
       <c r="P444" s="1" t="n"/>
+      <c r="R444" s="20" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="1" t="n"/>
@@ -10667,6 +11260,7 @@
       <c r="N445" s="2" t="n"/>
       <c r="O445" s="1" t="n"/>
       <c r="P445" s="1" t="n"/>
+      <c r="R445" s="20" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="1" t="n"/>
@@ -10685,6 +11279,7 @@
       <c r="N446" s="2" t="n"/>
       <c r="O446" s="1" t="n"/>
       <c r="P446" s="1" t="n"/>
+      <c r="R446" s="20" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="1" t="n"/>
@@ -10703,6 +11298,7 @@
       <c r="N447" s="2" t="n"/>
       <c r="O447" s="1" t="n"/>
       <c r="P447" s="1" t="n"/>
+      <c r="R447" s="20" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="1" t="n"/>
@@ -10721,6 +11317,7 @@
       <c r="N448" s="2" t="n"/>
       <c r="O448" s="1" t="n"/>
       <c r="P448" s="1" t="n"/>
+      <c r="R448" s="20" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="1" t="n"/>
@@ -10739,6 +11336,7 @@
       <c r="N449" s="2" t="n"/>
       <c r="O449" s="1" t="n"/>
       <c r="P449" s="1" t="n"/>
+      <c r="R449" s="20" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="1" t="n"/>
@@ -10757,6 +11355,7 @@
       <c r="N450" s="2" t="n"/>
       <c r="O450" s="1" t="n"/>
       <c r="P450" s="1" t="n"/>
+      <c r="R450" s="20" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="1" t="n"/>
@@ -10775,6 +11374,7 @@
       <c r="N451" s="2" t="n"/>
       <c r="O451" s="1" t="n"/>
       <c r="P451" s="1" t="n"/>
+      <c r="R451" s="20" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="1" t="n"/>
@@ -10793,6 +11393,7 @@
       <c r="N452" s="2" t="n"/>
       <c r="O452" s="1" t="n"/>
       <c r="P452" s="1" t="n"/>
+      <c r="R452" s="20" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="1" t="n"/>
@@ -10811,6 +11412,7 @@
       <c r="N453" s="2" t="n"/>
       <c r="O453" s="1" t="n"/>
       <c r="P453" s="1" t="n"/>
+      <c r="R453" s="20" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="1" t="n"/>
@@ -10829,6 +11431,7 @@
       <c r="N454" s="2" t="n"/>
       <c r="O454" s="1" t="n"/>
       <c r="P454" s="1" t="n"/>
+      <c r="R454" s="20" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="1" t="n"/>
@@ -10847,6 +11450,7 @@
       <c r="N455" s="2" t="n"/>
       <c r="O455" s="1" t="n"/>
       <c r="P455" s="1" t="n"/>
+      <c r="R455" s="20" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="1" t="n"/>
@@ -10865,6 +11469,7 @@
       <c r="N456" s="2" t="n"/>
       <c r="O456" s="1" t="n"/>
       <c r="P456" s="1" t="n"/>
+      <c r="R456" s="20" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="1" t="n"/>
@@ -10883,6 +11488,7 @@
       <c r="N457" s="2" t="n"/>
       <c r="O457" s="1" t="n"/>
       <c r="P457" s="1" t="n"/>
+      <c r="R457" s="20" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="1" t="n"/>
@@ -10901,6 +11507,7 @@
       <c r="N458" s="2" t="n"/>
       <c r="O458" s="1" t="n"/>
       <c r="P458" s="1" t="n"/>
+      <c r="R458" s="20" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="1" t="n"/>
@@ -10919,6 +11526,7 @@
       <c r="N459" s="2" t="n"/>
       <c r="O459" s="1" t="n"/>
       <c r="P459" s="1" t="n"/>
+      <c r="R459" s="20" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="1" t="n"/>
@@ -10937,6 +11545,7 @@
       <c r="N460" s="2" t="n"/>
       <c r="O460" s="1" t="n"/>
       <c r="P460" s="1" t="n"/>
+      <c r="R460" s="20" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="1" t="n"/>
@@ -10955,6 +11564,7 @@
       <c r="N461" s="2" t="n"/>
       <c r="O461" s="1" t="n"/>
       <c r="P461" s="1" t="n"/>
+      <c r="R461" s="20" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="1" t="n"/>
@@ -10973,6 +11583,7 @@
       <c r="N462" s="2" t="n"/>
       <c r="O462" s="1" t="n"/>
       <c r="P462" s="1" t="n"/>
+      <c r="R462" s="20" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="1" t="n"/>
@@ -10991,6 +11602,7 @@
       <c r="N463" s="2" t="n"/>
       <c r="O463" s="1" t="n"/>
       <c r="P463" s="1" t="n"/>
+      <c r="R463" s="20" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="1" t="n"/>
@@ -11009,6 +11621,7 @@
       <c r="N464" s="2" t="n"/>
       <c r="O464" s="1" t="n"/>
       <c r="P464" s="1" t="n"/>
+      <c r="R464" s="20" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="1" t="n"/>
@@ -11027,6 +11640,7 @@
       <c r="N465" s="2" t="n"/>
       <c r="O465" s="1" t="n"/>
       <c r="P465" s="1" t="n"/>
+      <c r="R465" s="20" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="1" t="n"/>
@@ -11045,6 +11659,7 @@
       <c r="N466" s="2" t="n"/>
       <c r="O466" s="1" t="n"/>
       <c r="P466" s="1" t="n"/>
+      <c r="R466" s="20" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="1" t="n"/>
@@ -11063,6 +11678,7 @@
       <c r="N467" s="2" t="n"/>
       <c r="O467" s="1" t="n"/>
       <c r="P467" s="1" t="n"/>
+      <c r="R467" s="20" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="1" t="n"/>
@@ -11081,6 +11697,7 @@
       <c r="N468" s="2" t="n"/>
       <c r="O468" s="1" t="n"/>
       <c r="P468" s="1" t="n"/>
+      <c r="R468" s="20" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="1" t="n"/>
@@ -11099,6 +11716,7 @@
       <c r="N469" s="2" t="n"/>
       <c r="O469" s="1" t="n"/>
       <c r="P469" s="1" t="n"/>
+      <c r="R469" s="20" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="1" t="n"/>
@@ -11117,6 +11735,7 @@
       <c r="N470" s="2" t="n"/>
       <c r="O470" s="1" t="n"/>
       <c r="P470" s="1" t="n"/>
+      <c r="R470" s="20" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="1" t="n"/>
@@ -11135,6 +11754,7 @@
       <c r="N471" s="2" t="n"/>
       <c r="O471" s="1" t="n"/>
       <c r="P471" s="1" t="n"/>
+      <c r="R471" s="20" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="1" t="n"/>
@@ -11153,6 +11773,7 @@
       <c r="N472" s="2" t="n"/>
       <c r="O472" s="1" t="n"/>
       <c r="P472" s="1" t="n"/>
+      <c r="R472" s="20" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="1" t="n"/>
@@ -11171,6 +11792,7 @@
       <c r="N473" s="2" t="n"/>
       <c r="O473" s="1" t="n"/>
       <c r="P473" s="1" t="n"/>
+      <c r="R473" s="20" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="1" t="n"/>
@@ -11189,6 +11811,7 @@
       <c r="N474" s="2" t="n"/>
       <c r="O474" s="1" t="n"/>
       <c r="P474" s="1" t="n"/>
+      <c r="R474" s="20" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="1" t="n"/>
@@ -11207,6 +11830,7 @@
       <c r="N475" s="2" t="n"/>
       <c r="O475" s="1" t="n"/>
       <c r="P475" s="1" t="n"/>
+      <c r="R475" s="20" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="1" t="n"/>
@@ -11225,6 +11849,7 @@
       <c r="N476" s="2" t="n"/>
       <c r="O476" s="1" t="n"/>
       <c r="P476" s="1" t="n"/>
+      <c r="R476" s="20" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="1" t="n"/>
@@ -11243,6 +11868,7 @@
       <c r="N477" s="2" t="n"/>
       <c r="O477" s="1" t="n"/>
       <c r="P477" s="1" t="n"/>
+      <c r="R477" s="20" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="1" t="n"/>
@@ -11261,6 +11887,7 @@
       <c r="N478" s="2" t="n"/>
       <c r="O478" s="1" t="n"/>
       <c r="P478" s="1" t="n"/>
+      <c r="R478" s="20" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="1" t="n"/>
@@ -11279,6 +11906,7 @@
       <c r="N479" s="2" t="n"/>
       <c r="O479" s="1" t="n"/>
       <c r="P479" s="1" t="n"/>
+      <c r="R479" s="20" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="1" t="n"/>
@@ -11297,6 +11925,7 @@
       <c r="N480" s="2" t="n"/>
       <c r="O480" s="1" t="n"/>
       <c r="P480" s="1" t="n"/>
+      <c r="R480" s="20" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="1" t="n"/>
@@ -11315,6 +11944,7 @@
       <c r="N481" s="2" t="n"/>
       <c r="O481" s="1" t="n"/>
       <c r="P481" s="1" t="n"/>
+      <c r="R481" s="20" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="1" t="n"/>
@@ -11333,6 +11963,7 @@
       <c r="N482" s="2" t="n"/>
       <c r="O482" s="1" t="n"/>
       <c r="P482" s="1" t="n"/>
+      <c r="R482" s="20" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="1" t="n"/>
@@ -11351,6 +11982,7 @@
       <c r="N483" s="2" t="n"/>
       <c r="O483" s="1" t="n"/>
       <c r="P483" s="1" t="n"/>
+      <c r="R483" s="20" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="1" t="n"/>
@@ -11369,6 +12001,7 @@
       <c r="N484" s="2" t="n"/>
       <c r="O484" s="1" t="n"/>
       <c r="P484" s="1" t="n"/>
+      <c r="R484" s="20" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="1" t="n"/>
@@ -11387,6 +12020,7 @@
       <c r="N485" s="2" t="n"/>
       <c r="O485" s="1" t="n"/>
       <c r="P485" s="1" t="n"/>
+      <c r="R485" s="20" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="1" t="n"/>
@@ -11405,6 +12039,7 @@
       <c r="N486" s="2" t="n"/>
       <c r="O486" s="1" t="n"/>
       <c r="P486" s="1" t="n"/>
+      <c r="R486" s="20" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="1" t="n"/>
@@ -11423,6 +12058,7 @@
       <c r="N487" s="2" t="n"/>
       <c r="O487" s="1" t="n"/>
       <c r="P487" s="1" t="n"/>
+      <c r="R487" s="20" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="1" t="n"/>
@@ -11441,6 +12077,7 @@
       <c r="N488" s="2" t="n"/>
       <c r="O488" s="1" t="n"/>
       <c r="P488" s="1" t="n"/>
+      <c r="R488" s="20" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="1" t="n"/>
@@ -11459,6 +12096,7 @@
       <c r="N489" s="2" t="n"/>
       <c r="O489" s="1" t="n"/>
       <c r="P489" s="1" t="n"/>
+      <c r="R489" s="20" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="1" t="n"/>
@@ -11477,6 +12115,7 @@
       <c r="N490" s="2" t="n"/>
       <c r="O490" s="1" t="n"/>
       <c r="P490" s="1" t="n"/>
+      <c r="R490" s="20" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="1" t="n"/>
@@ -11495,6 +12134,7 @@
       <c r="N491" s="2" t="n"/>
       <c r="O491" s="1" t="n"/>
       <c r="P491" s="1" t="n"/>
+      <c r="R491" s="20" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="1" t="n"/>
@@ -11513,6 +12153,7 @@
       <c r="N492" s="2" t="n"/>
       <c r="O492" s="1" t="n"/>
       <c r="P492" s="1" t="n"/>
+      <c r="R492" s="20" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="1" t="n"/>
@@ -11531,6 +12172,7 @@
       <c r="N493" s="2" t="n"/>
       <c r="O493" s="1" t="n"/>
       <c r="P493" s="1" t="n"/>
+      <c r="R493" s="20" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="1" t="n"/>
@@ -11549,6 +12191,7 @@
       <c r="N494" s="2" t="n"/>
       <c r="O494" s="1" t="n"/>
       <c r="P494" s="1" t="n"/>
+      <c r="R494" s="20" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="1" t="n"/>
@@ -11567,6 +12210,7 @@
       <c r="N495" s="2" t="n"/>
       <c r="O495" s="1" t="n"/>
       <c r="P495" s="1" t="n"/>
+      <c r="R495" s="20" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="1" t="n"/>
@@ -11585,6 +12229,7 @@
       <c r="N496" s="2" t="n"/>
       <c r="O496" s="1" t="n"/>
       <c r="P496" s="1" t="n"/>
+      <c r="R496" s="20" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="1" t="n"/>
@@ -11603,6 +12248,7 @@
       <c r="N497" s="2" t="n"/>
       <c r="O497" s="1" t="n"/>
       <c r="P497" s="1" t="n"/>
+      <c r="R497" s="20" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="1" t="n"/>
@@ -11621,6 +12267,7 @@
       <c r="N498" s="2" t="n"/>
       <c r="O498" s="1" t="n"/>
       <c r="P498" s="1" t="n"/>
+      <c r="R498" s="20" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="1" t="n"/>
@@ -11639,6 +12286,7 @@
       <c r="N499" s="2" t="n"/>
       <c r="O499" s="1" t="n"/>
       <c r="P499" s="1" t="n"/>
+      <c r="R499" s="20" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="1" t="n"/>
@@ -11657,6 +12305,7 @@
       <c r="N500" s="2" t="n"/>
       <c r="O500" s="1" t="n"/>
       <c r="P500" s="1" t="n"/>
+      <c r="R500" s="20" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="1" t="n"/>
@@ -11675,9 +12324,10 @@
       <c r="N501" s="2" t="n"/>
       <c r="O501" s="1" t="n"/>
       <c r="P501" s="1" t="n"/>
+      <c r="R501" s="20" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q501"/>
+  <autoFilter ref="A1:R501"/>
   <dataValidations count="5">
     <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Projects!$A$2:$A$51</formula1>
@@ -12703,4 +13353,527 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="86" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>Price Schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Rebuilt automatically from the Selections sheet - do not edit here. Enter prices in the Unit Price column on Selections; Price = Qty x Unit Price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>S.No</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>UH-101   The Magnolia Residence</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>EXTERIOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>EX-01</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>James Hardie HardiePlank Lap – Arctic White</t>
+        </is>
+      </c>
+      <c r="D7" s="30">
+        <f>IF(Selections!H2="",1,Selections!H2)</f>
+        <v/>
+      </c>
+      <c r="E7" s="31">
+        <f>IF(Selections!R2="","",Selections!R2)</f>
+        <v/>
+      </c>
+      <c r="F7" s="31">
+        <f>IF(ISNUMBER(E7),D7*E7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="32" t="inlineStr">
+        <is>
+          <t>Exterior subtotal</t>
+        </is>
+      </c>
+      <c r="F8" s="33">
+        <f>SUM(F7:F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>WINDOWS &amp; DOORS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>EX-02</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Therma-Tru S4108 – Black</t>
+        </is>
+      </c>
+      <c r="D10" s="30">
+        <f>IF(Selections!H3="",1,Selections!H3)</f>
+        <v/>
+      </c>
+      <c r="E10" s="31">
+        <f>IF(Selections!R3="","",Selections!R3)</f>
+        <v/>
+      </c>
+      <c r="F10" s="31">
+        <f>IF(ISNUMBER(E10),D10*E10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>Windows &amp; Doors subtotal</t>
+        </is>
+      </c>
+      <c r="F11" s="33">
+        <f>SUM(F10:F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>KITCHEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>EX-03</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Moen 7594ESRS – Spot Resist Stainless</t>
+        </is>
+      </c>
+      <c r="D13" s="30">
+        <f>IF(Selections!H4="",1,Selections!H4)</f>
+        <v/>
+      </c>
+      <c r="E13" s="31">
+        <f>IF(Selections!R4="","",Selections!R4)</f>
+        <v/>
+      </c>
+      <c r="F13" s="31">
+        <f>IF(ISNUMBER(E13),D13*E13,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>Kitchen subtotal</t>
+        </is>
+      </c>
+      <c r="F14" s="33">
+        <f>SUM(F13:F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>BATHROOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>EX-04</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>Delta 559LF-PP – Chrome</t>
+        </is>
+      </c>
+      <c r="D16" s="30">
+        <f>IF(Selections!H5="",1,Selections!H5)</f>
+        <v/>
+      </c>
+      <c r="E16" s="31">
+        <f>IF(Selections!R5="","",Selections!R5)</f>
+        <v/>
+      </c>
+      <c r="F16" s="31">
+        <f>IF(ISNUMBER(E16),D16*E16,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>Bathrooms subtotal</t>
+        </is>
+      </c>
+      <c r="F17" s="33">
+        <f>SUM(F16:F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>PAINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>EX-05</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>Sherwin-Williams SW 7005 – Pure White</t>
+        </is>
+      </c>
+      <c r="D19" s="30">
+        <f>IF(Selections!H6="",1,Selections!H6)</f>
+        <v/>
+      </c>
+      <c r="E19" s="31">
+        <f>IF(Selections!R6="","",Selections!R6)</f>
+        <v/>
+      </c>
+      <c r="F19" s="31">
+        <f>IF(ISNUMBER(E19),D19*E19,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>Paint subtotal</t>
+        </is>
+      </c>
+      <c r="F20" s="33">
+        <f>SUM(F19:F19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="n"/>
+      <c r="B21" s="34" t="n"/>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>UH-101 total</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="n"/>
+      <c r="E21" s="34" t="n"/>
+      <c r="F21" s="36">
+        <f>F8+F11+F14+F17+F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>UH-102   Cedar Ridge Custom Build</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="26" t="inlineStr">
+        <is>
+          <t>KITCHEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>EX-01</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>Kohler K-5540 – White</t>
+        </is>
+      </c>
+      <c r="D25" s="30">
+        <f>IF(Selections!H7="",1,Selections!H7)</f>
+        <v/>
+      </c>
+      <c r="E25" s="31">
+        <f>IF(Selections!R7="","",Selections!R7)</f>
+        <v/>
+      </c>
+      <c r="F25" s="31">
+        <f>IF(ISNUMBER(E25),D25*E25,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>Kitchen subtotal</t>
+        </is>
+      </c>
+      <c r="F26" s="33">
+        <f>SUM(F25:F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>LIGHTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>EX-02</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>Kichler Olde Bronze – Model TBD</t>
+        </is>
+      </c>
+      <c r="D28" s="30">
+        <f>IF(Selections!H8="",1,Selections!H8)</f>
+        <v/>
+      </c>
+      <c r="E28" s="31">
+        <f>IF(Selections!R8="","",Selections!R8)</f>
+        <v/>
+      </c>
+      <c r="F28" s="31">
+        <f>IF(ISNUMBER(E28),D28*E28,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" s="32" t="inlineStr">
+        <is>
+          <t>Lighting subtotal</t>
+        </is>
+      </c>
+      <c r="F29" s="33">
+        <f>SUM(F28:F28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="34" t="n"/>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="35" t="inlineStr">
+        <is>
+          <t>UH-102 total</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="n"/>
+      <c r="E30" s="34" t="n"/>
+      <c r="F30" s="36">
+        <f>F26+F29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>UH-103   Velora</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>WINDOWS &amp; DOORS</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>EX-01</t>
+        </is>
+      </c>
+      <c r="C34" s="29" t="inlineStr">
+        <is>
+          <t>Dfw company Main Door (Model xyz) – Black – Nothing</t>
+        </is>
+      </c>
+      <c r="D34" s="30">
+        <f>IF(Selections!H9="",1,Selections!H9)</f>
+        <v/>
+      </c>
+      <c r="E34" s="31">
+        <f>IF(Selections!R9="","",Selections!R9)</f>
+        <v/>
+      </c>
+      <c r="F34" s="31">
+        <f>IF(ISNUMBER(E34),D34*E34,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="32" t="inlineStr">
+        <is>
+          <t>Windows &amp; Doors subtotal</t>
+        </is>
+      </c>
+      <c r="F35" s="33">
+        <f>SUM(F34:F34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="34" t="n"/>
+      <c r="B36" s="34" t="n"/>
+      <c r="C36" s="35" t="inlineStr">
+        <is>
+          <t>UH-103 total</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="n"/>
+      <c r="E36" s="34" t="n"/>
+      <c r="F36" s="36">
+        <f>F35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34" t="n"/>
+      <c r="B38" s="34" t="n"/>
+      <c r="C38" s="37" t="inlineStr">
+        <is>
+          <t>Grand total</t>
+        </is>
+      </c>
+      <c r="D38" s="34" t="n"/>
+      <c r="E38" s="34" t="n"/>
+      <c r="F38" s="38">
+        <f>F21+F30+F36</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Markup % to selections and the price schedule
Markup % is a numeric Selections column editable in the spec sheet
editor and inline in the spec table. The Price Schedule gains a Markup
column and its line total becomes Qty x Unit Price x (1 + Markup %),
with the subtotals, project totals and grand total following it.

Supplier and Unit were tried alongside it and reverted: reserving a
name that an existing workbook may already use for a custom field
makes that workbook unreadable, which the custom-field tests caught.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Projects'!$A$1:$L$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$R$501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Selections'!$A$1:$S$501</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Manufacturers'!$A$1:$C$101</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -24,7 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.##"/>
+  </numFmts>
   <fonts count="15">
     <font>
       <name val="Calibri"/>
@@ -190,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -292,6 +294,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="12" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -593,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="118" customWidth="1" style="4" min="1" max="1"/>
@@ -738,83 +744,87 @@
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>Unit Price       Cost per unit. The Price Schedule sheet multiplies it by Qty and totals it.</t>
+          <t>Unit             Unit of measure, for example EA, LF, SQ FT or GAL.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>Client Notes     Short note printed with the item on the client schedule.</t>
+          <t>Unit Price       Cost per unit. The Price Schedule multiplies it by Qty and adds the markup.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>Include in Lookbook   No hides the row from client exports without deleting it. Dropdown.</t>
+          <t>Markup %         Percentage added to the line, for example 15. Leave blank for none.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>Client Status    Proposed / Presented / Approved / Rejected / Changed. Dropdown.</t>
+          <t>Supplier         Who you are buying it from.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="n"/>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Client Notes     Short note printed with the item on the client schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>Price Schedule sheet</t>
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Include in Lookbook   No hides the row from client exports without deleting it. Dropdown.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>Every selection grouped by project and category with S.No, Code, Description, Qty, Unit Price and Price, plus a subtotal per category, a total per project and a grand total.</t>
+          <t>Client Status    Proposed / Presented / Approved / Rejected / Changed. Dropdown.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>It is rebuilt automatically each time the workbook is saved, so do not type into it. Enter costs in the Unit Price column on Selections and they flow through.</t>
-        </is>
-      </c>
+      <c r="A29" s="16" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>Prices stay internal: they never appear on the client PDF or PowerPoint.</t>
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Price Schedule sheet</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="n"/>
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Every selection grouped by project and category with S.No, Code, Description, Qty, Unit Price, Markup % and Price, plus a subtotal per category, a total per project and a grand total.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>Columns filled in for you</t>
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Price = Qty x Unit Price x (1 + Markup %).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Product URL, Product Name, Image URL, Lookup Status, Checked On, Lookup Notes are written by the product lookup. You may correct any of them by hand.</t>
+          <t>It is rebuilt automatically each time the workbook is saved, so do not type into it. Enter costs in the Unit Price column on Selections and they flow through.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>On the Projects sheet, Total Items, Links Found, Verified and Needs Review are formulas.</t>
+          <t>Prices stay internal: they never appear on the client PDF or PowerPoint.</t>
         </is>
       </c>
     </row>
@@ -824,47 +834,71 @@
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>Rules worth knowing</t>
+          <t>Columns filled in for you</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>- Changing Item, Product Name, Manufacturer, Model # or Finish clears the old link and verification, because they no longer describe the same product.</t>
+          <t>Product URL, Product Name, Image URL, Lookup Status, Checked On, Lookup Notes are written by the product lookup. You may correct any of them by hand.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>- A Verified link older than six months is flagged for re-checking in the web app.</t>
+          <t>On the Projects sheet, Total Items, Links Found, Verified and Needs Review are formulas.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>- Close this workbook in Excel before saving from the web app; the app will not write to a file Excel has open.</t>
-        </is>
-      </c>
+      <c r="A39" s="16" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>- Every save keeps a timestamped copy in the backups folder.</t>
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Rules worth knowing</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>- Product URLs and images are internal review aids and never appear on client documents.</t>
+          <t>- Changing Item, Product Name, Manufacturer, Model # or Finish clears the old link and verification, because they no longer describe the same product.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>- A Verified link older than six months is flagged for re-checking in the web app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>- Close this workbook in Excel before saving from the web app; the app will not write to a file Excel has open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>- Every save keeps a timestamped copy in the backups folder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>- Product URLs and images are internal review aids and never appear on client documents.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <t>- Section order on the Lists sheet controls the order of categories in the client schedule.</t>
         </is>
@@ -2355,7 +2389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R501"/>
+  <dimension ref="A1:S501"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2374,6 +2408,9 @@
     <col width="17" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2465,6 +2502,11 @@
       <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Markup %</t>
         </is>
       </c>
     </row>
@@ -2527,6 +2569,7 @@
         </is>
       </c>
       <c r="R2" s="20" t="n"/>
+      <c r="S2" s="39" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -2589,6 +2632,7 @@
         </is>
       </c>
       <c r="R3" s="20" t="n"/>
+      <c r="S3" s="39" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
@@ -2651,6 +2695,7 @@
         </is>
       </c>
       <c r="R4" s="20" t="n"/>
+      <c r="S4" s="39" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -2713,6 +2758,7 @@
         </is>
       </c>
       <c r="R5" s="20" t="n"/>
+      <c r="S5" s="39" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2773,6 +2819,7 @@
         </is>
       </c>
       <c r="R6" s="20" t="n"/>
+      <c r="S6" s="39" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2835,6 +2882,7 @@
         </is>
       </c>
       <c r="R7" s="20" t="n"/>
+      <c r="S7" s="39" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -2897,6 +2945,7 @@
         </is>
       </c>
       <c r="R8" s="20" t="n"/>
+      <c r="S8" s="39" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -2977,6 +3026,7 @@
         </is>
       </c>
       <c r="R9" s="20" t="n"/>
+      <c r="S9" s="39" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n"/>
@@ -2996,6 +3046,7 @@
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="n"/>
       <c r="R10" s="20" t="n"/>
+      <c r="S10" s="39" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n"/>
@@ -3015,6 +3066,7 @@
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="n"/>
       <c r="R11" s="20" t="n"/>
+      <c r="S11" s="39" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n"/>
@@ -3034,6 +3086,7 @@
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="n"/>
       <c r="R12" s="20" t="n"/>
+      <c r="S12" s="39" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
@@ -3053,6 +3106,7 @@
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="n"/>
       <c r="R13" s="20" t="n"/>
+      <c r="S13" s="39" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n"/>
@@ -3072,6 +3126,7 @@
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="n"/>
       <c r="R14" s="20" t="n"/>
+      <c r="S14" s="39" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
@@ -3091,6 +3146,7 @@
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="n"/>
       <c r="R15" s="20" t="n"/>
+      <c r="S15" s="39" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n"/>
@@ -3110,6 +3166,7 @@
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="n"/>
       <c r="R16" s="20" t="n"/>
+      <c r="S16" s="39" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
@@ -3129,6 +3186,7 @@
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="n"/>
       <c r="R17" s="20" t="n"/>
+      <c r="S17" s="39" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n"/>
@@ -3148,6 +3206,7 @@
       <c r="O18" s="1" t="n"/>
       <c r="P18" s="1" t="n"/>
       <c r="R18" s="20" t="n"/>
+      <c r="S18" s="39" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n"/>
@@ -3167,6 +3226,7 @@
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="n"/>
       <c r="R19" s="20" t="n"/>
+      <c r="S19" s="39" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
@@ -3186,6 +3246,7 @@
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="n"/>
       <c r="R20" s="20" t="n"/>
+      <c r="S20" s="39" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n"/>
@@ -3205,6 +3266,7 @@
       <c r="O21" s="1" t="n"/>
       <c r="P21" s="1" t="n"/>
       <c r="R21" s="20" t="n"/>
+      <c r="S21" s="39" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n"/>
@@ -3224,6 +3286,7 @@
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="n"/>
       <c r="R22" s="20" t="n"/>
+      <c r="S22" s="39" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
@@ -3243,6 +3306,7 @@
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="n"/>
       <c r="R23" s="20" t="n"/>
+      <c r="S23" s="39" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n"/>
@@ -3262,6 +3326,7 @@
       <c r="O24" s="1" t="n"/>
       <c r="P24" s="1" t="n"/>
       <c r="R24" s="20" t="n"/>
+      <c r="S24" s="39" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n"/>
@@ -3281,6 +3346,7 @@
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="n"/>
       <c r="R25" s="20" t="n"/>
+      <c r="S25" s="39" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
@@ -3300,6 +3366,7 @@
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="n"/>
       <c r="R26" s="20" t="n"/>
+      <c r="S26" s="39" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n"/>
@@ -3319,6 +3386,7 @@
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="n"/>
       <c r="R27" s="20" t="n"/>
+      <c r="S27" s="39" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n"/>
@@ -3338,6 +3406,7 @@
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="n"/>
       <c r="R28" s="20" t="n"/>
+      <c r="S28" s="39" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n"/>
@@ -3357,6 +3426,7 @@
       <c r="O29" s="1" t="n"/>
       <c r="P29" s="1" t="n"/>
       <c r="R29" s="20" t="n"/>
+      <c r="S29" s="39" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
@@ -3376,6 +3446,7 @@
       <c r="O30" s="1" t="n"/>
       <c r="P30" s="1" t="n"/>
       <c r="R30" s="20" t="n"/>
+      <c r="S30" s="39" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
@@ -3395,6 +3466,7 @@
       <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="n"/>
       <c r="R31" s="20" t="n"/>
+      <c r="S31" s="39" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n"/>
@@ -3414,6 +3486,7 @@
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="n"/>
       <c r="R32" s="20" t="n"/>
+      <c r="S32" s="39" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n"/>
@@ -3433,6 +3506,7 @@
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="n"/>
       <c r="R33" s="20" t="n"/>
+      <c r="S33" s="39" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n"/>
@@ -3452,6 +3526,7 @@
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="n"/>
       <c r="R34" s="20" t="n"/>
+      <c r="S34" s="39" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n"/>
@@ -3471,6 +3546,7 @@
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="n"/>
       <c r="R35" s="20" t="n"/>
+      <c r="S35" s="39" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n"/>
@@ -3490,6 +3566,7 @@
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="n"/>
       <c r="R36" s="20" t="n"/>
+      <c r="S36" s="39" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n"/>
@@ -3509,6 +3586,7 @@
       <c r="O37" s="1" t="n"/>
       <c r="P37" s="1" t="n"/>
       <c r="R37" s="20" t="n"/>
+      <c r="S37" s="39" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n"/>
@@ -3528,6 +3606,7 @@
       <c r="O38" s="1" t="n"/>
       <c r="P38" s="1" t="n"/>
       <c r="R38" s="20" t="n"/>
+      <c r="S38" s="39" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n"/>
@@ -3547,6 +3626,7 @@
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="n"/>
       <c r="R39" s="20" t="n"/>
+      <c r="S39" s="39" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n"/>
@@ -3566,6 +3646,7 @@
       <c r="O40" s="1" t="n"/>
       <c r="P40" s="1" t="n"/>
       <c r="R40" s="20" t="n"/>
+      <c r="S40" s="39" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n"/>
@@ -3585,6 +3666,7 @@
       <c r="O41" s="1" t="n"/>
       <c r="P41" s="1" t="n"/>
       <c r="R41" s="20" t="n"/>
+      <c r="S41" s="39" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n"/>
@@ -3604,6 +3686,7 @@
       <c r="O42" s="1" t="n"/>
       <c r="P42" s="1" t="n"/>
       <c r="R42" s="20" t="n"/>
+      <c r="S42" s="39" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n"/>
@@ -3623,6 +3706,7 @@
       <c r="O43" s="1" t="n"/>
       <c r="P43" s="1" t="n"/>
       <c r="R43" s="20" t="n"/>
+      <c r="S43" s="39" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n"/>
@@ -3642,6 +3726,7 @@
       <c r="O44" s="1" t="n"/>
       <c r="P44" s="1" t="n"/>
       <c r="R44" s="20" t="n"/>
+      <c r="S44" s="39" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n"/>
@@ -3661,6 +3746,7 @@
       <c r="O45" s="1" t="n"/>
       <c r="P45" s="1" t="n"/>
       <c r="R45" s="20" t="n"/>
+      <c r="S45" s="39" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n"/>
@@ -3680,6 +3766,7 @@
       <c r="O46" s="1" t="n"/>
       <c r="P46" s="1" t="n"/>
       <c r="R46" s="20" t="n"/>
+      <c r="S46" s="39" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n"/>
@@ -3699,6 +3786,7 @@
       <c r="O47" s="1" t="n"/>
       <c r="P47" s="1" t="n"/>
       <c r="R47" s="20" t="n"/>
+      <c r="S47" s="39" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n"/>
@@ -3718,6 +3806,7 @@
       <c r="O48" s="1" t="n"/>
       <c r="P48" s="1" t="n"/>
       <c r="R48" s="20" t="n"/>
+      <c r="S48" s="39" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n"/>
@@ -3737,6 +3826,7 @@
       <c r="O49" s="1" t="n"/>
       <c r="P49" s="1" t="n"/>
       <c r="R49" s="20" t="n"/>
+      <c r="S49" s="39" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n"/>
@@ -3756,6 +3846,7 @@
       <c r="O50" s="1" t="n"/>
       <c r="P50" s="1" t="n"/>
       <c r="R50" s="20" t="n"/>
+      <c r="S50" s="39" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n"/>
@@ -3775,6 +3866,7 @@
       <c r="O51" s="1" t="n"/>
       <c r="P51" s="1" t="n"/>
       <c r="R51" s="20" t="n"/>
+      <c r="S51" s="39" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n"/>
@@ -3794,6 +3886,7 @@
       <c r="O52" s="1" t="n"/>
       <c r="P52" s="1" t="n"/>
       <c r="R52" s="20" t="n"/>
+      <c r="S52" s="39" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n"/>
@@ -3813,6 +3906,7 @@
       <c r="O53" s="1" t="n"/>
       <c r="P53" s="1" t="n"/>
       <c r="R53" s="20" t="n"/>
+      <c r="S53" s="39" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n"/>
@@ -3832,6 +3926,7 @@
       <c r="O54" s="1" t="n"/>
       <c r="P54" s="1" t="n"/>
       <c r="R54" s="20" t="n"/>
+      <c r="S54" s="39" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n"/>
@@ -3851,6 +3946,7 @@
       <c r="O55" s="1" t="n"/>
       <c r="P55" s="1" t="n"/>
       <c r="R55" s="20" t="n"/>
+      <c r="S55" s="39" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n"/>
@@ -3870,6 +3966,7 @@
       <c r="O56" s="1" t="n"/>
       <c r="P56" s="1" t="n"/>
       <c r="R56" s="20" t="n"/>
+      <c r="S56" s="39" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n"/>
@@ -3889,6 +3986,7 @@
       <c r="O57" s="1" t="n"/>
       <c r="P57" s="1" t="n"/>
       <c r="R57" s="20" t="n"/>
+      <c r="S57" s="39" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n"/>
@@ -3908,6 +4006,7 @@
       <c r="O58" s="1" t="n"/>
       <c r="P58" s="1" t="n"/>
       <c r="R58" s="20" t="n"/>
+      <c r="S58" s="39" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n"/>
@@ -3927,6 +4026,7 @@
       <c r="O59" s="1" t="n"/>
       <c r="P59" s="1" t="n"/>
       <c r="R59" s="20" t="n"/>
+      <c r="S59" s="39" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n"/>
@@ -3946,6 +4046,7 @@
       <c r="O60" s="1" t="n"/>
       <c r="P60" s="1" t="n"/>
       <c r="R60" s="20" t="n"/>
+      <c r="S60" s="39" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n"/>
@@ -3965,6 +4066,7 @@
       <c r="O61" s="1" t="n"/>
       <c r="P61" s="1" t="n"/>
       <c r="R61" s="20" t="n"/>
+      <c r="S61" s="39" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n"/>
@@ -3984,6 +4086,7 @@
       <c r="O62" s="1" t="n"/>
       <c r="P62" s="1" t="n"/>
       <c r="R62" s="20" t="n"/>
+      <c r="S62" s="39" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n"/>
@@ -4003,6 +4106,7 @@
       <c r="O63" s="1" t="n"/>
       <c r="P63" s="1" t="n"/>
       <c r="R63" s="20" t="n"/>
+      <c r="S63" s="39" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n"/>
@@ -4022,6 +4126,7 @@
       <c r="O64" s="1" t="n"/>
       <c r="P64" s="1" t="n"/>
       <c r="R64" s="20" t="n"/>
+      <c r="S64" s="39" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n"/>
@@ -4041,6 +4146,7 @@
       <c r="O65" s="1" t="n"/>
       <c r="P65" s="1" t="n"/>
       <c r="R65" s="20" t="n"/>
+      <c r="S65" s="39" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n"/>
@@ -4060,6 +4166,7 @@
       <c r="O66" s="1" t="n"/>
       <c r="P66" s="1" t="n"/>
       <c r="R66" s="20" t="n"/>
+      <c r="S66" s="39" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n"/>
@@ -4079,6 +4186,7 @@
       <c r="O67" s="1" t="n"/>
       <c r="P67" s="1" t="n"/>
       <c r="R67" s="20" t="n"/>
+      <c r="S67" s="39" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n"/>
@@ -4098,6 +4206,7 @@
       <c r="O68" s="1" t="n"/>
       <c r="P68" s="1" t="n"/>
       <c r="R68" s="20" t="n"/>
+      <c r="S68" s="39" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n"/>
@@ -4117,6 +4226,7 @@
       <c r="O69" s="1" t="n"/>
       <c r="P69" s="1" t="n"/>
       <c r="R69" s="20" t="n"/>
+      <c r="S69" s="39" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n"/>
@@ -4136,6 +4246,7 @@
       <c r="O70" s="1" t="n"/>
       <c r="P70" s="1" t="n"/>
       <c r="R70" s="20" t="n"/>
+      <c r="S70" s="39" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n"/>
@@ -4155,6 +4266,7 @@
       <c r="O71" s="1" t="n"/>
       <c r="P71" s="1" t="n"/>
       <c r="R71" s="20" t="n"/>
+      <c r="S71" s="39" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n"/>
@@ -4174,6 +4286,7 @@
       <c r="O72" s="1" t="n"/>
       <c r="P72" s="1" t="n"/>
       <c r="R72" s="20" t="n"/>
+      <c r="S72" s="39" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n"/>
@@ -4193,6 +4306,7 @@
       <c r="O73" s="1" t="n"/>
       <c r="P73" s="1" t="n"/>
       <c r="R73" s="20" t="n"/>
+      <c r="S73" s="39" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n"/>
@@ -4212,6 +4326,7 @@
       <c r="O74" s="1" t="n"/>
       <c r="P74" s="1" t="n"/>
       <c r="R74" s="20" t="n"/>
+      <c r="S74" s="39" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n"/>
@@ -4231,6 +4346,7 @@
       <c r="O75" s="1" t="n"/>
       <c r="P75" s="1" t="n"/>
       <c r="R75" s="20" t="n"/>
+      <c r="S75" s="39" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n"/>
@@ -4250,6 +4366,7 @@
       <c r="O76" s="1" t="n"/>
       <c r="P76" s="1" t="n"/>
       <c r="R76" s="20" t="n"/>
+      <c r="S76" s="39" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n"/>
@@ -4269,6 +4386,7 @@
       <c r="O77" s="1" t="n"/>
       <c r="P77" s="1" t="n"/>
       <c r="R77" s="20" t="n"/>
+      <c r="S77" s="39" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n"/>
@@ -4288,6 +4406,7 @@
       <c r="O78" s="1" t="n"/>
       <c r="P78" s="1" t="n"/>
       <c r="R78" s="20" t="n"/>
+      <c r="S78" s="39" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n"/>
@@ -4307,6 +4426,7 @@
       <c r="O79" s="1" t="n"/>
       <c r="P79" s="1" t="n"/>
       <c r="R79" s="20" t="n"/>
+      <c r="S79" s="39" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n"/>
@@ -4326,6 +4446,7 @@
       <c r="O80" s="1" t="n"/>
       <c r="P80" s="1" t="n"/>
       <c r="R80" s="20" t="n"/>
+      <c r="S80" s="39" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n"/>
@@ -4345,6 +4466,7 @@
       <c r="O81" s="1" t="n"/>
       <c r="P81" s="1" t="n"/>
       <c r="R81" s="20" t="n"/>
+      <c r="S81" s="39" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n"/>
@@ -4364,6 +4486,7 @@
       <c r="O82" s="1" t="n"/>
       <c r="P82" s="1" t="n"/>
       <c r="R82" s="20" t="n"/>
+      <c r="S82" s="39" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n"/>
@@ -4383,6 +4506,7 @@
       <c r="O83" s="1" t="n"/>
       <c r="P83" s="1" t="n"/>
       <c r="R83" s="20" t="n"/>
+      <c r="S83" s="39" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n"/>
@@ -4402,6 +4526,7 @@
       <c r="O84" s="1" t="n"/>
       <c r="P84" s="1" t="n"/>
       <c r="R84" s="20" t="n"/>
+      <c r="S84" s="39" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n"/>
@@ -4421,6 +4546,7 @@
       <c r="O85" s="1" t="n"/>
       <c r="P85" s="1" t="n"/>
       <c r="R85" s="20" t="n"/>
+      <c r="S85" s="39" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n"/>
@@ -4440,6 +4566,7 @@
       <c r="O86" s="1" t="n"/>
       <c r="P86" s="1" t="n"/>
       <c r="R86" s="20" t="n"/>
+      <c r="S86" s="39" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n"/>
@@ -4459,6 +4586,7 @@
       <c r="O87" s="1" t="n"/>
       <c r="P87" s="1" t="n"/>
       <c r="R87" s="20" t="n"/>
+      <c r="S87" s="39" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n"/>
@@ -4478,6 +4606,7 @@
       <c r="O88" s="1" t="n"/>
       <c r="P88" s="1" t="n"/>
       <c r="R88" s="20" t="n"/>
+      <c r="S88" s="39" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n"/>
@@ -4497,6 +4626,7 @@
       <c r="O89" s="1" t="n"/>
       <c r="P89" s="1" t="n"/>
       <c r="R89" s="20" t="n"/>
+      <c r="S89" s="39" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n"/>
@@ -4516,6 +4646,7 @@
       <c r="O90" s="1" t="n"/>
       <c r="P90" s="1" t="n"/>
       <c r="R90" s="20" t="n"/>
+      <c r="S90" s="39" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n"/>
@@ -4535,6 +4666,7 @@
       <c r="O91" s="1" t="n"/>
       <c r="P91" s="1" t="n"/>
       <c r="R91" s="20" t="n"/>
+      <c r="S91" s="39" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n"/>
@@ -4554,6 +4686,7 @@
       <c r="O92" s="1" t="n"/>
       <c r="P92" s="1" t="n"/>
       <c r="R92" s="20" t="n"/>
+      <c r="S92" s="39" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n"/>
@@ -4573,6 +4706,7 @@
       <c r="O93" s="1" t="n"/>
       <c r="P93" s="1" t="n"/>
       <c r="R93" s="20" t="n"/>
+      <c r="S93" s="39" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n"/>
@@ -4592,6 +4726,7 @@
       <c r="O94" s="1" t="n"/>
       <c r="P94" s="1" t="n"/>
       <c r="R94" s="20" t="n"/>
+      <c r="S94" s="39" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n"/>
@@ -4611,6 +4746,7 @@
       <c r="O95" s="1" t="n"/>
       <c r="P95" s="1" t="n"/>
       <c r="R95" s="20" t="n"/>
+      <c r="S95" s="39" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n"/>
@@ -4630,6 +4766,7 @@
       <c r="O96" s="1" t="n"/>
       <c r="P96" s="1" t="n"/>
       <c r="R96" s="20" t="n"/>
+      <c r="S96" s="39" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n"/>
@@ -4649,6 +4786,7 @@
       <c r="O97" s="1" t="n"/>
       <c r="P97" s="1" t="n"/>
       <c r="R97" s="20" t="n"/>
+      <c r="S97" s="39" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n"/>
@@ -4668,6 +4806,7 @@
       <c r="O98" s="1" t="n"/>
       <c r="P98" s="1" t="n"/>
       <c r="R98" s="20" t="n"/>
+      <c r="S98" s="39" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n"/>
@@ -4687,6 +4826,7 @@
       <c r="O99" s="1" t="n"/>
       <c r="P99" s="1" t="n"/>
       <c r="R99" s="20" t="n"/>
+      <c r="S99" s="39" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n"/>
@@ -4706,6 +4846,7 @@
       <c r="O100" s="1" t="n"/>
       <c r="P100" s="1" t="n"/>
       <c r="R100" s="20" t="n"/>
+      <c r="S100" s="39" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n"/>
@@ -4725,6 +4866,7 @@
       <c r="O101" s="1" t="n"/>
       <c r="P101" s="1" t="n"/>
       <c r="R101" s="20" t="n"/>
+      <c r="S101" s="39" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n"/>
@@ -4744,6 +4886,7 @@
       <c r="O102" s="1" t="n"/>
       <c r="P102" s="1" t="n"/>
       <c r="R102" s="20" t="n"/>
+      <c r="S102" s="39" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n"/>
@@ -4763,6 +4906,7 @@
       <c r="O103" s="1" t="n"/>
       <c r="P103" s="1" t="n"/>
       <c r="R103" s="20" t="n"/>
+      <c r="S103" s="39" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n"/>
@@ -4782,6 +4926,7 @@
       <c r="O104" s="1" t="n"/>
       <c r="P104" s="1" t="n"/>
       <c r="R104" s="20" t="n"/>
+      <c r="S104" s="39" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n"/>
@@ -4801,6 +4946,7 @@
       <c r="O105" s="1" t="n"/>
       <c r="P105" s="1" t="n"/>
       <c r="R105" s="20" t="n"/>
+      <c r="S105" s="39" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n"/>
@@ -4820,6 +4966,7 @@
       <c r="O106" s="1" t="n"/>
       <c r="P106" s="1" t="n"/>
       <c r="R106" s="20" t="n"/>
+      <c r="S106" s="39" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n"/>
@@ -4839,6 +4986,7 @@
       <c r="O107" s="1" t="n"/>
       <c r="P107" s="1" t="n"/>
       <c r="R107" s="20" t="n"/>
+      <c r="S107" s="39" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n"/>
@@ -4858,6 +5006,7 @@
       <c r="O108" s="1" t="n"/>
       <c r="P108" s="1" t="n"/>
       <c r="R108" s="20" t="n"/>
+      <c r="S108" s="39" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n"/>
@@ -4877,6 +5026,7 @@
       <c r="O109" s="1" t="n"/>
       <c r="P109" s="1" t="n"/>
       <c r="R109" s="20" t="n"/>
+      <c r="S109" s="39" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n"/>
@@ -4896,6 +5046,7 @@
       <c r="O110" s="1" t="n"/>
       <c r="P110" s="1" t="n"/>
       <c r="R110" s="20" t="n"/>
+      <c r="S110" s="39" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n"/>
@@ -4915,6 +5066,7 @@
       <c r="O111" s="1" t="n"/>
       <c r="P111" s="1" t="n"/>
       <c r="R111" s="20" t="n"/>
+      <c r="S111" s="39" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n"/>
@@ -4934,6 +5086,7 @@
       <c r="O112" s="1" t="n"/>
       <c r="P112" s="1" t="n"/>
       <c r="R112" s="20" t="n"/>
+      <c r="S112" s="39" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n"/>
@@ -4953,6 +5106,7 @@
       <c r="O113" s="1" t="n"/>
       <c r="P113" s="1" t="n"/>
       <c r="R113" s="20" t="n"/>
+      <c r="S113" s="39" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n"/>
@@ -4972,6 +5126,7 @@
       <c r="O114" s="1" t="n"/>
       <c r="P114" s="1" t="n"/>
       <c r="R114" s="20" t="n"/>
+      <c r="S114" s="39" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n"/>
@@ -4991,6 +5146,7 @@
       <c r="O115" s="1" t="n"/>
       <c r="P115" s="1" t="n"/>
       <c r="R115" s="20" t="n"/>
+      <c r="S115" s="39" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n"/>
@@ -5010,6 +5166,7 @@
       <c r="O116" s="1" t="n"/>
       <c r="P116" s="1" t="n"/>
       <c r="R116" s="20" t="n"/>
+      <c r="S116" s="39" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n"/>
@@ -5029,6 +5186,7 @@
       <c r="O117" s="1" t="n"/>
       <c r="P117" s="1" t="n"/>
       <c r="R117" s="20" t="n"/>
+      <c r="S117" s="39" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n"/>
@@ -5048,6 +5206,7 @@
       <c r="O118" s="1" t="n"/>
       <c r="P118" s="1" t="n"/>
       <c r="R118" s="20" t="n"/>
+      <c r="S118" s="39" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n"/>
@@ -5067,6 +5226,7 @@
       <c r="O119" s="1" t="n"/>
       <c r="P119" s="1" t="n"/>
       <c r="R119" s="20" t="n"/>
+      <c r="S119" s="39" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n"/>
@@ -5086,6 +5246,7 @@
       <c r="O120" s="1" t="n"/>
       <c r="P120" s="1" t="n"/>
       <c r="R120" s="20" t="n"/>
+      <c r="S120" s="39" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n"/>
@@ -5105,6 +5266,7 @@
       <c r="O121" s="1" t="n"/>
       <c r="P121" s="1" t="n"/>
       <c r="R121" s="20" t="n"/>
+      <c r="S121" s="39" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n"/>
@@ -5124,6 +5286,7 @@
       <c r="O122" s="1" t="n"/>
       <c r="P122" s="1" t="n"/>
       <c r="R122" s="20" t="n"/>
+      <c r="S122" s="39" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n"/>
@@ -5143,6 +5306,7 @@
       <c r="O123" s="1" t="n"/>
       <c r="P123" s="1" t="n"/>
       <c r="R123" s="20" t="n"/>
+      <c r="S123" s="39" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n"/>
@@ -5162,6 +5326,7 @@
       <c r="O124" s="1" t="n"/>
       <c r="P124" s="1" t="n"/>
       <c r="R124" s="20" t="n"/>
+      <c r="S124" s="39" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n"/>
@@ -5181,6 +5346,7 @@
       <c r="O125" s="1" t="n"/>
       <c r="P125" s="1" t="n"/>
       <c r="R125" s="20" t="n"/>
+      <c r="S125" s="39" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n"/>
@@ -5200,6 +5366,7 @@
       <c r="O126" s="1" t="n"/>
       <c r="P126" s="1" t="n"/>
       <c r="R126" s="20" t="n"/>
+      <c r="S126" s="39" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n"/>
@@ -5219,6 +5386,7 @@
       <c r="O127" s="1" t="n"/>
       <c r="P127" s="1" t="n"/>
       <c r="R127" s="20" t="n"/>
+      <c r="S127" s="39" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n"/>
@@ -5238,6 +5406,7 @@
       <c r="O128" s="1" t="n"/>
       <c r="P128" s="1" t="n"/>
       <c r="R128" s="20" t="n"/>
+      <c r="S128" s="39" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n"/>
@@ -5257,6 +5426,7 @@
       <c r="O129" s="1" t="n"/>
       <c r="P129" s="1" t="n"/>
       <c r="R129" s="20" t="n"/>
+      <c r="S129" s="39" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n"/>
@@ -5276,6 +5446,7 @@
       <c r="O130" s="1" t="n"/>
       <c r="P130" s="1" t="n"/>
       <c r="R130" s="20" t="n"/>
+      <c r="S130" s="39" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n"/>
@@ -5295,6 +5466,7 @@
       <c r="O131" s="1" t="n"/>
       <c r="P131" s="1" t="n"/>
       <c r="R131" s="20" t="n"/>
+      <c r="S131" s="39" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n"/>
@@ -5314,6 +5486,7 @@
       <c r="O132" s="1" t="n"/>
       <c r="P132" s="1" t="n"/>
       <c r="R132" s="20" t="n"/>
+      <c r="S132" s="39" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n"/>
@@ -5333,6 +5506,7 @@
       <c r="O133" s="1" t="n"/>
       <c r="P133" s="1" t="n"/>
       <c r="R133" s="20" t="n"/>
+      <c r="S133" s="39" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n"/>
@@ -5352,6 +5526,7 @@
       <c r="O134" s="1" t="n"/>
       <c r="P134" s="1" t="n"/>
       <c r="R134" s="20" t="n"/>
+      <c r="S134" s="39" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n"/>
@@ -5371,6 +5546,7 @@
       <c r="O135" s="1" t="n"/>
       <c r="P135" s="1" t="n"/>
       <c r="R135" s="20" t="n"/>
+      <c r="S135" s="39" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n"/>
@@ -5390,6 +5566,7 @@
       <c r="O136" s="1" t="n"/>
       <c r="P136" s="1" t="n"/>
       <c r="R136" s="20" t="n"/>
+      <c r="S136" s="39" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n"/>
@@ -5409,6 +5586,7 @@
       <c r="O137" s="1" t="n"/>
       <c r="P137" s="1" t="n"/>
       <c r="R137" s="20" t="n"/>
+      <c r="S137" s="39" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n"/>
@@ -5428,6 +5606,7 @@
       <c r="O138" s="1" t="n"/>
       <c r="P138" s="1" t="n"/>
       <c r="R138" s="20" t="n"/>
+      <c r="S138" s="39" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n"/>
@@ -5447,6 +5626,7 @@
       <c r="O139" s="1" t="n"/>
       <c r="P139" s="1" t="n"/>
       <c r="R139" s="20" t="n"/>
+      <c r="S139" s="39" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n"/>
@@ -5466,6 +5646,7 @@
       <c r="O140" s="1" t="n"/>
       <c r="P140" s="1" t="n"/>
       <c r="R140" s="20" t="n"/>
+      <c r="S140" s="39" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n"/>
@@ -5485,6 +5666,7 @@
       <c r="O141" s="1" t="n"/>
       <c r="P141" s="1" t="n"/>
       <c r="R141" s="20" t="n"/>
+      <c r="S141" s="39" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n"/>
@@ -5504,6 +5686,7 @@
       <c r="O142" s="1" t="n"/>
       <c r="P142" s="1" t="n"/>
       <c r="R142" s="20" t="n"/>
+      <c r="S142" s="39" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n"/>
@@ -5523,6 +5706,7 @@
       <c r="O143" s="1" t="n"/>
       <c r="P143" s="1" t="n"/>
       <c r="R143" s="20" t="n"/>
+      <c r="S143" s="39" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n"/>
@@ -5542,6 +5726,7 @@
       <c r="O144" s="1" t="n"/>
       <c r="P144" s="1" t="n"/>
       <c r="R144" s="20" t="n"/>
+      <c r="S144" s="39" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n"/>
@@ -5561,6 +5746,7 @@
       <c r="O145" s="1" t="n"/>
       <c r="P145" s="1" t="n"/>
       <c r="R145" s="20" t="n"/>
+      <c r="S145" s="39" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="1" t="n"/>
@@ -5580,6 +5766,7 @@
       <c r="O146" s="1" t="n"/>
       <c r="P146" s="1" t="n"/>
       <c r="R146" s="20" t="n"/>
+      <c r="S146" s="39" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="1" t="n"/>
@@ -5599,6 +5786,7 @@
       <c r="O147" s="1" t="n"/>
       <c r="P147" s="1" t="n"/>
       <c r="R147" s="20" t="n"/>
+      <c r="S147" s="39" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="1" t="n"/>
@@ -5618,6 +5806,7 @@
       <c r="O148" s="1" t="n"/>
       <c r="P148" s="1" t="n"/>
       <c r="R148" s="20" t="n"/>
+      <c r="S148" s="39" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="1" t="n"/>
@@ -5637,6 +5826,7 @@
       <c r="O149" s="1" t="n"/>
       <c r="P149" s="1" t="n"/>
       <c r="R149" s="20" t="n"/>
+      <c r="S149" s="39" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="1" t="n"/>
@@ -5656,6 +5846,7 @@
       <c r="O150" s="1" t="n"/>
       <c r="P150" s="1" t="n"/>
       <c r="R150" s="20" t="n"/>
+      <c r="S150" s="39" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="1" t="n"/>
@@ -5675,6 +5866,7 @@
       <c r="O151" s="1" t="n"/>
       <c r="P151" s="1" t="n"/>
       <c r="R151" s="20" t="n"/>
+      <c r="S151" s="39" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="1" t="n"/>
@@ -5694,6 +5886,7 @@
       <c r="O152" s="1" t="n"/>
       <c r="P152" s="1" t="n"/>
       <c r="R152" s="20" t="n"/>
+      <c r="S152" s="39" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="1" t="n"/>
@@ -5713,6 +5906,7 @@
       <c r="O153" s="1" t="n"/>
       <c r="P153" s="1" t="n"/>
       <c r="R153" s="20" t="n"/>
+      <c r="S153" s="39" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="1" t="n"/>
@@ -5732,6 +5926,7 @@
       <c r="O154" s="1" t="n"/>
       <c r="P154" s="1" t="n"/>
       <c r="R154" s="20" t="n"/>
+      <c r="S154" s="39" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="1" t="n"/>
@@ -5751,6 +5946,7 @@
       <c r="O155" s="1" t="n"/>
       <c r="P155" s="1" t="n"/>
       <c r="R155" s="20" t="n"/>
+      <c r="S155" s="39" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="1" t="n"/>
@@ -5770,6 +5966,7 @@
       <c r="O156" s="1" t="n"/>
       <c r="P156" s="1" t="n"/>
       <c r="R156" s="20" t="n"/>
+      <c r="S156" s="39" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="1" t="n"/>
@@ -5789,6 +5986,7 @@
       <c r="O157" s="1" t="n"/>
       <c r="P157" s="1" t="n"/>
       <c r="R157" s="20" t="n"/>
+      <c r="S157" s="39" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="1" t="n"/>
@@ -5808,6 +6006,7 @@
       <c r="O158" s="1" t="n"/>
       <c r="P158" s="1" t="n"/>
       <c r="R158" s="20" t="n"/>
+      <c r="S158" s="39" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="1" t="n"/>
@@ -5827,6 +6026,7 @@
       <c r="O159" s="1" t="n"/>
       <c r="P159" s="1" t="n"/>
       <c r="R159" s="20" t="n"/>
+      <c r="S159" s="39" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="1" t="n"/>
@@ -5846,6 +6046,7 @@
       <c r="O160" s="1" t="n"/>
       <c r="P160" s="1" t="n"/>
       <c r="R160" s="20" t="n"/>
+      <c r="S160" s="39" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="1" t="n"/>
@@ -5865,6 +6066,7 @@
       <c r="O161" s="1" t="n"/>
       <c r="P161" s="1" t="n"/>
       <c r="R161" s="20" t="n"/>
+      <c r="S161" s="39" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="1" t="n"/>
@@ -5884,6 +6086,7 @@
       <c r="O162" s="1" t="n"/>
       <c r="P162" s="1" t="n"/>
       <c r="R162" s="20" t="n"/>
+      <c r="S162" s="39" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="1" t="n"/>
@@ -5903,6 +6106,7 @@
       <c r="O163" s="1" t="n"/>
       <c r="P163" s="1" t="n"/>
       <c r="R163" s="20" t="n"/>
+      <c r="S163" s="39" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="1" t="n"/>
@@ -5922,6 +6126,7 @@
       <c r="O164" s="1" t="n"/>
       <c r="P164" s="1" t="n"/>
       <c r="R164" s="20" t="n"/>
+      <c r="S164" s="39" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="1" t="n"/>
@@ -5941,6 +6146,7 @@
       <c r="O165" s="1" t="n"/>
       <c r="P165" s="1" t="n"/>
       <c r="R165" s="20" t="n"/>
+      <c r="S165" s="39" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="1" t="n"/>
@@ -5960,6 +6166,7 @@
       <c r="O166" s="1" t="n"/>
       <c r="P166" s="1" t="n"/>
       <c r="R166" s="20" t="n"/>
+      <c r="S166" s="39" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="1" t="n"/>
@@ -5979,6 +6186,7 @@
       <c r="O167" s="1" t="n"/>
       <c r="P167" s="1" t="n"/>
       <c r="R167" s="20" t="n"/>
+      <c r="S167" s="39" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="1" t="n"/>
@@ -5998,6 +6206,7 @@
       <c r="O168" s="1" t="n"/>
       <c r="P168" s="1" t="n"/>
       <c r="R168" s="20" t="n"/>
+      <c r="S168" s="39" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="1" t="n"/>
@@ -6017,6 +6226,7 @@
       <c r="O169" s="1" t="n"/>
       <c r="P169" s="1" t="n"/>
       <c r="R169" s="20" t="n"/>
+      <c r="S169" s="39" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="1" t="n"/>
@@ -6036,6 +6246,7 @@
       <c r="O170" s="1" t="n"/>
       <c r="P170" s="1" t="n"/>
       <c r="R170" s="20" t="n"/>
+      <c r="S170" s="39" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="1" t="n"/>
@@ -6055,6 +6266,7 @@
       <c r="O171" s="1" t="n"/>
       <c r="P171" s="1" t="n"/>
       <c r="R171" s="20" t="n"/>
+      <c r="S171" s="39" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="1" t="n"/>
@@ -6074,6 +6286,7 @@
       <c r="O172" s="1" t="n"/>
       <c r="P172" s="1" t="n"/>
       <c r="R172" s="20" t="n"/>
+      <c r="S172" s="39" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="1" t="n"/>
@@ -6093,6 +6306,7 @@
       <c r="O173" s="1" t="n"/>
       <c r="P173" s="1" t="n"/>
       <c r="R173" s="20" t="n"/>
+      <c r="S173" s="39" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="1" t="n"/>
@@ -6112,6 +6326,7 @@
       <c r="O174" s="1" t="n"/>
       <c r="P174" s="1" t="n"/>
       <c r="R174" s="20" t="n"/>
+      <c r="S174" s="39" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="1" t="n"/>
@@ -6131,6 +6346,7 @@
       <c r="O175" s="1" t="n"/>
       <c r="P175" s="1" t="n"/>
       <c r="R175" s="20" t="n"/>
+      <c r="S175" s="39" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="1" t="n"/>
@@ -6150,6 +6366,7 @@
       <c r="O176" s="1" t="n"/>
       <c r="P176" s="1" t="n"/>
       <c r="R176" s="20" t="n"/>
+      <c r="S176" s="39" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="1" t="n"/>
@@ -6169,6 +6386,7 @@
       <c r="O177" s="1" t="n"/>
       <c r="P177" s="1" t="n"/>
       <c r="R177" s="20" t="n"/>
+      <c r="S177" s="39" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="1" t="n"/>
@@ -6188,6 +6406,7 @@
       <c r="O178" s="1" t="n"/>
       <c r="P178" s="1" t="n"/>
       <c r="R178" s="20" t="n"/>
+      <c r="S178" s="39" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="1" t="n"/>
@@ -6207,6 +6426,7 @@
       <c r="O179" s="1" t="n"/>
       <c r="P179" s="1" t="n"/>
       <c r="R179" s="20" t="n"/>
+      <c r="S179" s="39" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="1" t="n"/>
@@ -6226,6 +6446,7 @@
       <c r="O180" s="1" t="n"/>
       <c r="P180" s="1" t="n"/>
       <c r="R180" s="20" t="n"/>
+      <c r="S180" s="39" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="1" t="n"/>
@@ -6245,6 +6466,7 @@
       <c r="O181" s="1" t="n"/>
       <c r="P181" s="1" t="n"/>
       <c r="R181" s="20" t="n"/>
+      <c r="S181" s="39" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="1" t="n"/>
@@ -6264,6 +6486,7 @@
       <c r="O182" s="1" t="n"/>
       <c r="P182" s="1" t="n"/>
       <c r="R182" s="20" t="n"/>
+      <c r="S182" s="39" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="1" t="n"/>
@@ -6283,6 +6506,7 @@
       <c r="O183" s="1" t="n"/>
       <c r="P183" s="1" t="n"/>
       <c r="R183" s="20" t="n"/>
+      <c r="S183" s="39" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="1" t="n"/>
@@ -6302,6 +6526,7 @@
       <c r="O184" s="1" t="n"/>
       <c r="P184" s="1" t="n"/>
       <c r="R184" s="20" t="n"/>
+      <c r="S184" s="39" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="1" t="n"/>
@@ -6321,6 +6546,7 @@
       <c r="O185" s="1" t="n"/>
       <c r="P185" s="1" t="n"/>
       <c r="R185" s="20" t="n"/>
+      <c r="S185" s="39" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="1" t="n"/>
@@ -6340,6 +6566,7 @@
       <c r="O186" s="1" t="n"/>
       <c r="P186" s="1" t="n"/>
       <c r="R186" s="20" t="n"/>
+      <c r="S186" s="39" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="1" t="n"/>
@@ -6359,6 +6586,7 @@
       <c r="O187" s="1" t="n"/>
       <c r="P187" s="1" t="n"/>
       <c r="R187" s="20" t="n"/>
+      <c r="S187" s="39" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="1" t="n"/>
@@ -6378,6 +6606,7 @@
       <c r="O188" s="1" t="n"/>
       <c r="P188" s="1" t="n"/>
       <c r="R188" s="20" t="n"/>
+      <c r="S188" s="39" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="1" t="n"/>
@@ -6397,6 +6626,7 @@
       <c r="O189" s="1" t="n"/>
       <c r="P189" s="1" t="n"/>
       <c r="R189" s="20" t="n"/>
+      <c r="S189" s="39" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="1" t="n"/>
@@ -6416,6 +6646,7 @@
       <c r="O190" s="1" t="n"/>
       <c r="P190" s="1" t="n"/>
       <c r="R190" s="20" t="n"/>
+      <c r="S190" s="39" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="1" t="n"/>
@@ -6435,6 +6666,7 @@
       <c r="O191" s="1" t="n"/>
       <c r="P191" s="1" t="n"/>
       <c r="R191" s="20" t="n"/>
+      <c r="S191" s="39" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="1" t="n"/>
@@ -6454,6 +6686,7 @@
       <c r="O192" s="1" t="n"/>
       <c r="P192" s="1" t="n"/>
       <c r="R192" s="20" t="n"/>
+      <c r="S192" s="39" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="1" t="n"/>
@@ -6473,6 +6706,7 @@
       <c r="O193" s="1" t="n"/>
       <c r="P193" s="1" t="n"/>
       <c r="R193" s="20" t="n"/>
+      <c r="S193" s="39" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="1" t="n"/>
@@ -6492,6 +6726,7 @@
       <c r="O194" s="1" t="n"/>
       <c r="P194" s="1" t="n"/>
       <c r="R194" s="20" t="n"/>
+      <c r="S194" s="39" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="1" t="n"/>
@@ -6511,6 +6746,7 @@
       <c r="O195" s="1" t="n"/>
       <c r="P195" s="1" t="n"/>
       <c r="R195" s="20" t="n"/>
+      <c r="S195" s="39" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="1" t="n"/>
@@ -6530,6 +6766,7 @@
       <c r="O196" s="1" t="n"/>
       <c r="P196" s="1" t="n"/>
       <c r="R196" s="20" t="n"/>
+      <c r="S196" s="39" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="1" t="n"/>
@@ -6549,6 +6786,7 @@
       <c r="O197" s="1" t="n"/>
       <c r="P197" s="1" t="n"/>
       <c r="R197" s="20" t="n"/>
+      <c r="S197" s="39" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="1" t="n"/>
@@ -6568,6 +6806,7 @@
       <c r="O198" s="1" t="n"/>
       <c r="P198" s="1" t="n"/>
       <c r="R198" s="20" t="n"/>
+      <c r="S198" s="39" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="1" t="n"/>
@@ -6587,6 +6826,7 @@
       <c r="O199" s="1" t="n"/>
       <c r="P199" s="1" t="n"/>
       <c r="R199" s="20" t="n"/>
+      <c r="S199" s="39" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="1" t="n"/>
@@ -6606,6 +6846,7 @@
       <c r="O200" s="1" t="n"/>
       <c r="P200" s="1" t="n"/>
       <c r="R200" s="20" t="n"/>
+      <c r="S200" s="39" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="1" t="n"/>
@@ -6625,6 +6866,7 @@
       <c r="O201" s="1" t="n"/>
       <c r="P201" s="1" t="n"/>
       <c r="R201" s="20" t="n"/>
+      <c r="S201" s="39" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="1" t="n"/>
@@ -6644,6 +6886,7 @@
       <c r="O202" s="1" t="n"/>
       <c r="P202" s="1" t="n"/>
       <c r="R202" s="20" t="n"/>
+      <c r="S202" s="39" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="1" t="n"/>
@@ -6663,6 +6906,7 @@
       <c r="O203" s="1" t="n"/>
       <c r="P203" s="1" t="n"/>
       <c r="R203" s="20" t="n"/>
+      <c r="S203" s="39" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="1" t="n"/>
@@ -6682,6 +6926,7 @@
       <c r="O204" s="1" t="n"/>
       <c r="P204" s="1" t="n"/>
       <c r="R204" s="20" t="n"/>
+      <c r="S204" s="39" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="1" t="n"/>
@@ -6701,6 +6946,7 @@
       <c r="O205" s="1" t="n"/>
       <c r="P205" s="1" t="n"/>
       <c r="R205" s="20" t="n"/>
+      <c r="S205" s="39" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="1" t="n"/>
@@ -6720,6 +6966,7 @@
       <c r="O206" s="1" t="n"/>
       <c r="P206" s="1" t="n"/>
       <c r="R206" s="20" t="n"/>
+      <c r="S206" s="39" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="1" t="n"/>
@@ -6739,6 +6986,7 @@
       <c r="O207" s="1" t="n"/>
       <c r="P207" s="1" t="n"/>
       <c r="R207" s="20" t="n"/>
+      <c r="S207" s="39" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="1" t="n"/>
@@ -6758,6 +7006,7 @@
       <c r="O208" s="1" t="n"/>
       <c r="P208" s="1" t="n"/>
       <c r="R208" s="20" t="n"/>
+      <c r="S208" s="39" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="1" t="n"/>
@@ -6777,6 +7026,7 @@
       <c r="O209" s="1" t="n"/>
       <c r="P209" s="1" t="n"/>
       <c r="R209" s="20" t="n"/>
+      <c r="S209" s="39" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="1" t="n"/>
@@ -6796,6 +7046,7 @@
       <c r="O210" s="1" t="n"/>
       <c r="P210" s="1" t="n"/>
       <c r="R210" s="20" t="n"/>
+      <c r="S210" s="39" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="1" t="n"/>
@@ -6815,6 +7066,7 @@
       <c r="O211" s="1" t="n"/>
       <c r="P211" s="1" t="n"/>
       <c r="R211" s="20" t="n"/>
+      <c r="S211" s="39" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="1" t="n"/>
@@ -6834,6 +7086,7 @@
       <c r="O212" s="1" t="n"/>
       <c r="P212" s="1" t="n"/>
       <c r="R212" s="20" t="n"/>
+      <c r="S212" s="39" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="1" t="n"/>
@@ -6853,6 +7106,7 @@
       <c r="O213" s="1" t="n"/>
       <c r="P213" s="1" t="n"/>
       <c r="R213" s="20" t="n"/>
+      <c r="S213" s="39" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="1" t="n"/>
@@ -6872,6 +7126,7 @@
       <c r="O214" s="1" t="n"/>
       <c r="P214" s="1" t="n"/>
       <c r="R214" s="20" t="n"/>
+      <c r="S214" s="39" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="1" t="n"/>
@@ -6891,6 +7146,7 @@
       <c r="O215" s="1" t="n"/>
       <c r="P215" s="1" t="n"/>
       <c r="R215" s="20" t="n"/>
+      <c r="S215" s="39" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="1" t="n"/>
@@ -6910,6 +7166,7 @@
       <c r="O216" s="1" t="n"/>
       <c r="P216" s="1" t="n"/>
       <c r="R216" s="20" t="n"/>
+      <c r="S216" s="39" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="1" t="n"/>
@@ -6929,6 +7186,7 @@
       <c r="O217" s="1" t="n"/>
       <c r="P217" s="1" t="n"/>
       <c r="R217" s="20" t="n"/>
+      <c r="S217" s="39" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="1" t="n"/>
@@ -6948,6 +7206,7 @@
       <c r="O218" s="1" t="n"/>
       <c r="P218" s="1" t="n"/>
       <c r="R218" s="20" t="n"/>
+      <c r="S218" s="39" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="1" t="n"/>
@@ -6967,6 +7226,7 @@
       <c r="O219" s="1" t="n"/>
       <c r="P219" s="1" t="n"/>
       <c r="R219" s="20" t="n"/>
+      <c r="S219" s="39" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="1" t="n"/>
@@ -6986,6 +7246,7 @@
       <c r="O220" s="1" t="n"/>
       <c r="P220" s="1" t="n"/>
       <c r="R220" s="20" t="n"/>
+      <c r="S220" s="39" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="1" t="n"/>
@@ -7005,6 +7266,7 @@
       <c r="O221" s="1" t="n"/>
       <c r="P221" s="1" t="n"/>
       <c r="R221" s="20" t="n"/>
+      <c r="S221" s="39" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="1" t="n"/>
@@ -7024,6 +7286,7 @@
       <c r="O222" s="1" t="n"/>
       <c r="P222" s="1" t="n"/>
       <c r="R222" s="20" t="n"/>
+      <c r="S222" s="39" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="1" t="n"/>
@@ -7043,6 +7306,7 @@
       <c r="O223" s="1" t="n"/>
       <c r="P223" s="1" t="n"/>
       <c r="R223" s="20" t="n"/>
+      <c r="S223" s="39" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="1" t="n"/>
@@ -7062,6 +7326,7 @@
       <c r="O224" s="1" t="n"/>
       <c r="P224" s="1" t="n"/>
       <c r="R224" s="20" t="n"/>
+      <c r="S224" s="39" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="1" t="n"/>
@@ -7081,6 +7346,7 @@
       <c r="O225" s="1" t="n"/>
       <c r="P225" s="1" t="n"/>
       <c r="R225" s="20" t="n"/>
+      <c r="S225" s="39" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="1" t="n"/>
@@ -7100,6 +7366,7 @@
       <c r="O226" s="1" t="n"/>
       <c r="P226" s="1" t="n"/>
       <c r="R226" s="20" t="n"/>
+      <c r="S226" s="39" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="1" t="n"/>
@@ -7119,6 +7386,7 @@
       <c r="O227" s="1" t="n"/>
       <c r="P227" s="1" t="n"/>
       <c r="R227" s="20" t="n"/>
+      <c r="S227" s="39" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="1" t="n"/>
@@ -7138,6 +7406,7 @@
       <c r="O228" s="1" t="n"/>
       <c r="P228" s="1" t="n"/>
       <c r="R228" s="20" t="n"/>
+      <c r="S228" s="39" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="1" t="n"/>
@@ -7157,6 +7426,7 @@
       <c r="O229" s="1" t="n"/>
       <c r="P229" s="1" t="n"/>
       <c r="R229" s="20" t="n"/>
+      <c r="S229" s="39" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="1" t="n"/>
@@ -7176,6 +7446,7 @@
       <c r="O230" s="1" t="n"/>
       <c r="P230" s="1" t="n"/>
       <c r="R230" s="20" t="n"/>
+      <c r="S230" s="39" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="1" t="n"/>
@@ -7195,6 +7466,7 @@
       <c r="O231" s="1" t="n"/>
       <c r="P231" s="1" t="n"/>
       <c r="R231" s="20" t="n"/>
+      <c r="S231" s="39" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="1" t="n"/>
@@ -7214,6 +7486,7 @@
       <c r="O232" s="1" t="n"/>
       <c r="P232" s="1" t="n"/>
       <c r="R232" s="20" t="n"/>
+      <c r="S232" s="39" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="1" t="n"/>
@@ -7233,6 +7506,7 @@
       <c r="O233" s="1" t="n"/>
       <c r="P233" s="1" t="n"/>
       <c r="R233" s="20" t="n"/>
+      <c r="S233" s="39" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="1" t="n"/>
@@ -7252,6 +7526,7 @@
       <c r="O234" s="1" t="n"/>
       <c r="P234" s="1" t="n"/>
       <c r="R234" s="20" t="n"/>
+      <c r="S234" s="39" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="1" t="n"/>
@@ -7271,6 +7546,7 @@
       <c r="O235" s="1" t="n"/>
       <c r="P235" s="1" t="n"/>
       <c r="R235" s="20" t="n"/>
+      <c r="S235" s="39" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="1" t="n"/>
@@ -7290,6 +7566,7 @@
       <c r="O236" s="1" t="n"/>
       <c r="P236" s="1" t="n"/>
       <c r="R236" s="20" t="n"/>
+      <c r="S236" s="39" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="1" t="n"/>
@@ -7309,6 +7586,7 @@
       <c r="O237" s="1" t="n"/>
       <c r="P237" s="1" t="n"/>
       <c r="R237" s="20" t="n"/>
+      <c r="S237" s="39" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="1" t="n"/>
@@ -7328,6 +7606,7 @@
       <c r="O238" s="1" t="n"/>
       <c r="P238" s="1" t="n"/>
       <c r="R238" s="20" t="n"/>
+      <c r="S238" s="39" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="1" t="n"/>
@@ -7347,6 +7626,7 @@
       <c r="O239" s="1" t="n"/>
       <c r="P239" s="1" t="n"/>
       <c r="R239" s="20" t="n"/>
+      <c r="S239" s="39" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="1" t="n"/>
@@ -7366,6 +7646,7 @@
       <c r="O240" s="1" t="n"/>
       <c r="P240" s="1" t="n"/>
       <c r="R240" s="20" t="n"/>
+      <c r="S240" s="39" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="1" t="n"/>
@@ -7385,6 +7666,7 @@
       <c r="O241" s="1" t="n"/>
       <c r="P241" s="1" t="n"/>
       <c r="R241" s="20" t="n"/>
+      <c r="S241" s="39" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="1" t="n"/>
@@ -7404,6 +7686,7 @@
       <c r="O242" s="1" t="n"/>
       <c r="P242" s="1" t="n"/>
       <c r="R242" s="20" t="n"/>
+      <c r="S242" s="39" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="1" t="n"/>
@@ -7423,6 +7706,7 @@
       <c r="O243" s="1" t="n"/>
       <c r="P243" s="1" t="n"/>
       <c r="R243" s="20" t="n"/>
+      <c r="S243" s="39" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="1" t="n"/>
@@ -7442,6 +7726,7 @@
       <c r="O244" s="1" t="n"/>
       <c r="P244" s="1" t="n"/>
       <c r="R244" s="20" t="n"/>
+      <c r="S244" s="39" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="1" t="n"/>
@@ -7461,6 +7746,7 @@
       <c r="O245" s="1" t="n"/>
       <c r="P245" s="1" t="n"/>
       <c r="R245" s="20" t="n"/>
+      <c r="S245" s="39" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="1" t="n"/>
@@ -7480,6 +7766,7 @@
       <c r="O246" s="1" t="n"/>
       <c r="P246" s="1" t="n"/>
       <c r="R246" s="20" t="n"/>
+      <c r="S246" s="39" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="1" t="n"/>
@@ -7499,6 +7786,7 @@
       <c r="O247" s="1" t="n"/>
       <c r="P247" s="1" t="n"/>
       <c r="R247" s="20" t="n"/>
+      <c r="S247" s="39" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="1" t="n"/>
@@ -7518,6 +7806,7 @@
       <c r="O248" s="1" t="n"/>
       <c r="P248" s="1" t="n"/>
       <c r="R248" s="20" t="n"/>
+      <c r="S248" s="39" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="1" t="n"/>
@@ -7537,6 +7826,7 @@
       <c r="O249" s="1" t="n"/>
       <c r="P249" s="1" t="n"/>
       <c r="R249" s="20" t="n"/>
+      <c r="S249" s="39" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="1" t="n"/>
@@ -7556,6 +7846,7 @@
       <c r="O250" s="1" t="n"/>
       <c r="P250" s="1" t="n"/>
       <c r="R250" s="20" t="n"/>
+      <c r="S250" s="39" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="1" t="n"/>
@@ -7575,6 +7866,7 @@
       <c r="O251" s="1" t="n"/>
       <c r="P251" s="1" t="n"/>
       <c r="R251" s="20" t="n"/>
+      <c r="S251" s="39" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="1" t="n"/>
@@ -7594,6 +7886,7 @@
       <c r="O252" s="1" t="n"/>
       <c r="P252" s="1" t="n"/>
       <c r="R252" s="20" t="n"/>
+      <c r="S252" s="39" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="1" t="n"/>
@@ -7613,6 +7906,7 @@
       <c r="O253" s="1" t="n"/>
       <c r="P253" s="1" t="n"/>
       <c r="R253" s="20" t="n"/>
+      <c r="S253" s="39" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="1" t="n"/>
@@ -7632,6 +7926,7 @@
       <c r="O254" s="1" t="n"/>
       <c r="P254" s="1" t="n"/>
       <c r="R254" s="20" t="n"/>
+      <c r="S254" s="39" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="1" t="n"/>
@@ -7651,6 +7946,7 @@
       <c r="O255" s="1" t="n"/>
       <c r="P255" s="1" t="n"/>
       <c r="R255" s="20" t="n"/>
+      <c r="S255" s="39" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="1" t="n"/>
@@ -7670,6 +7966,7 @@
       <c r="O256" s="1" t="n"/>
       <c r="P256" s="1" t="n"/>
       <c r="R256" s="20" t="n"/>
+      <c r="S256" s="39" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="1" t="n"/>
@@ -7689,6 +7986,7 @@
       <c r="O257" s="1" t="n"/>
       <c r="P257" s="1" t="n"/>
       <c r="R257" s="20" t="n"/>
+      <c r="S257" s="39" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="1" t="n"/>
@@ -7708,6 +8006,7 @@
       <c r="O258" s="1" t="n"/>
       <c r="P258" s="1" t="n"/>
       <c r="R258" s="20" t="n"/>
+      <c r="S258" s="39" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="1" t="n"/>
@@ -7727,6 +8026,7 @@
       <c r="O259" s="1" t="n"/>
       <c r="P259" s="1" t="n"/>
       <c r="R259" s="20" t="n"/>
+      <c r="S259" s="39" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="1" t="n"/>
@@ -7746,6 +8046,7 @@
       <c r="O260" s="1" t="n"/>
       <c r="P260" s="1" t="n"/>
       <c r="R260" s="20" t="n"/>
+      <c r="S260" s="39" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="1" t="n"/>
@@ -7765,6 +8066,7 @@
       <c r="O261" s="1" t="n"/>
       <c r="P261" s="1" t="n"/>
       <c r="R261" s="20" t="n"/>
+      <c r="S261" s="39" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="1" t="n"/>
@@ -7784,6 +8086,7 @@
       <c r="O262" s="1" t="n"/>
       <c r="P262" s="1" t="n"/>
       <c r="R262" s="20" t="n"/>
+      <c r="S262" s="39" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="1" t="n"/>
@@ -7803,6 +8106,7 @@
       <c r="O263" s="1" t="n"/>
       <c r="P263" s="1" t="n"/>
       <c r="R263" s="20" t="n"/>
+      <c r="S263" s="39" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="1" t="n"/>
@@ -7822,6 +8126,7 @@
       <c r="O264" s="1" t="n"/>
       <c r="P264" s="1" t="n"/>
       <c r="R264" s="20" t="n"/>
+      <c r="S264" s="39" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="1" t="n"/>
@@ -7841,6 +8146,7 @@
       <c r="O265" s="1" t="n"/>
       <c r="P265" s="1" t="n"/>
       <c r="R265" s="20" t="n"/>
+      <c r="S265" s="39" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="1" t="n"/>
@@ -7860,6 +8166,7 @@
       <c r="O266" s="1" t="n"/>
       <c r="P266" s="1" t="n"/>
       <c r="R266" s="20" t="n"/>
+      <c r="S266" s="39" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="1" t="n"/>
@@ -7879,6 +8186,7 @@
       <c r="O267" s="1" t="n"/>
       <c r="P267" s="1" t="n"/>
       <c r="R267" s="20" t="n"/>
+      <c r="S267" s="39" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="1" t="n"/>
@@ -7898,6 +8206,7 @@
       <c r="O268" s="1" t="n"/>
       <c r="P268" s="1" t="n"/>
       <c r="R268" s="20" t="n"/>
+      <c r="S268" s="39" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="1" t="n"/>
@@ -7917,6 +8226,7 @@
       <c r="O269" s="1" t="n"/>
       <c r="P269" s="1" t="n"/>
       <c r="R269" s="20" t="n"/>
+      <c r="S269" s="39" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="1" t="n"/>
@@ -7936,6 +8246,7 @@
       <c r="O270" s="1" t="n"/>
       <c r="P270" s="1" t="n"/>
       <c r="R270" s="20" t="n"/>
+      <c r="S270" s="39" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="1" t="n"/>
@@ -7955,6 +8266,7 @@
       <c r="O271" s="1" t="n"/>
       <c r="P271" s="1" t="n"/>
       <c r="R271" s="20" t="n"/>
+      <c r="S271" s="39" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="1" t="n"/>
@@ -7974,6 +8286,7 @@
       <c r="O272" s="1" t="n"/>
       <c r="P272" s="1" t="n"/>
       <c r="R272" s="20" t="n"/>
+      <c r="S272" s="39" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="1" t="n"/>
@@ -7993,6 +8306,7 @@
       <c r="O273" s="1" t="n"/>
       <c r="P273" s="1" t="n"/>
       <c r="R273" s="20" t="n"/>
+      <c r="S273" s="39" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="1" t="n"/>
@@ -8012,6 +8326,7 @@
       <c r="O274" s="1" t="n"/>
       <c r="P274" s="1" t="n"/>
       <c r="R274" s="20" t="n"/>
+      <c r="S274" s="39" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="1" t="n"/>
@@ -8031,6 +8346,7 @@
       <c r="O275" s="1" t="n"/>
       <c r="P275" s="1" t="n"/>
       <c r="R275" s="20" t="n"/>
+      <c r="S275" s="39" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="1" t="n"/>
@@ -8050,6 +8366,7 @@
       <c r="O276" s="1" t="n"/>
       <c r="P276" s="1" t="n"/>
       <c r="R276" s="20" t="n"/>
+      <c r="S276" s="39" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="1" t="n"/>
@@ -8069,6 +8386,7 @@
       <c r="O277" s="1" t="n"/>
       <c r="P277" s="1" t="n"/>
       <c r="R277" s="20" t="n"/>
+      <c r="S277" s="39" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="1" t="n"/>
@@ -8088,6 +8406,7 @@
       <c r="O278" s="1" t="n"/>
       <c r="P278" s="1" t="n"/>
       <c r="R278" s="20" t="n"/>
+      <c r="S278" s="39" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="1" t="n"/>
@@ -8107,6 +8426,7 @@
       <c r="O279" s="1" t="n"/>
       <c r="P279" s="1" t="n"/>
       <c r="R279" s="20" t="n"/>
+      <c r="S279" s="39" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="1" t="n"/>
@@ -8126,6 +8446,7 @@
       <c r="O280" s="1" t="n"/>
       <c r="P280" s="1" t="n"/>
       <c r="R280" s="20" t="n"/>
+      <c r="S280" s="39" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="1" t="n"/>
@@ -8145,6 +8466,7 @@
       <c r="O281" s="1" t="n"/>
       <c r="P281" s="1" t="n"/>
       <c r="R281" s="20" t="n"/>
+      <c r="S281" s="39" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="1" t="n"/>
@@ -8164,6 +8486,7 @@
       <c r="O282" s="1" t="n"/>
       <c r="P282" s="1" t="n"/>
       <c r="R282" s="20" t="n"/>
+      <c r="S282" s="39" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="1" t="n"/>
@@ -8183,6 +8506,7 @@
       <c r="O283" s="1" t="n"/>
       <c r="P283" s="1" t="n"/>
       <c r="R283" s="20" t="n"/>
+      <c r="S283" s="39" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="1" t="n"/>
@@ -8202,6 +8526,7 @@
       <c r="O284" s="1" t="n"/>
       <c r="P284" s="1" t="n"/>
       <c r="R284" s="20" t="n"/>
+      <c r="S284" s="39" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="1" t="n"/>
@@ -8221,6 +8546,7 @@
       <c r="O285" s="1" t="n"/>
       <c r="P285" s="1" t="n"/>
       <c r="R285" s="20" t="n"/>
+      <c r="S285" s="39" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="1" t="n"/>
@@ -8240,6 +8566,7 @@
       <c r="O286" s="1" t="n"/>
       <c r="P286" s="1" t="n"/>
       <c r="R286" s="20" t="n"/>
+      <c r="S286" s="39" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="1" t="n"/>
@@ -8259,6 +8586,7 @@
       <c r="O287" s="1" t="n"/>
       <c r="P287" s="1" t="n"/>
       <c r="R287" s="20" t="n"/>
+      <c r="S287" s="39" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="1" t="n"/>
@@ -8278,6 +8606,7 @@
       <c r="O288" s="1" t="n"/>
       <c r="P288" s="1" t="n"/>
       <c r="R288" s="20" t="n"/>
+      <c r="S288" s="39" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="1" t="n"/>
@@ -8297,6 +8626,7 @@
       <c r="O289" s="1" t="n"/>
       <c r="P289" s="1" t="n"/>
       <c r="R289" s="20" t="n"/>
+      <c r="S289" s="39" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="1" t="n"/>
@@ -8316,6 +8646,7 @@
       <c r="O290" s="1" t="n"/>
       <c r="P290" s="1" t="n"/>
       <c r="R290" s="20" t="n"/>
+      <c r="S290" s="39" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="1" t="n"/>
@@ -8335,6 +8666,7 @@
       <c r="O291" s="1" t="n"/>
       <c r="P291" s="1" t="n"/>
       <c r="R291" s="20" t="n"/>
+      <c r="S291" s="39" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="1" t="n"/>
@@ -8354,6 +8686,7 @@
       <c r="O292" s="1" t="n"/>
       <c r="P292" s="1" t="n"/>
       <c r="R292" s="20" t="n"/>
+      <c r="S292" s="39" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="1" t="n"/>
@@ -8373,6 +8706,7 @@
       <c r="O293" s="1" t="n"/>
       <c r="P293" s="1" t="n"/>
       <c r="R293" s="20" t="n"/>
+      <c r="S293" s="39" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="1" t="n"/>
@@ -8392,6 +8726,7 @@
       <c r="O294" s="1" t="n"/>
       <c r="P294" s="1" t="n"/>
       <c r="R294" s="20" t="n"/>
+      <c r="S294" s="39" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="1" t="n"/>
@@ -8411,6 +8746,7 @@
       <c r="O295" s="1" t="n"/>
       <c r="P295" s="1" t="n"/>
       <c r="R295" s="20" t="n"/>
+      <c r="S295" s="39" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="1" t="n"/>
@@ -8430,6 +8766,7 @@
       <c r="O296" s="1" t="n"/>
       <c r="P296" s="1" t="n"/>
       <c r="R296" s="20" t="n"/>
+      <c r="S296" s="39" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="1" t="n"/>
@@ -8449,6 +8786,7 @@
       <c r="O297" s="1" t="n"/>
       <c r="P297" s="1" t="n"/>
       <c r="R297" s="20" t="n"/>
+      <c r="S297" s="39" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="1" t="n"/>
@@ -8468,6 +8806,7 @@
       <c r="O298" s="1" t="n"/>
       <c r="P298" s="1" t="n"/>
       <c r="R298" s="20" t="n"/>
+      <c r="S298" s="39" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="1" t="n"/>
@@ -8487,6 +8826,7 @@
       <c r="O299" s="1" t="n"/>
       <c r="P299" s="1" t="n"/>
       <c r="R299" s="20" t="n"/>
+      <c r="S299" s="39" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="1" t="n"/>
@@ -8506,6 +8846,7 @@
       <c r="O300" s="1" t="n"/>
       <c r="P300" s="1" t="n"/>
       <c r="R300" s="20" t="n"/>
+      <c r="S300" s="39" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="1" t="n"/>
@@ -8525,6 +8866,7 @@
       <c r="O301" s="1" t="n"/>
       <c r="P301" s="1" t="n"/>
       <c r="R301" s="20" t="n"/>
+      <c r="S301" s="39" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="1" t="n"/>
@@ -8544,6 +8886,7 @@
       <c r="O302" s="1" t="n"/>
       <c r="P302" s="1" t="n"/>
       <c r="R302" s="20" t="n"/>
+      <c r="S302" s="39" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="1" t="n"/>
@@ -8563,6 +8906,7 @@
       <c r="O303" s="1" t="n"/>
       <c r="P303" s="1" t="n"/>
       <c r="R303" s="20" t="n"/>
+      <c r="S303" s="39" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="1" t="n"/>
@@ -8582,6 +8926,7 @@
       <c r="O304" s="1" t="n"/>
       <c r="P304" s="1" t="n"/>
       <c r="R304" s="20" t="n"/>
+      <c r="S304" s="39" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="1" t="n"/>
@@ -8601,6 +8946,7 @@
       <c r="O305" s="1" t="n"/>
       <c r="P305" s="1" t="n"/>
       <c r="R305" s="20" t="n"/>
+      <c r="S305" s="39" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="1" t="n"/>
@@ -8620,6 +8966,7 @@
       <c r="O306" s="1" t="n"/>
       <c r="P306" s="1" t="n"/>
       <c r="R306" s="20" t="n"/>
+      <c r="S306" s="39" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="1" t="n"/>
@@ -8639,6 +8986,7 @@
       <c r="O307" s="1" t="n"/>
       <c r="P307" s="1" t="n"/>
       <c r="R307" s="20" t="n"/>
+      <c r="S307" s="39" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="1" t="n"/>
@@ -8658,6 +9006,7 @@
       <c r="O308" s="1" t="n"/>
       <c r="P308" s="1" t="n"/>
       <c r="R308" s="20" t="n"/>
+      <c r="S308" s="39" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="1" t="n"/>
@@ -8677,6 +9026,7 @@
       <c r="O309" s="1" t="n"/>
       <c r="P309" s="1" t="n"/>
       <c r="R309" s="20" t="n"/>
+      <c r="S309" s="39" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="1" t="n"/>
@@ -8696,6 +9046,7 @@
       <c r="O310" s="1" t="n"/>
       <c r="P310" s="1" t="n"/>
       <c r="R310" s="20" t="n"/>
+      <c r="S310" s="39" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="1" t="n"/>
@@ -8715,6 +9066,7 @@
       <c r="O311" s="1" t="n"/>
       <c r="P311" s="1" t="n"/>
       <c r="R311" s="20" t="n"/>
+      <c r="S311" s="39" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="1" t="n"/>
@@ -8734,6 +9086,7 @@
       <c r="O312" s="1" t="n"/>
       <c r="P312" s="1" t="n"/>
       <c r="R312" s="20" t="n"/>
+      <c r="S312" s="39" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="1" t="n"/>
@@ -8753,6 +9106,7 @@
       <c r="O313" s="1" t="n"/>
       <c r="P313" s="1" t="n"/>
       <c r="R313" s="20" t="n"/>
+      <c r="S313" s="39" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="1" t="n"/>
@@ -8772,6 +9126,7 @@
       <c r="O314" s="1" t="n"/>
       <c r="P314" s="1" t="n"/>
       <c r="R314" s="20" t="n"/>
+      <c r="S314" s="39" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="1" t="n"/>
@@ -8791,6 +9146,7 @@
       <c r="O315" s="1" t="n"/>
       <c r="P315" s="1" t="n"/>
       <c r="R315" s="20" t="n"/>
+      <c r="S315" s="39" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="1" t="n"/>
@@ -8810,6 +9166,7 @@
       <c r="O316" s="1" t="n"/>
       <c r="P316" s="1" t="n"/>
       <c r="R316" s="20" t="n"/>
+      <c r="S316" s="39" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="1" t="n"/>
@@ -8829,6 +9186,7 @@
       <c r="O317" s="1" t="n"/>
       <c r="P317" s="1" t="n"/>
       <c r="R317" s="20" t="n"/>
+      <c r="S317" s="39" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="1" t="n"/>
@@ -8848,6 +9206,7 @@
       <c r="O318" s="1" t="n"/>
       <c r="P318" s="1" t="n"/>
       <c r="R318" s="20" t="n"/>
+      <c r="S318" s="39" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="1" t="n"/>
@@ -8867,6 +9226,7 @@
       <c r="O319" s="1" t="n"/>
       <c r="P319" s="1" t="n"/>
       <c r="R319" s="20" t="n"/>
+      <c r="S319" s="39" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="1" t="n"/>
@@ -8886,6 +9246,7 @@
       <c r="O320" s="1" t="n"/>
       <c r="P320" s="1" t="n"/>
       <c r="R320" s="20" t="n"/>
+      <c r="S320" s="39" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="1" t="n"/>
@@ -8905,6 +9266,7 @@
       <c r="O321" s="1" t="n"/>
       <c r="P321" s="1" t="n"/>
       <c r="R321" s="20" t="n"/>
+      <c r="S321" s="39" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="1" t="n"/>
@@ -8924,6 +9286,7 @@
       <c r="O322" s="1" t="n"/>
       <c r="P322" s="1" t="n"/>
       <c r="R322" s="20" t="n"/>
+      <c r="S322" s="39" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="1" t="n"/>
@@ -8943,6 +9306,7 @@
       <c r="O323" s="1" t="n"/>
       <c r="P323" s="1" t="n"/>
       <c r="R323" s="20" t="n"/>
+      <c r="S323" s="39" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="1" t="n"/>
@@ -8962,6 +9326,7 @@
       <c r="O324" s="1" t="n"/>
       <c r="P324" s="1" t="n"/>
       <c r="R324" s="20" t="n"/>
+      <c r="S324" s="39" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="1" t="n"/>
@@ -8981,6 +9346,7 @@
       <c r="O325" s="1" t="n"/>
       <c r="P325" s="1" t="n"/>
       <c r="R325" s="20" t="n"/>
+      <c r="S325" s="39" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="1" t="n"/>
@@ -9000,6 +9366,7 @@
       <c r="O326" s="1" t="n"/>
       <c r="P326" s="1" t="n"/>
       <c r="R326" s="20" t="n"/>
+      <c r="S326" s="39" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="1" t="n"/>
@@ -9019,6 +9386,7 @@
       <c r="O327" s="1" t="n"/>
       <c r="P327" s="1" t="n"/>
       <c r="R327" s="20" t="n"/>
+      <c r="S327" s="39" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="1" t="n"/>
@@ -9038,6 +9406,7 @@
       <c r="O328" s="1" t="n"/>
       <c r="P328" s="1" t="n"/>
       <c r="R328" s="20" t="n"/>
+      <c r="S328" s="39" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="1" t="n"/>
@@ -9057,6 +9426,7 @@
       <c r="O329" s="1" t="n"/>
       <c r="P329" s="1" t="n"/>
       <c r="R329" s="20" t="n"/>
+      <c r="S329" s="39" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="1" t="n"/>
@@ -9076,6 +9446,7 @@
       <c r="O330" s="1" t="n"/>
       <c r="P330" s="1" t="n"/>
       <c r="R330" s="20" t="n"/>
+      <c r="S330" s="39" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="1" t="n"/>
@@ -9095,6 +9466,7 @@
       <c r="O331" s="1" t="n"/>
       <c r="P331" s="1" t="n"/>
       <c r="R331" s="20" t="n"/>
+      <c r="S331" s="39" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="1" t="n"/>
@@ -9114,6 +9486,7 @@
       <c r="O332" s="1" t="n"/>
       <c r="P332" s="1" t="n"/>
       <c r="R332" s="20" t="n"/>
+      <c r="S332" s="39" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="1" t="n"/>
@@ -9133,6 +9506,7 @@
       <c r="O333" s="1" t="n"/>
       <c r="P333" s="1" t="n"/>
       <c r="R333" s="20" t="n"/>
+      <c r="S333" s="39" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="1" t="n"/>
@@ -9152,6 +9526,7 @@
       <c r="O334" s="1" t="n"/>
       <c r="P334" s="1" t="n"/>
       <c r="R334" s="20" t="n"/>
+      <c r="S334" s="39" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="1" t="n"/>
@@ -9171,6 +9546,7 @@
       <c r="O335" s="1" t="n"/>
       <c r="P335" s="1" t="n"/>
       <c r="R335" s="20" t="n"/>
+      <c r="S335" s="39" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="1" t="n"/>
@@ -9190,6 +9566,7 @@
       <c r="O336" s="1" t="n"/>
       <c r="P336" s="1" t="n"/>
       <c r="R336" s="20" t="n"/>
+      <c r="S336" s="39" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="1" t="n"/>
@@ -9209,6 +9586,7 @@
       <c r="O337" s="1" t="n"/>
       <c r="P337" s="1" t="n"/>
       <c r="R337" s="20" t="n"/>
+      <c r="S337" s="39" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="1" t="n"/>
@@ -9228,6 +9606,7 @@
       <c r="O338" s="1" t="n"/>
       <c r="P338" s="1" t="n"/>
       <c r="R338" s="20" t="n"/>
+      <c r="S338" s="39" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="1" t="n"/>
@@ -9247,6 +9626,7 @@
       <c r="O339" s="1" t="n"/>
       <c r="P339" s="1" t="n"/>
       <c r="R339" s="20" t="n"/>
+      <c r="S339" s="39" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="1" t="n"/>
@@ -9266,6 +9646,7 @@
       <c r="O340" s="1" t="n"/>
       <c r="P340" s="1" t="n"/>
       <c r="R340" s="20" t="n"/>
+      <c r="S340" s="39" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="1" t="n"/>
@@ -9285,6 +9666,7 @@
       <c r="O341" s="1" t="n"/>
       <c r="P341" s="1" t="n"/>
       <c r="R341" s="20" t="n"/>
+      <c r="S341" s="39" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="1" t="n"/>
@@ -9304,6 +9686,7 @@
       <c r="O342" s="1" t="n"/>
       <c r="P342" s="1" t="n"/>
       <c r="R342" s="20" t="n"/>
+      <c r="S342" s="39" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="1" t="n"/>
@@ -9323,6 +9706,7 @@
       <c r="O343" s="1" t="n"/>
       <c r="P343" s="1" t="n"/>
       <c r="R343" s="20" t="n"/>
+      <c r="S343" s="39" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="1" t="n"/>
@@ -9342,6 +9726,7 @@
       <c r="O344" s="1" t="n"/>
       <c r="P344" s="1" t="n"/>
       <c r="R344" s="20" t="n"/>
+      <c r="S344" s="39" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="1" t="n"/>
@@ -9361,6 +9746,7 @@
       <c r="O345" s="1" t="n"/>
       <c r="P345" s="1" t="n"/>
       <c r="R345" s="20" t="n"/>
+      <c r="S345" s="39" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="1" t="n"/>
@@ -9380,6 +9766,7 @@
       <c r="O346" s="1" t="n"/>
       <c r="P346" s="1" t="n"/>
       <c r="R346" s="20" t="n"/>
+      <c r="S346" s="39" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="1" t="n"/>
@@ -9399,6 +9786,7 @@
       <c r="O347" s="1" t="n"/>
       <c r="P347" s="1" t="n"/>
       <c r="R347" s="20" t="n"/>
+      <c r="S347" s="39" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="1" t="n"/>
@@ -9418,6 +9806,7 @@
       <c r="O348" s="1" t="n"/>
       <c r="P348" s="1" t="n"/>
       <c r="R348" s="20" t="n"/>
+      <c r="S348" s="39" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="1" t="n"/>
@@ -9437,6 +9826,7 @@
       <c r="O349" s="1" t="n"/>
       <c r="P349" s="1" t="n"/>
       <c r="R349" s="20" t="n"/>
+      <c r="S349" s="39" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="1" t="n"/>
@@ -9456,6 +9846,7 @@
       <c r="O350" s="1" t="n"/>
       <c r="P350" s="1" t="n"/>
       <c r="R350" s="20" t="n"/>
+      <c r="S350" s="39" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="1" t="n"/>
@@ -9475,6 +9866,7 @@
       <c r="O351" s="1" t="n"/>
       <c r="P351" s="1" t="n"/>
       <c r="R351" s="20" t="n"/>
+      <c r="S351" s="39" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="1" t="n"/>
@@ -9494,6 +9886,7 @@
       <c r="O352" s="1" t="n"/>
       <c r="P352" s="1" t="n"/>
       <c r="R352" s="20" t="n"/>
+      <c r="S352" s="39" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="1" t="n"/>
@@ -9513,6 +9906,7 @@
       <c r="O353" s="1" t="n"/>
       <c r="P353" s="1" t="n"/>
       <c r="R353" s="20" t="n"/>
+      <c r="S353" s="39" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="1" t="n"/>
@@ -9532,6 +9926,7 @@
       <c r="O354" s="1" t="n"/>
       <c r="P354" s="1" t="n"/>
       <c r="R354" s="20" t="n"/>
+      <c r="S354" s="39" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="1" t="n"/>
@@ -9551,6 +9946,7 @@
       <c r="O355" s="1" t="n"/>
       <c r="P355" s="1" t="n"/>
       <c r="R355" s="20" t="n"/>
+      <c r="S355" s="39" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="1" t="n"/>
@@ -9570,6 +9966,7 @@
       <c r="O356" s="1" t="n"/>
       <c r="P356" s="1" t="n"/>
       <c r="R356" s="20" t="n"/>
+      <c r="S356" s="39" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="1" t="n"/>
@@ -9589,6 +9986,7 @@
       <c r="O357" s="1" t="n"/>
       <c r="P357" s="1" t="n"/>
       <c r="R357" s="20" t="n"/>
+      <c r="S357" s="39" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="1" t="n"/>
@@ -9608,6 +10006,7 @@
       <c r="O358" s="1" t="n"/>
       <c r="P358" s="1" t="n"/>
       <c r="R358" s="20" t="n"/>
+      <c r="S358" s="39" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="1" t="n"/>
@@ -9627,6 +10026,7 @@
       <c r="O359" s="1" t="n"/>
       <c r="P359" s="1" t="n"/>
       <c r="R359" s="20" t="n"/>
+      <c r="S359" s="39" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="1" t="n"/>
@@ -9646,6 +10046,7 @@
       <c r="O360" s="1" t="n"/>
       <c r="P360" s="1" t="n"/>
       <c r="R360" s="20" t="n"/>
+      <c r="S360" s="39" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="1" t="n"/>
@@ -9665,6 +10066,7 @@
       <c r="O361" s="1" t="n"/>
       <c r="P361" s="1" t="n"/>
       <c r="R361" s="20" t="n"/>
+      <c r="S361" s="39" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="1" t="n"/>
@@ -9684,6 +10086,7 @@
       <c r="O362" s="1" t="n"/>
       <c r="P362" s="1" t="n"/>
       <c r="R362" s="20" t="n"/>
+      <c r="S362" s="39" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="1" t="n"/>
@@ -9703,6 +10106,7 @@
       <c r="O363" s="1" t="n"/>
       <c r="P363" s="1" t="n"/>
       <c r="R363" s="20" t="n"/>
+      <c r="S363" s="39" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="1" t="n"/>
@@ -9722,6 +10126,7 @@
       <c r="O364" s="1" t="n"/>
       <c r="P364" s="1" t="n"/>
       <c r="R364" s="20" t="n"/>
+      <c r="S364" s="39" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="1" t="n"/>
@@ -9741,6 +10146,7 @@
       <c r="O365" s="1" t="n"/>
       <c r="P365" s="1" t="n"/>
       <c r="R365" s="20" t="n"/>
+      <c r="S365" s="39" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="1" t="n"/>
@@ -9760,6 +10166,7 @@
       <c r="O366" s="1" t="n"/>
       <c r="P366" s="1" t="n"/>
       <c r="R366" s="20" t="n"/>
+      <c r="S366" s="39" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="1" t="n"/>
@@ -9779,6 +10186,7 @@
       <c r="O367" s="1" t="n"/>
       <c r="P367" s="1" t="n"/>
       <c r="R367" s="20" t="n"/>
+      <c r="S367" s="39" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="1" t="n"/>
@@ -9798,6 +10206,7 @@
       <c r="O368" s="1" t="n"/>
       <c r="P368" s="1" t="n"/>
       <c r="R368" s="20" t="n"/>
+      <c r="S368" s="39" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="1" t="n"/>
@@ -9817,6 +10226,7 @@
       <c r="O369" s="1" t="n"/>
       <c r="P369" s="1" t="n"/>
       <c r="R369" s="20" t="n"/>
+      <c r="S369" s="39" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="1" t="n"/>
@@ -9836,6 +10246,7 @@
       <c r="O370" s="1" t="n"/>
       <c r="P370" s="1" t="n"/>
       <c r="R370" s="20" t="n"/>
+      <c r="S370" s="39" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="1" t="n"/>
@@ -9855,6 +10266,7 @@
       <c r="O371" s="1" t="n"/>
       <c r="P371" s="1" t="n"/>
       <c r="R371" s="20" t="n"/>
+      <c r="S371" s="39" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="1" t="n"/>
@@ -9874,6 +10286,7 @@
       <c r="O372" s="1" t="n"/>
       <c r="P372" s="1" t="n"/>
       <c r="R372" s="20" t="n"/>
+      <c r="S372" s="39" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="1" t="n"/>
@@ -9893,6 +10306,7 @@
       <c r="O373" s="1" t="n"/>
       <c r="P373" s="1" t="n"/>
       <c r="R373" s="20" t="n"/>
+      <c r="S373" s="39" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="1" t="n"/>
@@ -9912,6 +10326,7 @@
       <c r="O374" s="1" t="n"/>
       <c r="P374" s="1" t="n"/>
       <c r="R374" s="20" t="n"/>
+      <c r="S374" s="39" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="1" t="n"/>
@@ -9931,6 +10346,7 @@
       <c r="O375" s="1" t="n"/>
       <c r="P375" s="1" t="n"/>
       <c r="R375" s="20" t="n"/>
+      <c r="S375" s="39" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="1" t="n"/>
@@ -9950,6 +10366,7 @@
       <c r="O376" s="1" t="n"/>
       <c r="P376" s="1" t="n"/>
       <c r="R376" s="20" t="n"/>
+      <c r="S376" s="39" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="1" t="n"/>
@@ -9969,6 +10386,7 @@
       <c r="O377" s="1" t="n"/>
       <c r="P377" s="1" t="n"/>
       <c r="R377" s="20" t="n"/>
+      <c r="S377" s="39" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="1" t="n"/>
@@ -9988,6 +10406,7 @@
       <c r="O378" s="1" t="n"/>
       <c r="P378" s="1" t="n"/>
       <c r="R378" s="20" t="n"/>
+      <c r="S378" s="39" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="1" t="n"/>
@@ -10007,6 +10426,7 @@
       <c r="O379" s="1" t="n"/>
       <c r="P379" s="1" t="n"/>
       <c r="R379" s="20" t="n"/>
+      <c r="S379" s="39" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="1" t="n"/>
@@ -10026,6 +10446,7 @@
       <c r="O380" s="1" t="n"/>
       <c r="P380" s="1" t="n"/>
       <c r="R380" s="20" t="n"/>
+      <c r="S380" s="39" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="1" t="n"/>
@@ -10045,6 +10466,7 @@
       <c r="O381" s="1" t="n"/>
       <c r="P381" s="1" t="n"/>
       <c r="R381" s="20" t="n"/>
+      <c r="S381" s="39" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="1" t="n"/>
@@ -10064,6 +10486,7 @@
       <c r="O382" s="1" t="n"/>
       <c r="P382" s="1" t="n"/>
       <c r="R382" s="20" t="n"/>
+      <c r="S382" s="39" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="1" t="n"/>
@@ -10083,6 +10506,7 @@
       <c r="O383" s="1" t="n"/>
       <c r="P383" s="1" t="n"/>
       <c r="R383" s="20" t="n"/>
+      <c r="S383" s="39" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="1" t="n"/>
@@ -10102,6 +10526,7 @@
       <c r="O384" s="1" t="n"/>
       <c r="P384" s="1" t="n"/>
       <c r="R384" s="20" t="n"/>
+      <c r="S384" s="39" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="1" t="n"/>
@@ -10121,6 +10546,7 @@
       <c r="O385" s="1" t="n"/>
       <c r="P385" s="1" t="n"/>
       <c r="R385" s="20" t="n"/>
+      <c r="S385" s="39" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="1" t="n"/>
@@ -10140,6 +10566,7 @@
       <c r="O386" s="1" t="n"/>
       <c r="P386" s="1" t="n"/>
       <c r="R386" s="20" t="n"/>
+      <c r="S386" s="39" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="1" t="n"/>
@@ -10159,6 +10586,7 @@
       <c r="O387" s="1" t="n"/>
       <c r="P387" s="1" t="n"/>
       <c r="R387" s="20" t="n"/>
+      <c r="S387" s="39" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="1" t="n"/>
@@ -10178,6 +10606,7 @@
       <c r="O388" s="1" t="n"/>
       <c r="P388" s="1" t="n"/>
       <c r="R388" s="20" t="n"/>
+      <c r="S388" s="39" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="1" t="n"/>
@@ -10197,6 +10626,7 @@
       <c r="O389" s="1" t="n"/>
       <c r="P389" s="1" t="n"/>
       <c r="R389" s="20" t="n"/>
+      <c r="S389" s="39" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="1" t="n"/>
@@ -10216,6 +10646,7 @@
       <c r="O390" s="1" t="n"/>
       <c r="P390" s="1" t="n"/>
       <c r="R390" s="20" t="n"/>
+      <c r="S390" s="39" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="1" t="n"/>
@@ -10235,6 +10666,7 @@
       <c r="O391" s="1" t="n"/>
       <c r="P391" s="1" t="n"/>
       <c r="R391" s="20" t="n"/>
+      <c r="S391" s="39" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="1" t="n"/>
@@ -10254,6 +10686,7 @@
       <c r="O392" s="1" t="n"/>
       <c r="P392" s="1" t="n"/>
       <c r="R392" s="20" t="n"/>
+      <c r="S392" s="39" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="1" t="n"/>
@@ -10273,6 +10706,7 @@
       <c r="O393" s="1" t="n"/>
       <c r="P393" s="1" t="n"/>
       <c r="R393" s="20" t="n"/>
+      <c r="S393" s="39" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="1" t="n"/>
@@ -10292,6 +10726,7 @@
       <c r="O394" s="1" t="n"/>
       <c r="P394" s="1" t="n"/>
       <c r="R394" s="20" t="n"/>
+      <c r="S394" s="39" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="1" t="n"/>
@@ -10311,6 +10746,7 @@
       <c r="O395" s="1" t="n"/>
       <c r="P395" s="1" t="n"/>
       <c r="R395" s="20" t="n"/>
+      <c r="S395" s="39" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="1" t="n"/>
@@ -10330,6 +10766,7 @@
       <c r="O396" s="1" t="n"/>
       <c r="P396" s="1" t="n"/>
       <c r="R396" s="20" t="n"/>
+      <c r="S396" s="39" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="1" t="n"/>
@@ -10349,6 +10786,7 @@
       <c r="O397" s="1" t="n"/>
       <c r="P397" s="1" t="n"/>
       <c r="R397" s="20" t="n"/>
+      <c r="S397" s="39" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="1" t="n"/>
@@ -10368,6 +10806,7 @@
       <c r="O398" s="1" t="n"/>
       <c r="P398" s="1" t="n"/>
       <c r="R398" s="20" t="n"/>
+      <c r="S398" s="39" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="1" t="n"/>
@@ -10387,6 +10826,7 @@
       <c r="O399" s="1" t="n"/>
       <c r="P399" s="1" t="n"/>
       <c r="R399" s="20" t="n"/>
+      <c r="S399" s="39" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="1" t="n"/>
@@ -10406,6 +10846,7 @@
       <c r="O400" s="1" t="n"/>
       <c r="P400" s="1" t="n"/>
       <c r="R400" s="20" t="n"/>
+      <c r="S400" s="39" t="n"/>
     </row>
     <row r="401">
       <c r="A401" s="1" t="n"/>
@@ -10425,6 +10866,7 @@
       <c r="O401" s="1" t="n"/>
       <c r="P401" s="1" t="n"/>
       <c r="R401" s="20" t="n"/>
+      <c r="S401" s="39" t="n"/>
     </row>
     <row r="402">
       <c r="A402" s="1" t="n"/>
@@ -10444,6 +10886,7 @@
       <c r="O402" s="1" t="n"/>
       <c r="P402" s="1" t="n"/>
       <c r="R402" s="20" t="n"/>
+      <c r="S402" s="39" t="n"/>
     </row>
     <row r="403">
       <c r="A403" s="1" t="n"/>
@@ -10463,6 +10906,7 @@
       <c r="O403" s="1" t="n"/>
       <c r="P403" s="1" t="n"/>
       <c r="R403" s="20" t="n"/>
+      <c r="S403" s="39" t="n"/>
     </row>
     <row r="404">
       <c r="A404" s="1" t="n"/>
@@ -10482,6 +10926,7 @@
       <c r="O404" s="1" t="n"/>
       <c r="P404" s="1" t="n"/>
       <c r="R404" s="20" t="n"/>
+      <c r="S404" s="39" t="n"/>
     </row>
     <row r="405">
       <c r="A405" s="1" t="n"/>
@@ -10501,6 +10946,7 @@
       <c r="O405" s="1" t="n"/>
       <c r="P405" s="1" t="n"/>
       <c r="R405" s="20" t="n"/>
+      <c r="S405" s="39" t="n"/>
     </row>
     <row r="406">
       <c r="A406" s="1" t="n"/>
@@ -10520,6 +10966,7 @@
       <c r="O406" s="1" t="n"/>
       <c r="P406" s="1" t="n"/>
       <c r="R406" s="20" t="n"/>
+      <c r="S406" s="39" t="n"/>
     </row>
     <row r="407">
       <c r="A407" s="1" t="n"/>
@@ -10539,6 +10986,7 @@
       <c r="O407" s="1" t="n"/>
       <c r="P407" s="1" t="n"/>
       <c r="R407" s="20" t="n"/>
+      <c r="S407" s="39" t="n"/>
     </row>
     <row r="408">
       <c r="A408" s="1" t="n"/>
@@ -10558,6 +11006,7 @@
       <c r="O408" s="1" t="n"/>
       <c r="P408" s="1" t="n"/>
       <c r="R408" s="20" t="n"/>
+      <c r="S408" s="39" t="n"/>
     </row>
     <row r="409">
       <c r="A409" s="1" t="n"/>
@@ -10577,6 +11026,7 @@
       <c r="O409" s="1" t="n"/>
       <c r="P409" s="1" t="n"/>
       <c r="R409" s="20" t="n"/>
+      <c r="S409" s="39" t="n"/>
     </row>
     <row r="410">
       <c r="A410" s="1" t="n"/>
@@ -10596,6 +11046,7 @@
       <c r="O410" s="1" t="n"/>
       <c r="P410" s="1" t="n"/>
       <c r="R410" s="20" t="n"/>
+      <c r="S410" s="39" t="n"/>
     </row>
     <row r="411">
       <c r="A411" s="1" t="n"/>
@@ -10615,6 +11066,7 @@
       <c r="O411" s="1" t="n"/>
       <c r="P411" s="1" t="n"/>
       <c r="R411" s="20" t="n"/>
+      <c r="S411" s="39" t="n"/>
     </row>
     <row r="412">
       <c r="A412" s="1" t="n"/>
@@ -10634,6 +11086,7 @@
       <c r="O412" s="1" t="n"/>
       <c r="P412" s="1" t="n"/>
       <c r="R412" s="20" t="n"/>
+      <c r="S412" s="39" t="n"/>
     </row>
     <row r="413">
       <c r="A413" s="1" t="n"/>
@@ -10653,6 +11106,7 @@
       <c r="O413" s="1" t="n"/>
       <c r="P413" s="1" t="n"/>
       <c r="R413" s="20" t="n"/>
+      <c r="S413" s="39" t="n"/>
     </row>
     <row r="414">
       <c r="A414" s="1" t="n"/>
@@ -10672,6 +11126,7 @@
       <c r="O414" s="1" t="n"/>
       <c r="P414" s="1" t="n"/>
       <c r="R414" s="20" t="n"/>
+      <c r="S414" s="39" t="n"/>
     </row>
     <row r="415">
       <c r="A415" s="1" t="n"/>
@@ -10691,6 +11146,7 @@
       <c r="O415" s="1" t="n"/>
       <c r="P415" s="1" t="n"/>
       <c r="R415" s="20" t="n"/>
+      <c r="S415" s="39" t="n"/>
     </row>
     <row r="416">
       <c r="A416" s="1" t="n"/>
@@ -10710,6 +11166,7 @@
       <c r="O416" s="1" t="n"/>
       <c r="P416" s="1" t="n"/>
       <c r="R416" s="20" t="n"/>
+      <c r="S416" s="39" t="n"/>
     </row>
     <row r="417">
       <c r="A417" s="1" t="n"/>
@@ -10729,6 +11186,7 @@
       <c r="O417" s="1" t="n"/>
       <c r="P417" s="1" t="n"/>
       <c r="R417" s="20" t="n"/>
+      <c r="S417" s="39" t="n"/>
     </row>
     <row r="418">
       <c r="A418" s="1" t="n"/>
@@ -10748,6 +11206,7 @@
       <c r="O418" s="1" t="n"/>
       <c r="P418" s="1" t="n"/>
       <c r="R418" s="20" t="n"/>
+      <c r="S418" s="39" t="n"/>
     </row>
     <row r="419">
       <c r="A419" s="1" t="n"/>
@@ -10767,6 +11226,7 @@
       <c r="O419" s="1" t="n"/>
       <c r="P419" s="1" t="n"/>
       <c r="R419" s="20" t="n"/>
+      <c r="S419" s="39" t="n"/>
     </row>
     <row r="420">
       <c r="A420" s="1" t="n"/>
@@ -10786,6 +11246,7 @@
       <c r="O420" s="1" t="n"/>
       <c r="P420" s="1" t="n"/>
       <c r="R420" s="20" t="n"/>
+      <c r="S420" s="39" t="n"/>
     </row>
     <row r="421">
       <c r="A421" s="1" t="n"/>
@@ -10805,6 +11266,7 @@
       <c r="O421" s="1" t="n"/>
       <c r="P421" s="1" t="n"/>
       <c r="R421" s="20" t="n"/>
+      <c r="S421" s="39" t="n"/>
     </row>
     <row r="422">
       <c r="A422" s="1" t="n"/>
@@ -10824,6 +11286,7 @@
       <c r="O422" s="1" t="n"/>
       <c r="P422" s="1" t="n"/>
       <c r="R422" s="20" t="n"/>
+      <c r="S422" s="39" t="n"/>
     </row>
     <row r="423">
       <c r="A423" s="1" t="n"/>
@@ -10843,6 +11306,7 @@
       <c r="O423" s="1" t="n"/>
       <c r="P423" s="1" t="n"/>
       <c r="R423" s="20" t="n"/>
+      <c r="S423" s="39" t="n"/>
     </row>
     <row r="424">
       <c r="A424" s="1" t="n"/>
@@ -10862,6 +11326,7 @@
       <c r="O424" s="1" t="n"/>
       <c r="P424" s="1" t="n"/>
       <c r="R424" s="20" t="n"/>
+      <c r="S424" s="39" t="n"/>
     </row>
     <row r="425">
       <c r="A425" s="1" t="n"/>
@@ -10881,6 +11346,7 @@
       <c r="O425" s="1" t="n"/>
       <c r="P425" s="1" t="n"/>
       <c r="R425" s="20" t="n"/>
+      <c r="S425" s="39" t="n"/>
     </row>
     <row r="426">
       <c r="A426" s="1" t="n"/>
@@ -10900,6 +11366,7 @@
       <c r="O426" s="1" t="n"/>
       <c r="P426" s="1" t="n"/>
       <c r="R426" s="20" t="n"/>
+      <c r="S426" s="39" t="n"/>
     </row>
     <row r="427">
       <c r="A427" s="1" t="n"/>
@@ -10919,6 +11386,7 @@
       <c r="O427" s="1" t="n"/>
       <c r="P427" s="1" t="n"/>
       <c r="R427" s="20" t="n"/>
+      <c r="S427" s="39" t="n"/>
     </row>
     <row r="428">
       <c r="A428" s="1" t="n"/>
@@ -10938,6 +11406,7 @@
       <c r="O428" s="1" t="n"/>
       <c r="P428" s="1" t="n"/>
       <c r="R428" s="20" t="n"/>
+      <c r="S428" s="39" t="n"/>
     </row>
     <row r="429">
       <c r="A429" s="1" t="n"/>
@@ -10957,6 +11426,7 @@
       <c r="O429" s="1" t="n"/>
       <c r="P429" s="1" t="n"/>
       <c r="R429" s="20" t="n"/>
+      <c r="S429" s="39" t="n"/>
     </row>
     <row r="430">
       <c r="A430" s="1" t="n"/>
@@ -10976,6 +11446,7 @@
       <c r="O430" s="1" t="n"/>
       <c r="P430" s="1" t="n"/>
       <c r="R430" s="20" t="n"/>
+      <c r="S430" s="39" t="n"/>
     </row>
     <row r="431">
       <c r="A431" s="1" t="n"/>
@@ -10995,6 +11466,7 @@
       <c r="O431" s="1" t="n"/>
       <c r="P431" s="1" t="n"/>
       <c r="R431" s="20" t="n"/>
+      <c r="S431" s="39" t="n"/>
     </row>
     <row r="432">
       <c r="A432" s="1" t="n"/>
@@ -11014,6 +11486,7 @@
       <c r="O432" s="1" t="n"/>
       <c r="P432" s="1" t="n"/>
       <c r="R432" s="20" t="n"/>
+      <c r="S432" s="39" t="n"/>
     </row>
     <row r="433">
       <c r="A433" s="1" t="n"/>
@@ -11033,6 +11506,7 @@
       <c r="O433" s="1" t="n"/>
       <c r="P433" s="1" t="n"/>
       <c r="R433" s="20" t="n"/>
+      <c r="S433" s="39" t="n"/>
     </row>
     <row r="434">
       <c r="A434" s="1" t="n"/>
@@ -11052,6 +11526,7 @@
       <c r="O434" s="1" t="n"/>
       <c r="P434" s="1" t="n"/>
       <c r="R434" s="20" t="n"/>
+      <c r="S434" s="39" t="n"/>
     </row>
     <row r="435">
       <c r="A435" s="1" t="n"/>
@@ -11071,6 +11546,7 @@
       <c r="O435" s="1" t="n"/>
       <c r="P435" s="1" t="n"/>
       <c r="R435" s="20" t="n"/>
+      <c r="S435" s="39" t="n"/>
     </row>
     <row r="436">
       <c r="A436" s="1" t="n"/>
@@ -11090,6 +11566,7 @@
       <c r="O436" s="1" t="n"/>
       <c r="P436" s="1" t="n"/>
       <c r="R436" s="20" t="n"/>
+      <c r="S436" s="39" t="n"/>
     </row>
     <row r="437">
       <c r="A437" s="1" t="n"/>
@@ -11109,6 +11586,7 @@
       <c r="O437" s="1" t="n"/>
       <c r="P437" s="1" t="n"/>
       <c r="R437" s="20" t="n"/>
+      <c r="S437" s="39" t="n"/>
     </row>
     <row r="438">
       <c r="A438" s="1" t="n"/>
@@ -11128,6 +11606,7 @@
       <c r="O438" s="1" t="n"/>
       <c r="P438" s="1" t="n"/>
       <c r="R438" s="20" t="n"/>
+      <c r="S438" s="39" t="n"/>
     </row>
     <row r="439">
       <c r="A439" s="1" t="n"/>
@@ -11147,6 +11626,7 @@
       <c r="O439" s="1" t="n"/>
       <c r="P439" s="1" t="n"/>
       <c r="R439" s="20" t="n"/>
+      <c r="S439" s="39" t="n"/>
     </row>
     <row r="440">
       <c r="A440" s="1" t="n"/>
@@ -11166,6 +11646,7 @@
       <c r="O440" s="1" t="n"/>
       <c r="P440" s="1" t="n"/>
       <c r="R440" s="20" t="n"/>
+      <c r="S440" s="39" t="n"/>
     </row>
     <row r="441">
       <c r="A441" s="1" t="n"/>
@@ -11185,6 +11666,7 @@
       <c r="O441" s="1" t="n"/>
       <c r="P441" s="1" t="n"/>
       <c r="R441" s="20" t="n"/>
+      <c r="S441" s="39" t="n"/>
     </row>
     <row r="442">
       <c r="A442" s="1" t="n"/>
@@ -11204,6 +11686,7 @@
       <c r="O442" s="1" t="n"/>
       <c r="P442" s="1" t="n"/>
       <c r="R442" s="20" t="n"/>
+      <c r="S442" s="39" t="n"/>
     </row>
     <row r="443">
       <c r="A443" s="1" t="n"/>
@@ -11223,6 +11706,7 @@
       <c r="O443" s="1" t="n"/>
       <c r="P443" s="1" t="n"/>
       <c r="R443" s="20" t="n"/>
+      <c r="S443" s="39" t="n"/>
     </row>
     <row r="444">
       <c r="A444" s="1" t="n"/>
@@ -11242,6 +11726,7 @@
       <c r="O444" s="1" t="n"/>
       <c r="P444" s="1" t="n"/>
       <c r="R444" s="20" t="n"/>
+      <c r="S444" s="39" t="n"/>
     </row>
     <row r="445">
       <c r="A445" s="1" t="n"/>
@@ -11261,6 +11746,7 @@
       <c r="O445" s="1" t="n"/>
       <c r="P445" s="1" t="n"/>
       <c r="R445" s="20" t="n"/>
+      <c r="S445" s="39" t="n"/>
     </row>
     <row r="446">
       <c r="A446" s="1" t="n"/>
@@ -11280,6 +11766,7 @@
       <c r="O446" s="1" t="n"/>
       <c r="P446" s="1" t="n"/>
       <c r="R446" s="20" t="n"/>
+      <c r="S446" s="39" t="n"/>
     </row>
     <row r="447">
       <c r="A447" s="1" t="n"/>
@@ -11299,6 +11786,7 @@
       <c r="O447" s="1" t="n"/>
       <c r="P447" s="1" t="n"/>
       <c r="R447" s="20" t="n"/>
+      <c r="S447" s="39" t="n"/>
     </row>
     <row r="448">
       <c r="A448" s="1" t="n"/>
@@ -11318,6 +11806,7 @@
       <c r="O448" s="1" t="n"/>
       <c r="P448" s="1" t="n"/>
       <c r="R448" s="20" t="n"/>
+      <c r="S448" s="39" t="n"/>
     </row>
     <row r="449">
       <c r="A449" s="1" t="n"/>
@@ -11337,6 +11826,7 @@
       <c r="O449" s="1" t="n"/>
       <c r="P449" s="1" t="n"/>
       <c r="R449" s="20" t="n"/>
+      <c r="S449" s="39" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="1" t="n"/>
@@ -11356,6 +11846,7 @@
       <c r="O450" s="1" t="n"/>
       <c r="P450" s="1" t="n"/>
       <c r="R450" s="20" t="n"/>
+      <c r="S450" s="39" t="n"/>
     </row>
     <row r="451">
       <c r="A451" s="1" t="n"/>
@@ -11375,6 +11866,7 @@
       <c r="O451" s="1" t="n"/>
       <c r="P451" s="1" t="n"/>
       <c r="R451" s="20" t="n"/>
+      <c r="S451" s="39" t="n"/>
     </row>
     <row r="452">
       <c r="A452" s="1" t="n"/>
@@ -11394,6 +11886,7 @@
       <c r="O452" s="1" t="n"/>
       <c r="P452" s="1" t="n"/>
       <c r="R452" s="20" t="n"/>
+      <c r="S452" s="39" t="n"/>
     </row>
     <row r="453">
       <c r="A453" s="1" t="n"/>
@@ -11413,6 +11906,7 @@
       <c r="O453" s="1" t="n"/>
       <c r="P453" s="1" t="n"/>
       <c r="R453" s="20" t="n"/>
+      <c r="S453" s="39" t="n"/>
     </row>
     <row r="454">
       <c r="A454" s="1" t="n"/>
@@ -11432,6 +11926,7 @@
       <c r="O454" s="1" t="n"/>
       <c r="P454" s="1" t="n"/>
       <c r="R454" s="20" t="n"/>
+      <c r="S454" s="39" t="n"/>
     </row>
     <row r="455">
       <c r="A455" s="1" t="n"/>
@@ -11451,6 +11946,7 @@
       <c r="O455" s="1" t="n"/>
       <c r="P455" s="1" t="n"/>
       <c r="R455" s="20" t="n"/>
+      <c r="S455" s="39" t="n"/>
     </row>
     <row r="456">
       <c r="A456" s="1" t="n"/>
@@ -11470,6 +11966,7 @@
       <c r="O456" s="1" t="n"/>
       <c r="P456" s="1" t="n"/>
       <c r="R456" s="20" t="n"/>
+      <c r="S456" s="39" t="n"/>
     </row>
     <row r="457">
       <c r="A457" s="1" t="n"/>
@@ -11489,6 +11986,7 @@
       <c r="O457" s="1" t="n"/>
       <c r="P457" s="1" t="n"/>
       <c r="R457" s="20" t="n"/>
+      <c r="S457" s="39" t="n"/>
     </row>
     <row r="458">
       <c r="A458" s="1" t="n"/>
@@ -11508,6 +12006,7 @@
       <c r="O458" s="1" t="n"/>
       <c r="P458" s="1" t="n"/>
       <c r="R458" s="20" t="n"/>
+      <c r="S458" s="39" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="1" t="n"/>
@@ -11527,6 +12026,7 @@
       <c r="O459" s="1" t="n"/>
       <c r="P459" s="1" t="n"/>
       <c r="R459" s="20" t="n"/>
+      <c r="S459" s="39" t="n"/>
     </row>
     <row r="460">
       <c r="A460" s="1" t="n"/>
@@ -11546,6 +12046,7 @@
       <c r="O460" s="1" t="n"/>
       <c r="P460" s="1" t="n"/>
       <c r="R460" s="20" t="n"/>
+      <c r="S460" s="39" t="n"/>
     </row>
     <row r="461">
       <c r="A461" s="1" t="n"/>
@@ -11565,6 +12066,7 @@
       <c r="O461" s="1" t="n"/>
       <c r="P461" s="1" t="n"/>
       <c r="R461" s="20" t="n"/>
+      <c r="S461" s="39" t="n"/>
     </row>
     <row r="462">
       <c r="A462" s="1" t="n"/>
@@ -11584,6 +12086,7 @@
       <c r="O462" s="1" t="n"/>
       <c r="P462" s="1" t="n"/>
       <c r="R462" s="20" t="n"/>
+      <c r="S462" s="39" t="n"/>
     </row>
     <row r="463">
       <c r="A463" s="1" t="n"/>
@@ -11603,6 +12106,7 @@
       <c r="O463" s="1" t="n"/>
       <c r="P463" s="1" t="n"/>
       <c r="R463" s="20" t="n"/>
+      <c r="S463" s="39" t="n"/>
     </row>
     <row r="464">
       <c r="A464" s="1" t="n"/>
@@ -11622,6 +12126,7 @@
       <c r="O464" s="1" t="n"/>
       <c r="P464" s="1" t="n"/>
       <c r="R464" s="20" t="n"/>
+      <c r="S464" s="39" t="n"/>
     </row>
     <row r="465">
       <c r="A465" s="1" t="n"/>
@@ -11641,6 +12146,7 @@
       <c r="O465" s="1" t="n"/>
       <c r="P465" s="1" t="n"/>
       <c r="R465" s="20" t="n"/>
+      <c r="S465" s="39" t="n"/>
     </row>
     <row r="466">
       <c r="A466" s="1" t="n"/>
@@ -11660,6 +12166,7 @@
       <c r="O466" s="1" t="n"/>
       <c r="P466" s="1" t="n"/>
       <c r="R466" s="20" t="n"/>
+      <c r="S466" s="39" t="n"/>
     </row>
     <row r="467">
       <c r="A467" s="1" t="n"/>
@@ -11679,6 +12186,7 @@
       <c r="O467" s="1" t="n"/>
       <c r="P467" s="1" t="n"/>
       <c r="R467" s="20" t="n"/>
+      <c r="S467" s="39" t="n"/>
     </row>
     <row r="468">
       <c r="A468" s="1" t="n"/>
@@ -11698,6 +12206,7 @@
       <c r="O468" s="1" t="n"/>
       <c r="P468" s="1" t="n"/>
       <c r="R468" s="20" t="n"/>
+      <c r="S468" s="39" t="n"/>
     </row>
     <row r="469">
       <c r="A469" s="1" t="n"/>
@@ -11717,6 +12226,7 @@
       <c r="O469" s="1" t="n"/>
       <c r="P469" s="1" t="n"/>
       <c r="R469" s="20" t="n"/>
+      <c r="S469" s="39" t="n"/>
     </row>
     <row r="470">
       <c r="A470" s="1" t="n"/>
@@ -11736,6 +12246,7 @@
       <c r="O470" s="1" t="n"/>
       <c r="P470" s="1" t="n"/>
       <c r="R470" s="20" t="n"/>
+      <c r="S470" s="39" t="n"/>
     </row>
     <row r="471">
       <c r="A471" s="1" t="n"/>
@@ -11755,6 +12266,7 @@
       <c r="O471" s="1" t="n"/>
       <c r="P471" s="1" t="n"/>
       <c r="R471" s="20" t="n"/>
+      <c r="S471" s="39" t="n"/>
     </row>
     <row r="472">
       <c r="A472" s="1" t="n"/>
@@ -11774,6 +12286,7 @@
       <c r="O472" s="1" t="n"/>
       <c r="P472" s="1" t="n"/>
       <c r="R472" s="20" t="n"/>
+      <c r="S472" s="39" t="n"/>
     </row>
     <row r="473">
       <c r="A473" s="1" t="n"/>
@@ -11793,6 +12306,7 @@
       <c r="O473" s="1" t="n"/>
       <c r="P473" s="1" t="n"/>
       <c r="R473" s="20" t="n"/>
+      <c r="S473" s="39" t="n"/>
     </row>
     <row r="474">
       <c r="A474" s="1" t="n"/>
@@ -11812,6 +12326,7 @@
       <c r="O474" s="1" t="n"/>
       <c r="P474" s="1" t="n"/>
       <c r="R474" s="20" t="n"/>
+      <c r="S474" s="39" t="n"/>
     </row>
     <row r="475">
       <c r="A475" s="1" t="n"/>
@@ -11831,6 +12346,7 @@
       <c r="O475" s="1" t="n"/>
       <c r="P475" s="1" t="n"/>
       <c r="R475" s="20" t="n"/>
+      <c r="S475" s="39" t="n"/>
     </row>
     <row r="476">
       <c r="A476" s="1" t="n"/>
@@ -11850,6 +12366,7 @@
       <c r="O476" s="1" t="n"/>
       <c r="P476" s="1" t="n"/>
       <c r="R476" s="20" t="n"/>
+      <c r="S476" s="39" t="n"/>
     </row>
     <row r="477">
       <c r="A477" s="1" t="n"/>
@@ -11869,6 +12386,7 @@
       <c r="O477" s="1" t="n"/>
       <c r="P477" s="1" t="n"/>
       <c r="R477" s="20" t="n"/>
+      <c r="S477" s="39" t="n"/>
     </row>
     <row r="478">
       <c r="A478" s="1" t="n"/>
@@ -11888,6 +12406,7 @@
       <c r="O478" s="1" t="n"/>
       <c r="P478" s="1" t="n"/>
       <c r="R478" s="20" t="n"/>
+      <c r="S478" s="39" t="n"/>
     </row>
     <row r="479">
       <c r="A479" s="1" t="n"/>
@@ -11907,6 +12426,7 @@
       <c r="O479" s="1" t="n"/>
       <c r="P479" s="1" t="n"/>
       <c r="R479" s="20" t="n"/>
+      <c r="S479" s="39" t="n"/>
     </row>
     <row r="480">
       <c r="A480" s="1" t="n"/>
@@ -11926,6 +12446,7 @@
       <c r="O480" s="1" t="n"/>
       <c r="P480" s="1" t="n"/>
       <c r="R480" s="20" t="n"/>
+      <c r="S480" s="39" t="n"/>
     </row>
     <row r="481">
       <c r="A481" s="1" t="n"/>
@@ -11945,6 +12466,7 @@
       <c r="O481" s="1" t="n"/>
       <c r="P481" s="1" t="n"/>
       <c r="R481" s="20" t="n"/>
+      <c r="S481" s="39" t="n"/>
     </row>
     <row r="482">
       <c r="A482" s="1" t="n"/>
@@ -11964,6 +12486,7 @@
       <c r="O482" s="1" t="n"/>
       <c r="P482" s="1" t="n"/>
       <c r="R482" s="20" t="n"/>
+      <c r="S482" s="39" t="n"/>
     </row>
     <row r="483">
       <c r="A483" s="1" t="n"/>
@@ -11983,6 +12506,7 @@
       <c r="O483" s="1" t="n"/>
       <c r="P483" s="1" t="n"/>
       <c r="R483" s="20" t="n"/>
+      <c r="S483" s="39" t="n"/>
     </row>
     <row r="484">
       <c r="A484" s="1" t="n"/>
@@ -12002,6 +12526,7 @@
       <c r="O484" s="1" t="n"/>
       <c r="P484" s="1" t="n"/>
       <c r="R484" s="20" t="n"/>
+      <c r="S484" s="39" t="n"/>
     </row>
     <row r="485">
       <c r="A485" s="1" t="n"/>
@@ -12021,6 +12546,7 @@
       <c r="O485" s="1" t="n"/>
       <c r="P485" s="1" t="n"/>
       <c r="R485" s="20" t="n"/>
+      <c r="S485" s="39" t="n"/>
     </row>
     <row r="486">
       <c r="A486" s="1" t="n"/>
@@ -12040,6 +12566,7 @@
       <c r="O486" s="1" t="n"/>
       <c r="P486" s="1" t="n"/>
       <c r="R486" s="20" t="n"/>
+      <c r="S486" s="39" t="n"/>
     </row>
     <row r="487">
       <c r="A487" s="1" t="n"/>
@@ -12059,6 +12586,7 @@
       <c r="O487" s="1" t="n"/>
       <c r="P487" s="1" t="n"/>
       <c r="R487" s="20" t="n"/>
+      <c r="S487" s="39" t="n"/>
     </row>
     <row r="488">
       <c r="A488" s="1" t="n"/>
@@ -12078,6 +12606,7 @@
       <c r="O488" s="1" t="n"/>
       <c r="P488" s="1" t="n"/>
       <c r="R488" s="20" t="n"/>
+      <c r="S488" s="39" t="n"/>
     </row>
     <row r="489">
       <c r="A489" s="1" t="n"/>
@@ -12097,6 +12626,7 @@
       <c r="O489" s="1" t="n"/>
       <c r="P489" s="1" t="n"/>
       <c r="R489" s="20" t="n"/>
+      <c r="S489" s="39" t="n"/>
     </row>
     <row r="490">
       <c r="A490" s="1" t="n"/>
@@ -12116,6 +12646,7 @@
       <c r="O490" s="1" t="n"/>
       <c r="P490" s="1" t="n"/>
       <c r="R490" s="20" t="n"/>
+      <c r="S490" s="39" t="n"/>
     </row>
     <row r="491">
       <c r="A491" s="1" t="n"/>
@@ -12135,6 +12666,7 @@
       <c r="O491" s="1" t="n"/>
       <c r="P491" s="1" t="n"/>
       <c r="R491" s="20" t="n"/>
+      <c r="S491" s="39" t="n"/>
     </row>
     <row r="492">
       <c r="A492" s="1" t="n"/>
@@ -12154,6 +12686,7 @@
       <c r="O492" s="1" t="n"/>
       <c r="P492" s="1" t="n"/>
       <c r="R492" s="20" t="n"/>
+      <c r="S492" s="39" t="n"/>
     </row>
     <row r="493">
       <c r="A493" s="1" t="n"/>
@@ -12173,6 +12706,7 @@
       <c r="O493" s="1" t="n"/>
       <c r="P493" s="1" t="n"/>
       <c r="R493" s="20" t="n"/>
+      <c r="S493" s="39" t="n"/>
     </row>
     <row r="494">
       <c r="A494" s="1" t="n"/>
@@ -12192,6 +12726,7 @@
       <c r="O494" s="1" t="n"/>
       <c r="P494" s="1" t="n"/>
       <c r="R494" s="20" t="n"/>
+      <c r="S494" s="39" t="n"/>
     </row>
     <row r="495">
       <c r="A495" s="1" t="n"/>
@@ -12211,6 +12746,7 @@
       <c r="O495" s="1" t="n"/>
       <c r="P495" s="1" t="n"/>
       <c r="R495" s="20" t="n"/>
+      <c r="S495" s="39" t="n"/>
     </row>
     <row r="496">
       <c r="A496" s="1" t="n"/>
@@ -12230,6 +12766,7 @@
       <c r="O496" s="1" t="n"/>
       <c r="P496" s="1" t="n"/>
       <c r="R496" s="20" t="n"/>
+      <c r="S496" s="39" t="n"/>
     </row>
     <row r="497">
       <c r="A497" s="1" t="n"/>
@@ -12249,6 +12786,7 @@
       <c r="O497" s="1" t="n"/>
       <c r="P497" s="1" t="n"/>
       <c r="R497" s="20" t="n"/>
+      <c r="S497" s="39" t="n"/>
     </row>
     <row r="498">
       <c r="A498" s="1" t="n"/>
@@ -12268,6 +12806,7 @@
       <c r="O498" s="1" t="n"/>
       <c r="P498" s="1" t="n"/>
       <c r="R498" s="20" t="n"/>
+      <c r="S498" s="39" t="n"/>
     </row>
     <row r="499">
       <c r="A499" s="1" t="n"/>
@@ -12287,6 +12826,7 @@
       <c r="O499" s="1" t="n"/>
       <c r="P499" s="1" t="n"/>
       <c r="R499" s="20" t="n"/>
+      <c r="S499" s="39" t="n"/>
     </row>
     <row r="500">
       <c r="A500" s="1" t="n"/>
@@ -12306,6 +12846,7 @@
       <c r="O500" s="1" t="n"/>
       <c r="P500" s="1" t="n"/>
       <c r="R500" s="20" t="n"/>
+      <c r="S500" s="39" t="n"/>
     </row>
     <row r="501">
       <c r="A501" s="1" t="n"/>
@@ -12325,9 +12866,10 @@
       <c r="O501" s="1" t="n"/>
       <c r="P501" s="1" t="n"/>
       <c r="R501" s="20" t="n"/>
+      <c r="S501" s="39" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R501"/>
+  <autoFilter ref="A1:S501"/>
   <dataValidations count="5">
     <dataValidation sqref="A2:A501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Projects!$A$2:$A$51</formula1>
@@ -13361,15 +13903,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="86" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13382,7 +13925,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Rebuilt automatically from the Selections sheet - do not edit here. Enter prices in the Unit Price column on Selections; Price = Qty x Unit Price.</t>
+          <t>Rebuilt automatically from the Selections sheet - do not edit here. Enter costs in the Unit Price and Markup % columns on Selections; Price = Qty x Unit Price x (1 + Markup %).</t>
         </is>
       </c>
     </row>
@@ -13413,6 +13956,11 @@
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>Markup %</t>
+        </is>
+      </c>
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
@@ -13454,8 +14002,12 @@
         <f>IF(Selections!R2="","",Selections!R2)</f>
         <v/>
       </c>
-      <c r="F7" s="31">
-        <f>IF(ISNUMBER(E7),D7*E7,"")</f>
+      <c r="F7" s="40">
+        <f>IF(Selections!S2="","",Selections!S2)</f>
+        <v/>
+      </c>
+      <c r="G7" s="31">
+        <f>IF(ISNUMBER(E7),D7*E7*(1+IF(ISNUMBER(F7),F7,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13465,8 +14017,8 @@
           <t>Exterior subtotal</t>
         </is>
       </c>
-      <c r="F8" s="33">
-        <f>SUM(F7:F7)</f>
+      <c r="G8" s="33">
+        <f>SUM(G7:G7)</f>
         <v/>
       </c>
     </row>
@@ -13499,8 +14051,12 @@
         <f>IF(Selections!R3="","",Selections!R3)</f>
         <v/>
       </c>
-      <c r="F10" s="31">
-        <f>IF(ISNUMBER(E10),D10*E10,"")</f>
+      <c r="F10" s="40">
+        <f>IF(Selections!S3="","",Selections!S3)</f>
+        <v/>
+      </c>
+      <c r="G10" s="31">
+        <f>IF(ISNUMBER(E10),D10*E10*(1+IF(ISNUMBER(F10),F10,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13510,8 +14066,8 @@
           <t>Windows &amp; Doors subtotal</t>
         </is>
       </c>
-      <c r="F11" s="33">
-        <f>SUM(F10:F10)</f>
+      <c r="G11" s="33">
+        <f>SUM(G10:G10)</f>
         <v/>
       </c>
     </row>
@@ -13544,8 +14100,12 @@
         <f>IF(Selections!R4="","",Selections!R4)</f>
         <v/>
       </c>
-      <c r="F13" s="31">
-        <f>IF(ISNUMBER(E13),D13*E13,"")</f>
+      <c r="F13" s="40">
+        <f>IF(Selections!S4="","",Selections!S4)</f>
+        <v/>
+      </c>
+      <c r="G13" s="31">
+        <f>IF(ISNUMBER(E13),D13*E13*(1+IF(ISNUMBER(F13),F13,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13555,8 +14115,8 @@
           <t>Kitchen subtotal</t>
         </is>
       </c>
-      <c r="F14" s="33">
-        <f>SUM(F13:F13)</f>
+      <c r="G14" s="33">
+        <f>SUM(G13:G13)</f>
         <v/>
       </c>
     </row>
@@ -13589,8 +14149,12 @@
         <f>IF(Selections!R5="","",Selections!R5)</f>
         <v/>
       </c>
-      <c r="F16" s="31">
-        <f>IF(ISNUMBER(E16),D16*E16,"")</f>
+      <c r="F16" s="40">
+        <f>IF(Selections!S5="","",Selections!S5)</f>
+        <v/>
+      </c>
+      <c r="G16" s="31">
+        <f>IF(ISNUMBER(E16),D16*E16*(1+IF(ISNUMBER(F16),F16,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13600,8 +14164,8 @@
           <t>Bathrooms subtotal</t>
         </is>
       </c>
-      <c r="F17" s="33">
-        <f>SUM(F16:F16)</f>
+      <c r="G17" s="33">
+        <f>SUM(G16:G16)</f>
         <v/>
       </c>
     </row>
@@ -13634,8 +14198,12 @@
         <f>IF(Selections!R6="","",Selections!R6)</f>
         <v/>
       </c>
-      <c r="F19" s="31">
-        <f>IF(ISNUMBER(E19),D19*E19,"")</f>
+      <c r="F19" s="40">
+        <f>IF(Selections!S6="","",Selections!S6)</f>
+        <v/>
+      </c>
+      <c r="G19" s="31">
+        <f>IF(ISNUMBER(E19),D19*E19*(1+IF(ISNUMBER(F19),F19,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13645,8 +14213,8 @@
           <t>Paint subtotal</t>
         </is>
       </c>
-      <c r="F20" s="33">
-        <f>SUM(F19:F19)</f>
+      <c r="G20" s="33">
+        <f>SUM(G19:G19)</f>
         <v/>
       </c>
     </row>
@@ -13660,8 +14228,9 @@
       </c>
       <c r="D21" s="34" t="n"/>
       <c r="E21" s="34" t="n"/>
-      <c r="F21" s="36">
-        <f>F8+F11+F14+F17+F20</f>
+      <c r="F21" s="34" t="n"/>
+      <c r="G21" s="36">
+        <f>G8+G11+G14+G17+G20</f>
         <v/>
       </c>
     </row>
@@ -13701,8 +14270,12 @@
         <f>IF(Selections!R7="","",Selections!R7)</f>
         <v/>
       </c>
-      <c r="F25" s="31">
-        <f>IF(ISNUMBER(E25),D25*E25,"")</f>
+      <c r="F25" s="40">
+        <f>IF(Selections!S7="","",Selections!S7)</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>IF(ISNUMBER(E25),D25*E25*(1+IF(ISNUMBER(F25),F25,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13712,8 +14285,8 @@
           <t>Kitchen subtotal</t>
         </is>
       </c>
-      <c r="F26" s="33">
-        <f>SUM(F25:F25)</f>
+      <c r="G26" s="33">
+        <f>SUM(G25:G25)</f>
         <v/>
       </c>
     </row>
@@ -13746,8 +14319,12 @@
         <f>IF(Selections!R8="","",Selections!R8)</f>
         <v/>
       </c>
-      <c r="F28" s="31">
-        <f>IF(ISNUMBER(E28),D28*E28,"")</f>
+      <c r="F28" s="40">
+        <f>IF(Selections!S8="","",Selections!S8)</f>
+        <v/>
+      </c>
+      <c r="G28" s="31">
+        <f>IF(ISNUMBER(E28),D28*E28*(1+IF(ISNUMBER(F28),F28,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13757,8 +14334,8 @@
           <t>Lighting subtotal</t>
         </is>
       </c>
-      <c r="F29" s="33">
-        <f>SUM(F28:F28)</f>
+      <c r="G29" s="33">
+        <f>SUM(G28:G28)</f>
         <v/>
       </c>
     </row>
@@ -13772,8 +14349,9 @@
       </c>
       <c r="D30" s="34" t="n"/>
       <c r="E30" s="34" t="n"/>
-      <c r="F30" s="36">
-        <f>F26+F29</f>
+      <c r="F30" s="34" t="n"/>
+      <c r="G30" s="36">
+        <f>G26+G29</f>
         <v/>
       </c>
     </row>
@@ -13813,8 +14391,12 @@
         <f>IF(Selections!R9="","",Selections!R9)</f>
         <v/>
       </c>
-      <c r="F34" s="31">
-        <f>IF(ISNUMBER(E34),D34*E34,"")</f>
+      <c r="F34" s="40">
+        <f>IF(Selections!S9="","",Selections!S9)</f>
+        <v/>
+      </c>
+      <c r="G34" s="31">
+        <f>IF(ISNUMBER(E34),D34*E34*(1+IF(ISNUMBER(F34),F34,0)/100),"")</f>
         <v/>
       </c>
     </row>
@@ -13824,8 +14406,8 @@
           <t>Windows &amp; Doors subtotal</t>
         </is>
       </c>
-      <c r="F35" s="33">
-        <f>SUM(F34:F34)</f>
+      <c r="G35" s="33">
+        <f>SUM(G34:G34)</f>
         <v/>
       </c>
     </row>
@@ -13839,8 +14421,9 @@
       </c>
       <c r="D36" s="34" t="n"/>
       <c r="E36" s="34" t="n"/>
-      <c r="F36" s="36">
-        <f>F35</f>
+      <c r="F36" s="34" t="n"/>
+      <c r="G36" s="36">
+        <f>G35</f>
         <v/>
       </c>
     </row>
@@ -13854,25 +14437,26 @@
       </c>
       <c r="D38" s="34" t="n"/>
       <c r="E38" s="34" t="n"/>
-      <c r="F38" s="38">
-        <f>F21+F30+F36</f>
+      <c r="F38" s="34" t="n"/>
+      <c r="G38" s="38">
+        <f>G21+G30+G36</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove the presentation deadline banner
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -2997,7 +2997,7 @@
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>Search error</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>Automatic lookup is waiting for SERPAPI_KEY in the local .env file. Restart the app after configuring it.</t>
+          <t>No page confirmed the model number. Try: https://www.google.com/search?q=Dfw+company+xyz</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Seed projects from a room-by-room spec template
spec_template.json holds the standard outline - floor or zone, room,
line item - which maps onto Section, Room / Area and Item. A Load room
template button on the spec sheet adds every missing line item for the
selected project in one save and registers any new sections on the
Lists sheet so they keep their print order and dropdown entry.

Applying is idempotent: existing rows are counted and skipped, so the
template can be re-run after it grows without duplicating work already
specified. 260 items apply in well under a second.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -2546,7 +2546,9 @@
           <t>Arctic White</t>
         </is>
       </c>
-      <c r="H2" s="7" t="n"/>
+      <c r="H2" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I2" s="8" t="n"/>
       <c r="J2" s="8" t="n"/>
       <c r="K2" s="8" t="n"/>
@@ -2997,7 +2999,7 @@
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Search error</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -3007,7 +3009,7 @@
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>No page confirmed the model number. Try: https://www.google.com/search?q=Dfw+company+xyz</t>
+          <t>Automatic lookup is waiting for SERPAPI_KEY in the local .env file. Restart the app after configuring it.</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -14448,8 +14450,8 @@
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="A24:G24"/>

</xml_diff>

<commit_message>
Leave unspecified line items alone instead of failing them
Seeding a project filled the queue with rows that name something to
specify later, and each was stamped "Not found" with an error note, so
a new home looked like hundreds of failed lookups.

A row is queued only when it can actually be searched - both a
manufacturer and a model - or when it carries metadata that an edit may
have made stale. Half-filled rows are skipped deliberately: queueing
one mid-typing would save the workbook under the next keystroke and
fail the user's own edit on the revision check. When a search cannot
run, the row stays "Not run" rather than reporting a failure.

Also ignore the temporary workbook an interrupted save can leave.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UH_Homes_Selections_Tracker.xlsx
+++ b/UH_Homes_Selections_Tracker.xlsx
@@ -3060,15 +3060,11 @@
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M10" s="8" t="n"/>
-      <c r="N10" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N10" s="8" t="n"/>
       <c r="O10" s="7" t="n"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
@@ -3113,15 +3109,11 @@
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M11" s="8" t="n"/>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N11" s="8" t="n"/>
       <c r="O11" s="7" t="n"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
@@ -3166,15 +3158,11 @@
       <c r="K12" s="8" t="n"/>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M12" s="8" t="n"/>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N12" s="8" t="n"/>
       <c r="O12" s="7" t="n"/>
       <c r="P12" s="7" t="inlineStr">
         <is>
@@ -3219,15 +3207,11 @@
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M13" s="8" t="n"/>
-      <c r="N13" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N13" s="8" t="n"/>
       <c r="O13" s="7" t="n"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
@@ -3272,15 +3256,11 @@
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M14" s="8" t="n"/>
-      <c r="N14" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N14" s="8" t="n"/>
       <c r="O14" s="7" t="n"/>
       <c r="P14" s="7" t="inlineStr">
         <is>
@@ -3325,15 +3305,11 @@
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M15" s="8" t="n"/>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N15" s="8" t="n"/>
       <c r="O15" s="7" t="n"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
@@ -3378,15 +3354,11 @@
       <c r="K16" s="8" t="n"/>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N16" s="8" t="n"/>
       <c r="O16" s="7" t="n"/>
       <c r="P16" s="7" t="inlineStr">
         <is>
@@ -3431,15 +3403,11 @@
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M17" s="8" t="n"/>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N17" s="8" t="n"/>
       <c r="O17" s="7" t="n"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
@@ -3484,15 +3452,11 @@
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M18" s="8" t="n"/>
-      <c r="N18" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N18" s="8" t="n"/>
       <c r="O18" s="7" t="n"/>
       <c r="P18" s="7" t="inlineStr">
         <is>
@@ -3537,15 +3501,11 @@
       <c r="K19" s="8" t="n"/>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M19" s="8" t="n"/>
-      <c r="N19" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N19" s="8" t="n"/>
       <c r="O19" s="7" t="n"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
@@ -3590,15 +3550,11 @@
       <c r="K20" s="8" t="n"/>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M20" s="8" t="n"/>
-      <c r="N20" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N20" s="8" t="n"/>
       <c r="O20" s="7" t="n"/>
       <c r="P20" s="7" t="inlineStr">
         <is>
@@ -3643,15 +3599,11 @@
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M21" s="8" t="n"/>
-      <c r="N21" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N21" s="8" t="n"/>
       <c r="O21" s="7" t="n"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
@@ -3696,15 +3648,11 @@
       <c r="K22" s="8" t="n"/>
       <c r="L22" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M22" s="8" t="n"/>
-      <c r="N22" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N22" s="8" t="n"/>
       <c r="O22" s="7" t="n"/>
       <c r="P22" s="7" t="inlineStr">
         <is>
@@ -3749,15 +3697,11 @@
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M23" s="8" t="n"/>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N23" s="8" t="n"/>
       <c r="O23" s="7" t="n"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
@@ -3802,15 +3746,11 @@
       <c r="K24" s="8" t="n"/>
       <c r="L24" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M24" s="8" t="n"/>
-      <c r="N24" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N24" s="8" t="n"/>
       <c r="O24" s="7" t="n"/>
       <c r="P24" s="7" t="inlineStr">
         <is>
@@ -3855,15 +3795,11 @@
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M25" s="8" t="n"/>
-      <c r="N25" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N25" s="8" t="n"/>
       <c r="O25" s="7" t="n"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
@@ -3908,15 +3844,11 @@
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M26" s="8" t="n"/>
-      <c r="N26" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N26" s="8" t="n"/>
       <c r="O26" s="7" t="n"/>
       <c r="P26" s="7" t="inlineStr">
         <is>
@@ -3961,15 +3893,11 @@
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M27" s="8" t="n"/>
-      <c r="N27" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N27" s="8" t="n"/>
       <c r="O27" s="7" t="n"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
@@ -4014,15 +3942,11 @@
       <c r="K28" s="8" t="n"/>
       <c r="L28" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M28" s="8" t="n"/>
-      <c r="N28" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N28" s="8" t="n"/>
       <c r="O28" s="7" t="n"/>
       <c r="P28" s="7" t="inlineStr">
         <is>
@@ -4067,15 +3991,11 @@
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M29" s="8" t="n"/>
-      <c r="N29" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N29" s="8" t="n"/>
       <c r="O29" s="7" t="n"/>
       <c r="P29" s="7" t="inlineStr">
         <is>
@@ -4120,15 +4040,11 @@
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M30" s="8" t="n"/>
-      <c r="N30" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N30" s="8" t="n"/>
       <c r="O30" s="7" t="n"/>
       <c r="P30" s="7" t="inlineStr">
         <is>
@@ -4173,15 +4089,11 @@
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M31" s="8" t="n"/>
-      <c r="N31" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N31" s="8" t="n"/>
       <c r="O31" s="7" t="n"/>
       <c r="P31" s="7" t="inlineStr">
         <is>
@@ -4226,15 +4138,11 @@
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M32" s="8" t="n"/>
-      <c r="N32" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N32" s="8" t="n"/>
       <c r="O32" s="7" t="n"/>
       <c r="P32" s="7" t="inlineStr">
         <is>
@@ -4279,15 +4187,11 @@
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M33" s="8" t="n"/>
-      <c r="N33" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N33" s="8" t="n"/>
       <c r="O33" s="7" t="n"/>
       <c r="P33" s="7" t="inlineStr">
         <is>
@@ -4332,15 +4236,11 @@
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M34" s="8" t="n"/>
-      <c r="N34" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N34" s="8" t="n"/>
       <c r="O34" s="7" t="n"/>
       <c r="P34" s="7" t="inlineStr">
         <is>
@@ -4385,15 +4285,11 @@
       <c r="K35" s="8" t="n"/>
       <c r="L35" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M35" s="8" t="n"/>
-      <c r="N35" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N35" s="8" t="n"/>
       <c r="O35" s="7" t="n"/>
       <c r="P35" s="7" t="inlineStr">
         <is>
@@ -4438,15 +4334,11 @@
       <c r="K36" s="8" t="n"/>
       <c r="L36" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M36" s="8" t="n"/>
-      <c r="N36" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N36" s="8" t="n"/>
       <c r="O36" s="7" t="n"/>
       <c r="P36" s="7" t="inlineStr">
         <is>
@@ -4491,15 +4383,11 @@
       <c r="K37" s="8" t="n"/>
       <c r="L37" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M37" s="8" t="n"/>
-      <c r="N37" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N37" s="8" t="n"/>
       <c r="O37" s="7" t="n"/>
       <c r="P37" s="7" t="inlineStr">
         <is>
@@ -4544,15 +4432,11 @@
       <c r="K38" s="8" t="n"/>
       <c r="L38" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M38" s="8" t="n"/>
-      <c r="N38" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N38" s="8" t="n"/>
       <c r="O38" s="7" t="n"/>
       <c r="P38" s="7" t="inlineStr">
         <is>
@@ -4597,15 +4481,11 @@
       <c r="K39" s="8" t="n"/>
       <c r="L39" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M39" s="8" t="n"/>
-      <c r="N39" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N39" s="8" t="n"/>
       <c r="O39" s="7" t="n"/>
       <c r="P39" s="7" t="inlineStr">
         <is>
@@ -4650,15 +4530,11 @@
       <c r="K40" s="8" t="n"/>
       <c r="L40" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M40" s="8" t="n"/>
-      <c r="N40" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N40" s="8" t="n"/>
       <c r="O40" s="7" t="n"/>
       <c r="P40" s="7" t="inlineStr">
         <is>
@@ -4703,15 +4579,11 @@
       <c r="K41" s="8" t="n"/>
       <c r="L41" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M41" s="8" t="n"/>
-      <c r="N41" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N41" s="8" t="n"/>
       <c r="O41" s="7" t="n"/>
       <c r="P41" s="7" t="inlineStr">
         <is>
@@ -4756,15 +4628,11 @@
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M42" s="8" t="n"/>
-      <c r="N42" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N42" s="8" t="n"/>
       <c r="O42" s="7" t="n"/>
       <c r="P42" s="7" t="inlineStr">
         <is>
@@ -4809,15 +4677,11 @@
       <c r="K43" s="8" t="n"/>
       <c r="L43" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M43" s="8" t="n"/>
-      <c r="N43" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N43" s="8" t="n"/>
       <c r="O43" s="7" t="n"/>
       <c r="P43" s="7" t="inlineStr">
         <is>
@@ -4862,15 +4726,11 @@
       <c r="K44" s="8" t="n"/>
       <c r="L44" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M44" s="8" t="n"/>
-      <c r="N44" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N44" s="8" t="n"/>
       <c r="O44" s="7" t="n"/>
       <c r="P44" s="7" t="inlineStr">
         <is>
@@ -4915,15 +4775,11 @@
       <c r="K45" s="8" t="n"/>
       <c r="L45" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M45" s="8" t="n"/>
-      <c r="N45" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N45" s="8" t="n"/>
       <c r="O45" s="7" t="n"/>
       <c r="P45" s="7" t="inlineStr">
         <is>
@@ -4968,15 +4824,11 @@
       <c r="K46" s="8" t="n"/>
       <c r="L46" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M46" s="8" t="n"/>
-      <c r="N46" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N46" s="8" t="n"/>
       <c r="O46" s="7" t="n"/>
       <c r="P46" s="7" t="inlineStr">
         <is>
@@ -5021,15 +4873,11 @@
       <c r="K47" s="8" t="n"/>
       <c r="L47" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M47" s="8" t="n"/>
-      <c r="N47" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N47" s="8" t="n"/>
       <c r="O47" s="7" t="n"/>
       <c r="P47" s="7" t="inlineStr">
         <is>
@@ -5074,15 +4922,11 @@
       <c r="K48" s="8" t="n"/>
       <c r="L48" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M48" s="8" t="n"/>
-      <c r="N48" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N48" s="8" t="n"/>
       <c r="O48" s="7" t="n"/>
       <c r="P48" s="7" t="inlineStr">
         <is>
@@ -5127,15 +4971,11 @@
       <c r="K49" s="8" t="n"/>
       <c r="L49" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M49" s="8" t="n"/>
-      <c r="N49" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N49" s="8" t="n"/>
       <c r="O49" s="7" t="n"/>
       <c r="P49" s="7" t="inlineStr">
         <is>
@@ -5180,15 +5020,11 @@
       <c r="K50" s="8" t="n"/>
       <c r="L50" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M50" s="8" t="n"/>
-      <c r="N50" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N50" s="8" t="n"/>
       <c r="O50" s="7" t="n"/>
       <c r="P50" s="7" t="inlineStr">
         <is>
@@ -5233,15 +5069,11 @@
       <c r="K51" s="8" t="n"/>
       <c r="L51" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M51" s="8" t="n"/>
-      <c r="N51" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N51" s="8" t="n"/>
       <c r="O51" s="7" t="n"/>
       <c r="P51" s="7" t="inlineStr">
         <is>
@@ -5286,15 +5118,11 @@
       <c r="K52" s="8" t="n"/>
       <c r="L52" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M52" s="8" t="n"/>
-      <c r="N52" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N52" s="8" t="n"/>
       <c r="O52" s="7" t="n"/>
       <c r="P52" s="7" t="inlineStr">
         <is>
@@ -5339,15 +5167,11 @@
       <c r="K53" s="8" t="n"/>
       <c r="L53" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M53" s="8" t="n"/>
-      <c r="N53" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N53" s="8" t="n"/>
       <c r="O53" s="7" t="n"/>
       <c r="P53" s="7" t="inlineStr">
         <is>
@@ -5392,15 +5216,11 @@
       <c r="K54" s="8" t="n"/>
       <c r="L54" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M54" s="8" t="n"/>
-      <c r="N54" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N54" s="8" t="n"/>
       <c r="O54" s="7" t="n"/>
       <c r="P54" s="7" t="inlineStr">
         <is>
@@ -5445,15 +5265,11 @@
       <c r="K55" s="8" t="n"/>
       <c r="L55" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M55" s="8" t="n"/>
-      <c r="N55" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N55" s="8" t="n"/>
       <c r="O55" s="7" t="n"/>
       <c r="P55" s="7" t="inlineStr">
         <is>
@@ -5498,15 +5314,11 @@
       <c r="K56" s="8" t="n"/>
       <c r="L56" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M56" s="8" t="n"/>
-      <c r="N56" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N56" s="8" t="n"/>
       <c r="O56" s="7" t="n"/>
       <c r="P56" s="7" t="inlineStr">
         <is>
@@ -5551,15 +5363,11 @@
       <c r="K57" s="8" t="n"/>
       <c r="L57" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M57" s="8" t="n"/>
-      <c r="N57" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N57" s="8" t="n"/>
       <c r="O57" s="7" t="n"/>
       <c r="P57" s="7" t="inlineStr">
         <is>
@@ -5604,15 +5412,11 @@
       <c r="K58" s="8" t="n"/>
       <c r="L58" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M58" s="8" t="n"/>
-      <c r="N58" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N58" s="8" t="n"/>
       <c r="O58" s="7" t="n"/>
       <c r="P58" s="7" t="inlineStr">
         <is>
@@ -5657,15 +5461,11 @@
       <c r="K59" s="8" t="n"/>
       <c r="L59" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M59" s="8" t="n"/>
-      <c r="N59" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N59" s="8" t="n"/>
       <c r="O59" s="7" t="n"/>
       <c r="P59" s="7" t="inlineStr">
         <is>
@@ -5710,15 +5510,11 @@
       <c r="K60" s="8" t="n"/>
       <c r="L60" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M60" s="8" t="n"/>
-      <c r="N60" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N60" s="8" t="n"/>
       <c r="O60" s="7" t="n"/>
       <c r="P60" s="7" t="inlineStr">
         <is>
@@ -5763,15 +5559,11 @@
       <c r="K61" s="8" t="n"/>
       <c r="L61" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M61" s="8" t="n"/>
-      <c r="N61" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N61" s="8" t="n"/>
       <c r="O61" s="7" t="n"/>
       <c r="P61" s="7" t="inlineStr">
         <is>
@@ -5816,15 +5608,11 @@
       <c r="K62" s="8" t="n"/>
       <c r="L62" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M62" s="8" t="n"/>
-      <c r="N62" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N62" s="8" t="n"/>
       <c r="O62" s="7" t="n"/>
       <c r="P62" s="7" t="inlineStr">
         <is>
@@ -5869,15 +5657,11 @@
       <c r="K63" s="8" t="n"/>
       <c r="L63" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M63" s="8" t="n"/>
-      <c r="N63" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N63" s="8" t="n"/>
       <c r="O63" s="7" t="n"/>
       <c r="P63" s="7" t="inlineStr">
         <is>
@@ -5922,15 +5706,11 @@
       <c r="K64" s="8" t="n"/>
       <c r="L64" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M64" s="8" t="n"/>
-      <c r="N64" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N64" s="8" t="n"/>
       <c r="O64" s="7" t="n"/>
       <c r="P64" s="7" t="inlineStr">
         <is>
@@ -5975,15 +5755,11 @@
       <c r="K65" s="8" t="n"/>
       <c r="L65" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M65" s="8" t="n"/>
-      <c r="N65" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N65" s="8" t="n"/>
       <c r="O65" s="7" t="n"/>
       <c r="P65" s="7" t="inlineStr">
         <is>
@@ -6028,15 +5804,11 @@
       <c r="K66" s="8" t="n"/>
       <c r="L66" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M66" s="8" t="n"/>
-      <c r="N66" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N66" s="8" t="n"/>
       <c r="O66" s="7" t="n"/>
       <c r="P66" s="7" t="inlineStr">
         <is>
@@ -6081,15 +5853,11 @@
       <c r="K67" s="8" t="n"/>
       <c r="L67" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M67" s="8" t="n"/>
-      <c r="N67" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N67" s="8" t="n"/>
       <c r="O67" s="7" t="n"/>
       <c r="P67" s="7" t="inlineStr">
         <is>
@@ -6134,15 +5902,11 @@
       <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M68" s="8" t="n"/>
-      <c r="N68" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N68" s="8" t="n"/>
       <c r="O68" s="7" t="n"/>
       <c r="P68" s="7" t="inlineStr">
         <is>
@@ -6187,15 +5951,11 @@
       <c r="K69" s="8" t="n"/>
       <c r="L69" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M69" s="8" t="n"/>
-      <c r="N69" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N69" s="8" t="n"/>
       <c r="O69" s="7" t="n"/>
       <c r="P69" s="7" t="inlineStr">
         <is>
@@ -6240,15 +6000,11 @@
       <c r="K70" s="8" t="n"/>
       <c r="L70" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M70" s="8" t="n"/>
-      <c r="N70" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N70" s="8" t="n"/>
       <c r="O70" s="7" t="n"/>
       <c r="P70" s="7" t="inlineStr">
         <is>
@@ -6293,15 +6049,11 @@
       <c r="K71" s="8" t="n"/>
       <c r="L71" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M71" s="8" t="n"/>
-      <c r="N71" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N71" s="8" t="n"/>
       <c r="O71" s="7" t="n"/>
       <c r="P71" s="7" t="inlineStr">
         <is>
@@ -6346,15 +6098,11 @@
       <c r="K72" s="8" t="n"/>
       <c r="L72" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M72" s="8" t="n"/>
-      <c r="N72" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N72" s="8" t="n"/>
       <c r="O72" s="7" t="n"/>
       <c r="P72" s="7" t="inlineStr">
         <is>
@@ -6399,15 +6147,11 @@
       <c r="K73" s="8" t="n"/>
       <c r="L73" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M73" s="8" t="n"/>
-      <c r="N73" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N73" s="8" t="n"/>
       <c r="O73" s="7" t="n"/>
       <c r="P73" s="7" t="inlineStr">
         <is>
@@ -6452,15 +6196,11 @@
       <c r="K74" s="8" t="n"/>
       <c r="L74" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M74" s="8" t="n"/>
-      <c r="N74" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N74" s="8" t="n"/>
       <c r="O74" s="7" t="n"/>
       <c r="P74" s="7" t="inlineStr">
         <is>
@@ -6505,15 +6245,11 @@
       <c r="K75" s="8" t="n"/>
       <c r="L75" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M75" s="8" t="n"/>
-      <c r="N75" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N75" s="8" t="n"/>
       <c r="O75" s="7" t="n"/>
       <c r="P75" s="7" t="inlineStr">
         <is>
@@ -6558,15 +6294,11 @@
       <c r="K76" s="8" t="n"/>
       <c r="L76" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M76" s="8" t="n"/>
-      <c r="N76" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N76" s="8" t="n"/>
       <c r="O76" s="7" t="n"/>
       <c r="P76" s="7" t="inlineStr">
         <is>
@@ -6611,15 +6343,11 @@
       <c r="K77" s="8" t="n"/>
       <c r="L77" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M77" s="8" t="n"/>
-      <c r="N77" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N77" s="8" t="n"/>
       <c r="O77" s="7" t="n"/>
       <c r="P77" s="7" t="inlineStr">
         <is>
@@ -6664,15 +6392,11 @@
       <c r="K78" s="8" t="n"/>
       <c r="L78" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M78" s="8" t="n"/>
-      <c r="N78" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N78" s="8" t="n"/>
       <c r="O78" s="7" t="n"/>
       <c r="P78" s="7" t="inlineStr">
         <is>
@@ -6717,15 +6441,11 @@
       <c r="K79" s="8" t="n"/>
       <c r="L79" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M79" s="8" t="n"/>
-      <c r="N79" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N79" s="8" t="n"/>
       <c r="O79" s="7" t="n"/>
       <c r="P79" s="7" t="inlineStr">
         <is>
@@ -6770,15 +6490,11 @@
       <c r="K80" s="8" t="n"/>
       <c r="L80" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M80" s="8" t="n"/>
-      <c r="N80" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N80" s="8" t="n"/>
       <c r="O80" s="7" t="n"/>
       <c r="P80" s="7" t="inlineStr">
         <is>
@@ -6823,15 +6539,11 @@
       <c r="K81" s="8" t="n"/>
       <c r="L81" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M81" s="8" t="n"/>
-      <c r="N81" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N81" s="8" t="n"/>
       <c r="O81" s="7" t="n"/>
       <c r="P81" s="7" t="inlineStr">
         <is>
@@ -6876,15 +6588,11 @@
       <c r="K82" s="8" t="n"/>
       <c r="L82" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M82" s="8" t="n"/>
-      <c r="N82" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N82" s="8" t="n"/>
       <c r="O82" s="7" t="n"/>
       <c r="P82" s="7" t="inlineStr">
         <is>
@@ -6929,15 +6637,11 @@
       <c r="K83" s="8" t="n"/>
       <c r="L83" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M83" s="8" t="n"/>
-      <c r="N83" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N83" s="8" t="n"/>
       <c r="O83" s="7" t="n"/>
       <c r="P83" s="7" t="inlineStr">
         <is>
@@ -6982,15 +6686,11 @@
       <c r="K84" s="8" t="n"/>
       <c r="L84" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M84" s="8" t="n"/>
-      <c r="N84" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N84" s="8" t="n"/>
       <c r="O84" s="7" t="n"/>
       <c r="P84" s="7" t="inlineStr">
         <is>
@@ -7035,15 +6735,11 @@
       <c r="K85" s="8" t="n"/>
       <c r="L85" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M85" s="8" t="n"/>
-      <c r="N85" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N85" s="8" t="n"/>
       <c r="O85" s="7" t="n"/>
       <c r="P85" s="7" t="inlineStr">
         <is>
@@ -7088,15 +6784,11 @@
       <c r="K86" s="8" t="n"/>
       <c r="L86" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M86" s="8" t="n"/>
-      <c r="N86" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N86" s="8" t="n"/>
       <c r="O86" s="7" t="n"/>
       <c r="P86" s="7" t="inlineStr">
         <is>
@@ -7141,15 +6833,11 @@
       <c r="K87" s="8" t="n"/>
       <c r="L87" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M87" s="8" t="n"/>
-      <c r="N87" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N87" s="8" t="n"/>
       <c r="O87" s="7" t="n"/>
       <c r="P87" s="7" t="inlineStr">
         <is>
@@ -7194,15 +6882,11 @@
       <c r="K88" s="8" t="n"/>
       <c r="L88" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M88" s="8" t="n"/>
-      <c r="N88" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N88" s="8" t="n"/>
       <c r="O88" s="7" t="n"/>
       <c r="P88" s="7" t="inlineStr">
         <is>
@@ -7247,15 +6931,11 @@
       <c r="K89" s="8" t="n"/>
       <c r="L89" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M89" s="8" t="n"/>
-      <c r="N89" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N89" s="8" t="n"/>
       <c r="O89" s="7" t="n"/>
       <c r="P89" s="7" t="inlineStr">
         <is>
@@ -7300,15 +6980,11 @@
       <c r="K90" s="8" t="n"/>
       <c r="L90" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M90" s="8" t="n"/>
-      <c r="N90" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N90" s="8" t="n"/>
       <c r="O90" s="7" t="n"/>
       <c r="P90" s="7" t="inlineStr">
         <is>
@@ -7353,15 +7029,11 @@
       <c r="K91" s="8" t="n"/>
       <c r="L91" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M91" s="8" t="n"/>
-      <c r="N91" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N91" s="8" t="n"/>
       <c r="O91" s="7" t="n"/>
       <c r="P91" s="7" t="inlineStr">
         <is>
@@ -7406,15 +7078,11 @@
       <c r="K92" s="8" t="n"/>
       <c r="L92" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M92" s="8" t="n"/>
-      <c r="N92" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N92" s="8" t="n"/>
       <c r="O92" s="7" t="n"/>
       <c r="P92" s="7" t="inlineStr">
         <is>
@@ -7459,15 +7127,11 @@
       <c r="K93" s="8" t="n"/>
       <c r="L93" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M93" s="8" t="n"/>
-      <c r="N93" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N93" s="8" t="n"/>
       <c r="O93" s="7" t="n"/>
       <c r="P93" s="7" t="inlineStr">
         <is>
@@ -7512,15 +7176,11 @@
       <c r="K94" s="8" t="n"/>
       <c r="L94" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M94" s="8" t="n"/>
-      <c r="N94" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N94" s="8" t="n"/>
       <c r="O94" s="7" t="n"/>
       <c r="P94" s="7" t="inlineStr">
         <is>
@@ -7565,15 +7225,11 @@
       <c r="K95" s="8" t="n"/>
       <c r="L95" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M95" s="8" t="n"/>
-      <c r="N95" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N95" s="8" t="n"/>
       <c r="O95" s="7" t="n"/>
       <c r="P95" s="7" t="inlineStr">
         <is>
@@ -7618,15 +7274,11 @@
       <c r="K96" s="8" t="n"/>
       <c r="L96" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M96" s="8" t="n"/>
-      <c r="N96" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N96" s="8" t="n"/>
       <c r="O96" s="7" t="n"/>
       <c r="P96" s="7" t="inlineStr">
         <is>
@@ -7671,15 +7323,11 @@
       <c r="K97" s="8" t="n"/>
       <c r="L97" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M97" s="8" t="n"/>
-      <c r="N97" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N97" s="8" t="n"/>
       <c r="O97" s="7" t="n"/>
       <c r="P97" s="7" t="inlineStr">
         <is>
@@ -7724,15 +7372,11 @@
       <c r="K98" s="8" t="n"/>
       <c r="L98" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M98" s="8" t="n"/>
-      <c r="N98" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N98" s="8" t="n"/>
       <c r="O98" s="7" t="n"/>
       <c r="P98" s="7" t="inlineStr">
         <is>
@@ -7777,15 +7421,11 @@
       <c r="K99" s="8" t="n"/>
       <c r="L99" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M99" s="8" t="n"/>
-      <c r="N99" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N99" s="8" t="n"/>
       <c r="O99" s="7" t="n"/>
       <c r="P99" s="7" t="inlineStr">
         <is>
@@ -7830,15 +7470,11 @@
       <c r="K100" s="8" t="n"/>
       <c r="L100" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M100" s="8" t="n"/>
-      <c r="N100" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N100" s="8" t="n"/>
       <c r="O100" s="7" t="n"/>
       <c r="P100" s="7" t="inlineStr">
         <is>
@@ -7883,15 +7519,11 @@
       <c r="K101" s="8" t="n"/>
       <c r="L101" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M101" s="8" t="n"/>
-      <c r="N101" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N101" s="8" t="n"/>
       <c r="O101" s="7" t="n"/>
       <c r="P101" s="7" t="inlineStr">
         <is>
@@ -7936,15 +7568,11 @@
       <c r="K102" s="8" t="n"/>
       <c r="L102" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M102" s="8" t="n"/>
-      <c r="N102" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N102" s="8" t="n"/>
       <c r="O102" s="7" t="n"/>
       <c r="P102" s="7" t="inlineStr">
         <is>
@@ -7989,15 +7617,11 @@
       <c r="K103" s="8" t="n"/>
       <c r="L103" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M103" s="8" t="n"/>
-      <c r="N103" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N103" s="8" t="n"/>
       <c r="O103" s="7" t="n"/>
       <c r="P103" s="7" t="inlineStr">
         <is>
@@ -8042,15 +7666,11 @@
       <c r="K104" s="8" t="n"/>
       <c r="L104" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M104" s="8" t="n"/>
-      <c r="N104" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N104" s="8" t="n"/>
       <c r="O104" s="7" t="n"/>
       <c r="P104" s="7" t="inlineStr">
         <is>
@@ -8095,15 +7715,11 @@
       <c r="K105" s="8" t="n"/>
       <c r="L105" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M105" s="8" t="n"/>
-      <c r="N105" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N105" s="8" t="n"/>
       <c r="O105" s="7" t="n"/>
       <c r="P105" s="7" t="inlineStr">
         <is>
@@ -8148,15 +7764,11 @@
       <c r="K106" s="8" t="n"/>
       <c r="L106" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M106" s="8" t="n"/>
-      <c r="N106" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N106" s="8" t="n"/>
       <c r="O106" s="7" t="n"/>
       <c r="P106" s="7" t="inlineStr">
         <is>
@@ -8201,15 +7813,11 @@
       <c r="K107" s="8" t="n"/>
       <c r="L107" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M107" s="8" t="n"/>
-      <c r="N107" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N107" s="8" t="n"/>
       <c r="O107" s="7" t="n"/>
       <c r="P107" s="7" t="inlineStr">
         <is>
@@ -8254,15 +7862,11 @@
       <c r="K108" s="8" t="n"/>
       <c r="L108" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M108" s="8" t="n"/>
-      <c r="N108" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N108" s="8" t="n"/>
       <c r="O108" s="7" t="n"/>
       <c r="P108" s="7" t="inlineStr">
         <is>
@@ -8307,15 +7911,11 @@
       <c r="K109" s="8" t="n"/>
       <c r="L109" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M109" s="8" t="n"/>
-      <c r="N109" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N109" s="8" t="n"/>
       <c r="O109" s="7" t="n"/>
       <c r="P109" s="7" t="inlineStr">
         <is>
@@ -8360,15 +7960,11 @@
       <c r="K110" s="8" t="n"/>
       <c r="L110" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M110" s="8" t="n"/>
-      <c r="N110" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N110" s="8" t="n"/>
       <c r="O110" s="7" t="n"/>
       <c r="P110" s="7" t="inlineStr">
         <is>
@@ -8413,15 +8009,11 @@
       <c r="K111" s="8" t="n"/>
       <c r="L111" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M111" s="8" t="n"/>
-      <c r="N111" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N111" s="8" t="n"/>
       <c r="O111" s="7" t="n"/>
       <c r="P111" s="7" t="inlineStr">
         <is>
@@ -8466,15 +8058,11 @@
       <c r="K112" s="8" t="n"/>
       <c r="L112" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M112" s="8" t="n"/>
-      <c r="N112" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N112" s="8" t="n"/>
       <c r="O112" s="7" t="n"/>
       <c r="P112" s="7" t="inlineStr">
         <is>
@@ -8519,15 +8107,11 @@
       <c r="K113" s="8" t="n"/>
       <c r="L113" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M113" s="8" t="n"/>
-      <c r="N113" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N113" s="8" t="n"/>
       <c r="O113" s="7" t="n"/>
       <c r="P113" s="7" t="inlineStr">
         <is>
@@ -8572,15 +8156,11 @@
       <c r="K114" s="8" t="n"/>
       <c r="L114" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M114" s="8" t="n"/>
-      <c r="N114" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N114" s="8" t="n"/>
       <c r="O114" s="7" t="n"/>
       <c r="P114" s="7" t="inlineStr">
         <is>
@@ -8625,15 +8205,11 @@
       <c r="K115" s="8" t="n"/>
       <c r="L115" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M115" s="8" t="n"/>
-      <c r="N115" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N115" s="8" t="n"/>
       <c r="O115" s="7" t="n"/>
       <c r="P115" s="7" t="inlineStr">
         <is>
@@ -8678,15 +8254,11 @@
       <c r="K116" s="8" t="n"/>
       <c r="L116" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M116" s="8" t="n"/>
-      <c r="N116" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N116" s="8" t="n"/>
       <c r="O116" s="7" t="n"/>
       <c r="P116" s="7" t="inlineStr">
         <is>
@@ -8731,15 +8303,11 @@
       <c r="K117" s="8" t="n"/>
       <c r="L117" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M117" s="8" t="n"/>
-      <c r="N117" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N117" s="8" t="n"/>
       <c r="O117" s="7" t="n"/>
       <c r="P117" s="7" t="inlineStr">
         <is>
@@ -8784,15 +8352,11 @@
       <c r="K118" s="8" t="n"/>
       <c r="L118" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M118" s="8" t="n"/>
-      <c r="N118" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N118" s="8" t="n"/>
       <c r="O118" s="7" t="n"/>
       <c r="P118" s="7" t="inlineStr">
         <is>
@@ -8837,15 +8401,11 @@
       <c r="K119" s="8" t="n"/>
       <c r="L119" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M119" s="8" t="n"/>
-      <c r="N119" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N119" s="8" t="n"/>
       <c r="O119" s="7" t="n"/>
       <c r="P119" s="7" t="inlineStr">
         <is>
@@ -8890,15 +8450,11 @@
       <c r="K120" s="8" t="n"/>
       <c r="L120" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M120" s="8" t="n"/>
-      <c r="N120" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N120" s="8" t="n"/>
       <c r="O120" s="7" t="n"/>
       <c r="P120" s="7" t="inlineStr">
         <is>
@@ -8943,15 +8499,11 @@
       <c r="K121" s="8" t="n"/>
       <c r="L121" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M121" s="8" t="n"/>
-      <c r="N121" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N121" s="8" t="n"/>
       <c r="O121" s="7" t="n"/>
       <c r="P121" s="7" t="inlineStr">
         <is>
@@ -8996,15 +8548,11 @@
       <c r="K122" s="8" t="n"/>
       <c r="L122" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M122" s="8" t="n"/>
-      <c r="N122" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N122" s="8" t="n"/>
       <c r="O122" s="7" t="n"/>
       <c r="P122" s="7" t="inlineStr">
         <is>
@@ -9049,15 +8597,11 @@
       <c r="K123" s="8" t="n"/>
       <c r="L123" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M123" s="8" t="n"/>
-      <c r="N123" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N123" s="8" t="n"/>
       <c r="O123" s="7" t="n"/>
       <c r="P123" s="7" t="inlineStr">
         <is>
@@ -9102,15 +8646,11 @@
       <c r="K124" s="8" t="n"/>
       <c r="L124" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M124" s="8" t="n"/>
-      <c r="N124" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N124" s="8" t="n"/>
       <c r="O124" s="7" t="n"/>
       <c r="P124" s="7" t="inlineStr">
         <is>
@@ -9155,15 +8695,11 @@
       <c r="K125" s="8" t="n"/>
       <c r="L125" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M125" s="8" t="n"/>
-      <c r="N125" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N125" s="8" t="n"/>
       <c r="O125" s="7" t="n"/>
       <c r="P125" s="7" t="inlineStr">
         <is>
@@ -9208,15 +8744,11 @@
       <c r="K126" s="8" t="n"/>
       <c r="L126" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M126" s="8" t="n"/>
-      <c r="N126" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N126" s="8" t="n"/>
       <c r="O126" s="7" t="n"/>
       <c r="P126" s="7" t="inlineStr">
         <is>
@@ -9261,15 +8793,11 @@
       <c r="K127" s="8" t="n"/>
       <c r="L127" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M127" s="8" t="n"/>
-      <c r="N127" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N127" s="8" t="n"/>
       <c r="O127" s="7" t="n"/>
       <c r="P127" s="7" t="inlineStr">
         <is>
@@ -9314,15 +8842,11 @@
       <c r="K128" s="8" t="n"/>
       <c r="L128" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M128" s="8" t="n"/>
-      <c r="N128" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N128" s="8" t="n"/>
       <c r="O128" s="7" t="n"/>
       <c r="P128" s="7" t="inlineStr">
         <is>
@@ -9367,15 +8891,11 @@
       <c r="K129" s="8" t="n"/>
       <c r="L129" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M129" s="8" t="n"/>
-      <c r="N129" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N129" s="8" t="n"/>
       <c r="O129" s="7" t="n"/>
       <c r="P129" s="7" t="inlineStr">
         <is>
@@ -9420,15 +8940,11 @@
       <c r="K130" s="8" t="n"/>
       <c r="L130" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M130" s="8" t="n"/>
-      <c r="N130" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N130" s="8" t="n"/>
       <c r="O130" s="7" t="n"/>
       <c r="P130" s="7" t="inlineStr">
         <is>
@@ -9473,15 +8989,11 @@
       <c r="K131" s="8" t="n"/>
       <c r="L131" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M131" s="8" t="n"/>
-      <c r="N131" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N131" s="8" t="n"/>
       <c r="O131" s="7" t="n"/>
       <c r="P131" s="7" t="inlineStr">
         <is>
@@ -9526,15 +9038,11 @@
       <c r="K132" s="8" t="n"/>
       <c r="L132" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M132" s="8" t="n"/>
-      <c r="N132" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N132" s="8" t="n"/>
       <c r="O132" s="7" t="n"/>
       <c r="P132" s="7" t="inlineStr">
         <is>
@@ -9579,15 +9087,11 @@
       <c r="K133" s="8" t="n"/>
       <c r="L133" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M133" s="8" t="n"/>
-      <c r="N133" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N133" s="8" t="n"/>
       <c r="O133" s="7" t="n"/>
       <c r="P133" s="7" t="inlineStr">
         <is>
@@ -9632,15 +9136,11 @@
       <c r="K134" s="8" t="n"/>
       <c r="L134" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M134" s="8" t="n"/>
-      <c r="N134" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N134" s="8" t="n"/>
       <c r="O134" s="7" t="n"/>
       <c r="P134" s="7" t="inlineStr">
         <is>
@@ -9685,15 +9185,11 @@
       <c r="K135" s="8" t="n"/>
       <c r="L135" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M135" s="8" t="n"/>
-      <c r="N135" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N135" s="8" t="n"/>
       <c r="O135" s="7" t="n"/>
       <c r="P135" s="7" t="inlineStr">
         <is>
@@ -9738,15 +9234,11 @@
       <c r="K136" s="8" t="n"/>
       <c r="L136" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M136" s="8" t="n"/>
-      <c r="N136" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N136" s="8" t="n"/>
       <c r="O136" s="7" t="n"/>
       <c r="P136" s="7" t="inlineStr">
         <is>
@@ -9787,15 +9279,11 @@
       <c r="K137" s="8" t="n"/>
       <c r="L137" s="8" t="inlineStr">
         <is>
-          <t>Not found</t>
+          <t>Not run</t>
         </is>
       </c>
       <c r="M137" s="8" t="n"/>
-      <c r="N137" s="8" t="inlineStr">
-        <is>
-          <t>Manufacturer and Model # are both required. Complete them to start automatic lookup.</t>
-        </is>
-      </c>
+      <c r="N137" s="8" t="n"/>
       <c r="O137" s="7" t="n"/>
       <c r="P137" s="7" t="inlineStr">
         <is>

</xml_diff>